<commit_message>
Actualizacion 10 Mar 10:25
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -66847,7 +66847,7 @@
         <v>8</v>
       </c>
       <c r="C20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D20">
         <v>7</v>
@@ -66901,7 +66901,7 @@
         <v>8</v>
       </c>
       <c r="U20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="V20">
         <v>7</v>
@@ -67771,7 +67771,7 @@
         <v>10</v>
       </c>
       <c r="C32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D32">
         <v>5</v>
@@ -67825,7 +67825,7 @@
         <v>10</v>
       </c>
       <c r="U32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="V32">
         <v>5</v>

</xml_diff>

<commit_message>
Actualizacion 11 Mar Tarde
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -57553,7 +57553,7 @@
         <v>-1</v>
       </c>
       <c r="G7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="H7">
         <v>-1</v>
@@ -57607,7 +57607,7 @@
         <v>-1</v>
       </c>
       <c r="Y7">
-        <v>-1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -58323,7 +58323,7 @@
         <v>-1</v>
       </c>
       <c r="G17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H17">
         <v>-1</v>
@@ -58377,7 +58377,7 @@
         <v>-1</v>
       </c>
       <c r="Y17">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:25">

</xml_diff>

<commit_message>
Actualización 16 de Mayo
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -9349,7 +9349,7 @@
         <v>8</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J4">
         <v>8</v>
@@ -9438,7 +9438,7 @@
         <v>8</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J5">
         <v>7</v>
@@ -9480,7 +9480,7 @@
         <v>-1</v>
       </c>
       <c r="W5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X5">
         <v>7</v>
@@ -9527,7 +9527,7 @@
         <v>7</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J6">
         <v>7</v>
@@ -9616,7 +9616,7 @@
         <v>-1</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J7">
         <v>5</v>
@@ -9658,7 +9658,7 @@
         <v>-1</v>
       </c>
       <c r="W7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X7">
         <v>5</v>
@@ -9705,7 +9705,7 @@
         <v>7</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J8">
         <v>7</v>
@@ -9794,7 +9794,7 @@
         <v>10</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J9">
         <v>7</v>
@@ -9836,7 +9836,7 @@
         <v>-1</v>
       </c>
       <c r="W9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X9">
         <v>7</v>
@@ -9883,7 +9883,7 @@
         <v>10</v>
       </c>
       <c r="I10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J10">
         <v>9</v>
@@ -9972,7 +9972,7 @@
         <v>8</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J11">
         <v>9</v>
@@ -10061,7 +10061,7 @@
         <v>9</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J12">
         <v>9</v>
@@ -10150,7 +10150,7 @@
         <v>-1</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J13">
         <v>5</v>
@@ -10239,7 +10239,7 @@
         <v>10</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J14">
         <v>9</v>
@@ -10328,7 +10328,7 @@
         <v>8</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J15">
         <v>8</v>
@@ -10417,7 +10417,7 @@
         <v>10</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>8</v>
@@ -10506,7 +10506,7 @@
         <v>8</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J17">
         <v>9</v>
@@ -10595,7 +10595,7 @@
         <v>8</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J18">
         <v>10</v>
@@ -10684,7 +10684,7 @@
         <v>-1</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J19">
         <v>5</v>
@@ -10773,7 +10773,7 @@
         <v>7</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J20">
         <v>9</v>
@@ -10862,7 +10862,7 @@
         <v>7</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J21">
         <v>9</v>
@@ -10951,7 +10951,7 @@
         <v>10</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J22">
         <v>9</v>
@@ -11040,7 +11040,7 @@
         <v>7</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J23">
         <v>5</v>
@@ -11082,7 +11082,7 @@
         <v>-1</v>
       </c>
       <c r="W23">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X23">
         <v>5</v>
@@ -11129,7 +11129,7 @@
         <v>6</v>
       </c>
       <c r="I24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J24">
         <v>5</v>
@@ -11171,7 +11171,7 @@
         <v>-1</v>
       </c>
       <c r="W24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X24">
         <v>5</v>
@@ -11218,7 +11218,7 @@
         <v>8</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J25">
         <v>5</v>
@@ -11307,7 +11307,7 @@
         <v>7</v>
       </c>
       <c r="I26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J26">
         <v>9</v>
@@ -11349,7 +11349,7 @@
         <v>-1</v>
       </c>
       <c r="W26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X26">
         <v>9</v>
@@ -11396,7 +11396,7 @@
         <v>6</v>
       </c>
       <c r="I27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J27">
         <v>7</v>
@@ -11438,7 +11438,7 @@
         <v>-1</v>
       </c>
       <c r="W27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X27">
         <v>7</v>
@@ -11485,7 +11485,7 @@
         <v>8</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J28">
         <v>7</v>
@@ -11574,7 +11574,7 @@
         <v>8</v>
       </c>
       <c r="I29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J29">
         <v>9</v>
@@ -11663,7 +11663,7 @@
         <v>7</v>
       </c>
       <c r="I30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J30">
         <v>9</v>
@@ -11752,7 +11752,7 @@
         <v>8</v>
       </c>
       <c r="I31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J31">
         <v>9</v>
@@ -11794,7 +11794,7 @@
         <v>-1</v>
       </c>
       <c r="W31">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X31">
         <v>8</v>
@@ -11841,7 +11841,7 @@
         <v>7</v>
       </c>
       <c r="I32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J32">
         <v>5</v>
@@ -11883,7 +11883,7 @@
         <v>-1</v>
       </c>
       <c r="W32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X32">
         <v>5</v>
@@ -11930,7 +11930,7 @@
         <v>7</v>
       </c>
       <c r="I33">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J33">
         <v>7</v>
@@ -12019,7 +12019,7 @@
         <v>6</v>
       </c>
       <c r="I34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J34">
         <v>7</v>
@@ -12108,7 +12108,7 @@
         <v>8</v>
       </c>
       <c r="I35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J35">
         <v>9</v>
@@ -36713,7 +36713,7 @@
         <v>5</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J6">
         <v>-1</v>
@@ -37204,7 +37204,7 @@
         <v>8</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J13">
         <v>9</v>
@@ -37666,7 +37666,7 @@
         <v>7</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J19">
         <v>-1</v>
@@ -37702,7 +37702,7 @@
         <v>7</v>
       </c>
       <c r="U19">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V19">
         <v>9</v>
@@ -38116,7 +38116,7 @@
         <v>6</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J25">
         <v>8</v>
@@ -38347,7 +38347,7 @@
         <v>5</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J28">
         <v>-1</v>
@@ -38915,7 +38915,7 @@
         <v>6</v>
       </c>
       <c r="I36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J36">
         <v>9</v>
@@ -38992,7 +38992,7 @@
         <v>5</v>
       </c>
       <c r="I37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J37">
         <v>9</v>
@@ -43474,7 +43474,7 @@
         <v>7</v>
       </c>
       <c r="F21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="G21">
         <v>10</v>
@@ -43492,7 +43492,7 @@
         <v>7</v>
       </c>
       <c r="L21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M21">
         <v>10</v>
@@ -43528,7 +43528,7 @@
         <v>7</v>
       </c>
       <c r="X21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Y21">
         <v>10</v>
@@ -43877,7 +43877,7 @@
         <v>6</v>
       </c>
       <c r="L26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="M26">
         <v>10</v>
@@ -52638,7 +52638,7 @@
         <v>10</v>
       </c>
       <c r="J4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K4">
         <v>9</v>
@@ -52680,7 +52680,7 @@
         <v>10</v>
       </c>
       <c r="X4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y4">
         <v>10</v>
@@ -52706,7 +52706,7 @@
         <v>7</v>
       </c>
       <c r="C5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D5">
         <v>7</v>
@@ -52769,7 +52769,7 @@
         <v>7</v>
       </c>
       <c r="X5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Y5">
         <v>7</v>
@@ -52816,7 +52816,7 @@
         <v>10</v>
       </c>
       <c r="J6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K6">
         <v>10</v>
@@ -52858,7 +52858,7 @@
         <v>10</v>
       </c>
       <c r="X6">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y6">
         <v>10</v>
@@ -52884,7 +52884,7 @@
         <v>8</v>
       </c>
       <c r="C7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D7">
         <v>9</v>
@@ -52947,7 +52947,7 @@
         <v>7</v>
       </c>
       <c r="X7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Y7">
         <v>9</v>
@@ -52973,7 +52973,7 @@
         <v>6</v>
       </c>
       <c r="C8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>6</v>
@@ -53036,7 +53036,7 @@
         <v>6</v>
       </c>
       <c r="X8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Y8">
         <v>6</v>
@@ -53062,7 +53062,7 @@
         <v>7</v>
       </c>
       <c r="C9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D9">
         <v>7</v>
@@ -53083,7 +53083,7 @@
         <v>8</v>
       </c>
       <c r="J9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K9">
         <v>10</v>
@@ -53125,7 +53125,7 @@
         <v>8</v>
       </c>
       <c r="X9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y9">
         <v>9</v>
@@ -53261,7 +53261,7 @@
         <v>9</v>
       </c>
       <c r="J11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K11">
         <v>10</v>
@@ -53350,7 +53350,7 @@
         <v>10</v>
       </c>
       <c r="J12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K12">
         <v>10</v>
@@ -53392,7 +53392,7 @@
         <v>10</v>
       </c>
       <c r="X12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y12">
         <v>10</v>
@@ -53418,7 +53418,7 @@
         <v>6</v>
       </c>
       <c r="C13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>10</v>
@@ -53439,7 +53439,7 @@
         <v>6</v>
       </c>
       <c r="J13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K13">
         <v>9</v>
@@ -53481,7 +53481,7 @@
         <v>6</v>
       </c>
       <c r="X13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y13">
         <v>10</v>
@@ -53507,7 +53507,7 @@
         <v>9</v>
       </c>
       <c r="C14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <v>10</v>
@@ -53528,7 +53528,7 @@
         <v>9</v>
       </c>
       <c r="J14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K14">
         <v>10</v>
@@ -53570,7 +53570,7 @@
         <v>9</v>
       </c>
       <c r="X14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y14">
         <v>10</v>
@@ -53617,7 +53617,7 @@
         <v>8</v>
       </c>
       <c r="J15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K15">
         <v>10</v>
@@ -53659,7 +53659,7 @@
         <v>8</v>
       </c>
       <c r="X15">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y15">
         <v>10</v>
@@ -53706,7 +53706,7 @@
         <v>9</v>
       </c>
       <c r="J16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K16">
         <v>10</v>
@@ -53774,7 +53774,7 @@
         <v>6</v>
       </c>
       <c r="C17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D17">
         <v>7</v>
@@ -53837,7 +53837,7 @@
         <v>6</v>
       </c>
       <c r="X17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Y17">
         <v>8</v>
@@ -53863,7 +53863,7 @@
         <v>10</v>
       </c>
       <c r="C18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D18">
         <v>10</v>
@@ -53884,7 +53884,7 @@
         <v>10</v>
       </c>
       <c r="J18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K18">
         <v>10</v>
@@ -53926,7 +53926,7 @@
         <v>10</v>
       </c>
       <c r="X18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y18">
         <v>10</v>
@@ -54207,7 +54207,7 @@
         <v>6</v>
       </c>
       <c r="C22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -54270,7 +54270,7 @@
         <v>6</v>
       </c>
       <c r="X22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Y22">
         <v>6</v>
@@ -54296,7 +54296,7 @@
         <v>6</v>
       </c>
       <c r="C23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D23">
         <v>-1</v>
@@ -54359,7 +54359,7 @@
         <v>6</v>
       </c>
       <c r="X23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Y23">
         <v>-1</v>

</xml_diff>

<commit_message>
Primer Parcial 2022 Final
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -55731,7 +55731,7 @@
         <v>7</v>
       </c>
       <c r="F4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G4">
         <v>-1</v>
@@ -55785,7 +55785,7 @@
         <v>7</v>
       </c>
       <c r="X4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y4">
         <v>-1</v>
@@ -56193,7 +56193,7 @@
         <v>-1</v>
       </c>
       <c r="F10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G10">
         <v>9</v>
@@ -56247,7 +56247,7 @@
         <v>-1</v>
       </c>
       <c r="X10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y10">
         <v>9</v>
@@ -56501,7 +56501,7 @@
         <v>-1</v>
       </c>
       <c r="F14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G14">
         <v>-1</v>
@@ -56555,7 +56555,7 @@
         <v>-1</v>
       </c>
       <c r="X14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y14">
         <v>-1</v>
@@ -56732,7 +56732,7 @@
         <v>8</v>
       </c>
       <c r="F17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G17">
         <v>8</v>
@@ -56786,7 +56786,7 @@
         <v>8</v>
       </c>
       <c r="X17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y17">
         <v>8</v>
@@ -57040,7 +57040,7 @@
         <v>6</v>
       </c>
       <c r="F21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G21">
         <v>-1</v>
@@ -57094,7 +57094,7 @@
         <v>6</v>
       </c>
       <c r="X21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y21">
         <v>-1</v>
@@ -57117,7 +57117,7 @@
         <v>-1</v>
       </c>
       <c r="F22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G22">
         <v>7</v>
@@ -57171,7 +57171,7 @@
         <v>-1</v>
       </c>
       <c r="X22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y22">
         <v>7</v>
@@ -57271,7 +57271,7 @@
         <v>7</v>
       </c>
       <c r="F24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G24">
         <v>7</v>
@@ -57325,7 +57325,7 @@
         <v>7</v>
       </c>
       <c r="X24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y24">
         <v>7</v>
@@ -57483,7 +57483,7 @@
         <v>8</v>
       </c>
       <c r="F28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G28">
         <v>-1</v>
@@ -57537,7 +57537,7 @@
         <v>8</v>
       </c>
       <c r="X28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y28">
         <v>-1</v>
@@ -57560,7 +57560,7 @@
         <v>-1</v>
       </c>
       <c r="F29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G29">
         <v>-1</v>
@@ -57614,7 +57614,7 @@
         <v>-1</v>
       </c>
       <c r="X29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y29">
         <v>-1</v>
@@ -71712,7 +71712,7 @@
         <v>-1</v>
       </c>
       <c r="G12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H12">
         <v>-1</v>
@@ -71766,7 +71766,7 @@
         <v>-1</v>
       </c>
       <c r="Y12">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -72328,7 +72328,7 @@
         <v>-1</v>
       </c>
       <c r="G20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="H20">
         <v>-1</v>
@@ -72382,7 +72382,7 @@
         <v>-1</v>
       </c>
       <c r="Y20">
-        <v>-1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:25">
@@ -73707,7 +73707,7 @@
         <v>-1</v>
       </c>
       <c r="G39">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H39">
         <v>-1</v>
@@ -73761,7 +73761,7 @@
         <v>-1</v>
       </c>
       <c r="Y39">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40" spans="1:25">
@@ -73772,7 +73772,7 @@
         <v>8</v>
       </c>
       <c r="G40">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L40">
         <v>-1</v>
@@ -73790,7 +73790,7 @@
         <v>8</v>
       </c>
       <c r="Y40">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41" spans="1:25">

</xml_diff>

<commit_message>
Primer Parcial Actualizacion 3 Octubre
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -2214,6 +2214,9 @@
     <t>GUERRA RIVERA CLAUDIA PAOLA</t>
   </si>
   <si>
+    <t>HERNANDEZ CADENA DANA PAOLA</t>
+  </si>
+  <si>
     <t>HERNANDEZ ROJAS LILIANA</t>
   </si>
   <si>
@@ -2221,9 +2224,6 @@
   </si>
   <si>
     <t>JIMENEZ COLMENARES ROSARIO DE JESUS</t>
-  </si>
-  <si>
-    <t>MARTINEZ PEREZ KATIA GUADALUPE</t>
   </si>
   <si>
     <t>MARTINEZ RODRIGUEZ EVIAN ISSAIAS</t>
@@ -38423,16 +38423,16 @@
         <v>-1</v>
       </c>
       <c r="D16">
-        <v>8</v>
+        <v>-1</v>
       </c>
       <c r="E16">
         <v>-1</v>
       </c>
       <c r="F16">
-        <v>7</v>
+        <v>-1</v>
       </c>
       <c r="G16">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="H16">
         <v>-1</v>
@@ -38477,16 +38477,16 @@
         <v>-1</v>
       </c>
       <c r="V16">
-        <v>8</v>
+        <v>-1</v>
       </c>
       <c r="W16">
         <v>-1</v>
       </c>
       <c r="X16">
-        <v>7</v>
+        <v>-1</v>
       </c>
       <c r="Y16">
-        <v>6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="17" spans="1:25">
@@ -38494,19 +38494,19 @@
         <v>723</v>
       </c>
       <c r="B17">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="C17">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="D17">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E17">
         <v>-1</v>
       </c>
       <c r="F17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G17">
         <v>6</v>
@@ -38548,19 +38548,19 @@
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="U17">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="V17">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W17">
         <v>-1</v>
       </c>
       <c r="X17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y17">
         <v>6</v>
@@ -38571,22 +38571,22 @@
         <v>724</v>
       </c>
       <c r="B18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C18">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18">
-        <v>9</v>
+        <v>-1</v>
       </c>
       <c r="F18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G18">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H18">
         <v>-1</v>
@@ -38625,22 +38625,22 @@
         <v>-1</v>
       </c>
       <c r="T18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U18">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="V18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W18">
-        <v>9</v>
+        <v>-1</v>
       </c>
       <c r="X18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y18">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:25">
@@ -38648,22 +38648,22 @@
         <v>725</v>
       </c>
       <c r="B19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="C19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="D19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E19">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="G19">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H19">
         <v>-1</v>
@@ -38702,22 +38702,22 @@
         <v>-1</v>
       </c>
       <c r="T19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="U19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W19">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="X19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y19">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:25">
@@ -49747,7 +49747,7 @@
         <v>-1</v>
       </c>
       <c r="D4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E4">
         <v>5</v>
@@ -49801,7 +49801,7 @@
         <v>-1</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W4">
         <v>5</v>
@@ -49889,7 +49889,7 @@
         <v>6</v>
       </c>
       <c r="D6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E6">
         <v>6</v>
@@ -49943,7 +49943,7 @@
         <v>6</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>6</v>
@@ -49966,7 +49966,7 @@
         <v>-1</v>
       </c>
       <c r="D7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -50020,7 +50020,7 @@
         <v>-1</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W7">
         <v>6</v>
@@ -50072,7 +50072,7 @@
         <v>6</v>
       </c>
       <c r="D9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E9">
         <v>7</v>
@@ -50126,7 +50126,7 @@
         <v>6</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W9">
         <v>7</v>
@@ -50149,7 +50149,7 @@
         <v>-1</v>
       </c>
       <c r="D10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E10">
         <v>5</v>
@@ -50203,7 +50203,7 @@
         <v>-1</v>
       </c>
       <c r="V10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W10">
         <v>5</v>
@@ -50226,7 +50226,7 @@
         <v>9</v>
       </c>
       <c r="D11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="E11">
         <v>8</v>
@@ -50280,7 +50280,7 @@
         <v>9</v>
       </c>
       <c r="V11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W11">
         <v>8</v>
@@ -50303,7 +50303,7 @@
         <v>8</v>
       </c>
       <c r="D12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E12">
         <v>8</v>
@@ -50357,7 +50357,7 @@
         <v>8</v>
       </c>
       <c r="V12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W12">
         <v>8</v>
@@ -50380,7 +50380,7 @@
         <v>8</v>
       </c>
       <c r="D13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E13">
         <v>6</v>
@@ -50434,7 +50434,7 @@
         <v>8</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W13">
         <v>6</v>
@@ -50534,7 +50534,7 @@
         <v>6</v>
       </c>
       <c r="D15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E15">
         <v>9</v>
@@ -50588,7 +50588,7 @@
         <v>6</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W15">
         <v>9</v>
@@ -50611,7 +50611,7 @@
         <v>8</v>
       </c>
       <c r="D16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E16">
         <v>6</v>
@@ -50665,7 +50665,7 @@
         <v>8</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W16">
         <v>6</v>
@@ -50688,7 +50688,7 @@
         <v>10</v>
       </c>
       <c r="D17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E17">
         <v>8</v>
@@ -50742,7 +50742,7 @@
         <v>10</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W17">
         <v>8</v>
@@ -50765,7 +50765,7 @@
         <v>8</v>
       </c>
       <c r="D18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="E18">
         <v>6</v>
@@ -50819,7 +50819,7 @@
         <v>8</v>
       </c>
       <c r="V18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W18">
         <v>6</v>
@@ -50859,7 +50859,7 @@
         <v>9</v>
       </c>
       <c r="D20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E20">
         <v>8</v>
@@ -50913,7 +50913,7 @@
         <v>9</v>
       </c>
       <c r="V20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W20">
         <v>8</v>
@@ -50936,7 +50936,7 @@
         <v>7</v>
       </c>
       <c r="D21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E21">
         <v>8</v>
@@ -50990,7 +50990,7 @@
         <v>7</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W21">
         <v>8</v>
@@ -51013,7 +51013,7 @@
         <v>8</v>
       </c>
       <c r="D22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E22">
         <v>8</v>
@@ -51067,7 +51067,7 @@
         <v>8</v>
       </c>
       <c r="V22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W22">
         <v>8</v>
@@ -51090,7 +51090,7 @@
         <v>10</v>
       </c>
       <c r="D23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E23">
         <v>7</v>
@@ -51144,7 +51144,7 @@
         <v>10</v>
       </c>
       <c r="V23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W23">
         <v>7</v>
@@ -51167,7 +51167,7 @@
         <v>10</v>
       </c>
       <c r="D24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E24">
         <v>8</v>
@@ -51221,7 +51221,7 @@
         <v>10</v>
       </c>
       <c r="V24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W24">
         <v>8</v>
@@ -51244,7 +51244,7 @@
         <v>10</v>
       </c>
       <c r="D25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E25">
         <v>8</v>
@@ -51298,7 +51298,7 @@
         <v>10</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W25">
         <v>8</v>
@@ -51321,7 +51321,7 @@
         <v>10</v>
       </c>
       <c r="D26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E26">
         <v>8</v>
@@ -51375,7 +51375,7 @@
         <v>10</v>
       </c>
       <c r="V26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W26">
         <v>8</v>
@@ -51439,7 +51439,7 @@
         <v>9</v>
       </c>
       <c r="D28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E28">
         <v>9</v>
@@ -51493,7 +51493,7 @@
         <v>9</v>
       </c>
       <c r="V28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W28">
         <v>9</v>
@@ -51670,7 +51670,7 @@
         <v>7</v>
       </c>
       <c r="D31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="E31">
         <v>6</v>
@@ -51724,7 +51724,7 @@
         <v>7</v>
       </c>
       <c r="V31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W31">
         <v>6</v>
@@ -51747,7 +51747,7 @@
         <v>10</v>
       </c>
       <c r="D32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="E32">
         <v>8</v>
@@ -51801,7 +51801,7 @@
         <v>10</v>
       </c>
       <c r="V32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W32">
         <v>8</v>
@@ -51853,7 +51853,7 @@
         <v>9</v>
       </c>
       <c r="D34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="E34">
         <v>9</v>
@@ -51907,7 +51907,7 @@
         <v>9</v>
       </c>
       <c r="V34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W34">
         <v>9</v>
@@ -51930,7 +51930,7 @@
         <v>9</v>
       </c>
       <c r="D35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="E35">
         <v>6</v>
@@ -51984,7 +51984,7 @@
         <v>9</v>
       </c>
       <c r="V35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W35">
         <v>6</v>
@@ -52007,7 +52007,7 @@
         <v>8</v>
       </c>
       <c r="D36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="E36">
         <v>7</v>
@@ -52061,7 +52061,7 @@
         <v>8</v>
       </c>
       <c r="V36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W36">
         <v>7</v>
@@ -52084,7 +52084,7 @@
         <v>8</v>
       </c>
       <c r="D37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E37">
         <v>9</v>
@@ -52138,7 +52138,7 @@
         <v>8</v>
       </c>
       <c r="V37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W37">
         <v>9</v>
@@ -52238,7 +52238,7 @@
         <v>7</v>
       </c>
       <c r="D39">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E39">
         <v>7</v>
@@ -52292,7 +52292,7 @@
         <v>7</v>
       </c>
       <c r="V39">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W39">
         <v>7</v>
@@ -52315,7 +52315,7 @@
         <v>9</v>
       </c>
       <c r="D40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="E40">
         <v>9</v>
@@ -52369,7 +52369,7 @@
         <v>9</v>
       </c>
       <c r="V40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W40">
         <v>9</v>
@@ -52392,7 +52392,7 @@
         <v>-1</v>
       </c>
       <c r="D41">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E41">
         <v>6</v>
@@ -52446,7 +52446,7 @@
         <v>-1</v>
       </c>
       <c r="V41">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W41">
         <v>6</v>
@@ -52640,7 +52640,7 @@
         <v>9</v>
       </c>
       <c r="F4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G4">
         <v>8</v>
@@ -52694,7 +52694,7 @@
         <v>9</v>
       </c>
       <c r="X4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y4">
         <v>8</v>
@@ -52871,7 +52871,7 @@
         <v>9</v>
       </c>
       <c r="F7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="G7">
         <v>8</v>
@@ -52925,7 +52925,7 @@
         <v>9</v>
       </c>
       <c r="X7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Y7">
         <v>8</v>
@@ -52948,7 +52948,7 @@
         <v>9</v>
       </c>
       <c r="F8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="G8">
         <v>8</v>
@@ -53002,7 +53002,7 @@
         <v>9</v>
       </c>
       <c r="X8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Y8">
         <v>8</v>
@@ -53025,7 +53025,7 @@
         <v>9</v>
       </c>
       <c r="F9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="G9">
         <v>8</v>
@@ -53079,7 +53079,7 @@
         <v>9</v>
       </c>
       <c r="X9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y9">
         <v>8</v>
@@ -53102,7 +53102,7 @@
         <v>9</v>
       </c>
       <c r="F10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="G10">
         <v>9</v>
@@ -53156,7 +53156,7 @@
         <v>9</v>
       </c>
       <c r="X10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Y10">
         <v>9</v>
@@ -53179,7 +53179,7 @@
         <v>9</v>
       </c>
       <c r="F11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="G11">
         <v>7</v>
@@ -53233,7 +53233,7 @@
         <v>9</v>
       </c>
       <c r="X11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Y11">
         <v>7</v>
@@ -53256,7 +53256,7 @@
         <v>9</v>
       </c>
       <c r="F12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="G12">
         <v>9</v>
@@ -53310,7 +53310,7 @@
         <v>9</v>
       </c>
       <c r="X12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Y12">
         <v>9</v>
@@ -53333,7 +53333,7 @@
         <v>9</v>
       </c>
       <c r="F13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G13">
         <v>7</v>
@@ -53387,7 +53387,7 @@
         <v>9</v>
       </c>
       <c r="X13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y13">
         <v>7</v>
@@ -53410,7 +53410,7 @@
         <v>7</v>
       </c>
       <c r="F14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="G14">
         <v>6</v>
@@ -53464,7 +53464,7 @@
         <v>7</v>
       </c>
       <c r="X14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y14">
         <v>6</v>
@@ -53487,7 +53487,7 @@
         <v>9</v>
       </c>
       <c r="F15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="G15">
         <v>7</v>
@@ -53541,7 +53541,7 @@
         <v>9</v>
       </c>
       <c r="X15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Y15">
         <v>7</v>
@@ -53564,7 +53564,7 @@
         <v>10</v>
       </c>
       <c r="F16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="G16">
         <v>9</v>
@@ -53618,7 +53618,7 @@
         <v>10</v>
       </c>
       <c r="X16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Y16">
         <v>9</v>
@@ -53641,7 +53641,7 @@
         <v>6</v>
       </c>
       <c r="F17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="G17">
         <v>-1</v>
@@ -53695,7 +53695,7 @@
         <v>6</v>
       </c>
       <c r="X17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y17">
         <v>-1</v>
@@ -53718,7 +53718,7 @@
         <v>9</v>
       </c>
       <c r="F18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="G18">
         <v>6</v>
@@ -53772,7 +53772,7 @@
         <v>9</v>
       </c>
       <c r="X18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y18">
         <v>6</v>
@@ -53795,7 +53795,7 @@
         <v>9</v>
       </c>
       <c r="F19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G19">
         <v>9</v>
@@ -53849,7 +53849,7 @@
         <v>9</v>
       </c>
       <c r="X19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y19">
         <v>9</v>
@@ -53872,7 +53872,7 @@
         <v>9</v>
       </c>
       <c r="F20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="G20">
         <v>10</v>
@@ -53926,7 +53926,7 @@
         <v>9</v>
       </c>
       <c r="X20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Y20">
         <v>10</v>
@@ -53949,7 +53949,7 @@
         <v>9</v>
       </c>
       <c r="F21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G21">
         <v>6</v>
@@ -54003,7 +54003,7 @@
         <v>9</v>
       </c>
       <c r="X21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y21">
         <v>6</v>
@@ -54026,7 +54026,7 @@
         <v>8</v>
       </c>
       <c r="F22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G22">
         <v>6</v>
@@ -54080,7 +54080,7 @@
         <v>8</v>
       </c>
       <c r="X22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y22">
         <v>6</v>
@@ -54103,7 +54103,7 @@
         <v>8</v>
       </c>
       <c r="F23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="G23">
         <v>6</v>
@@ -54157,7 +54157,7 @@
         <v>8</v>
       </c>
       <c r="X23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Y23">
         <v>6</v>
@@ -54209,7 +54209,7 @@
         <v>9</v>
       </c>
       <c r="F25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G25">
         <v>8</v>
@@ -54263,7 +54263,7 @@
         <v>9</v>
       </c>
       <c r="X25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y25">
         <v>8</v>
@@ -54286,7 +54286,7 @@
         <v>8</v>
       </c>
       <c r="F26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="G26">
         <v>6</v>
@@ -54340,7 +54340,7 @@
         <v>8</v>
       </c>
       <c r="X26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Y26">
         <v>6</v>
@@ -54363,7 +54363,7 @@
         <v>10</v>
       </c>
       <c r="F27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="G27">
         <v>9</v>
@@ -54417,7 +54417,7 @@
         <v>10</v>
       </c>
       <c r="X27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Y27">
         <v>9</v>
@@ -54440,7 +54440,7 @@
         <v>9</v>
       </c>
       <c r="F28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G28">
         <v>8</v>
@@ -54494,7 +54494,7 @@
         <v>9</v>
       </c>
       <c r="X28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y28">
         <v>8</v>
@@ -54517,7 +54517,7 @@
         <v>7</v>
       </c>
       <c r="F29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="G29">
         <v>9</v>
@@ -54571,7 +54571,7 @@
         <v>7</v>
       </c>
       <c r="X29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Y29">
         <v>9</v>
@@ -54671,7 +54671,7 @@
         <v>9</v>
       </c>
       <c r="F31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G31">
         <v>8</v>
@@ -54725,7 +54725,7 @@
         <v>9</v>
       </c>
       <c r="X31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y31">
         <v>8</v>
@@ -54748,7 +54748,7 @@
         <v>8</v>
       </c>
       <c r="F32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="G32">
         <v>7</v>
@@ -54802,7 +54802,7 @@
         <v>8</v>
       </c>
       <c r="X32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Y32">
         <v>7</v>
@@ -54825,7 +54825,7 @@
         <v>9</v>
       </c>
       <c r="F33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="G33">
         <v>6</v>
@@ -54879,7 +54879,7 @@
         <v>9</v>
       </c>
       <c r="X33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Y33">
         <v>6</v>
@@ -54902,7 +54902,7 @@
         <v>9</v>
       </c>
       <c r="F34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G34">
         <v>9</v>
@@ -54956,7 +54956,7 @@
         <v>9</v>
       </c>
       <c r="X34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y34">
         <v>9</v>
@@ -54979,7 +54979,7 @@
         <v>8</v>
       </c>
       <c r="F35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G35">
         <v>6</v>
@@ -55033,7 +55033,7 @@
         <v>8</v>
       </c>
       <c r="X35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y35">
         <v>6</v>
@@ -55056,7 +55056,7 @@
         <v>8</v>
       </c>
       <c r="F36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="G36">
         <v>6</v>
@@ -55110,7 +55110,7 @@
         <v>8</v>
       </c>
       <c r="X36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Y36">
         <v>6</v>
@@ -55133,7 +55133,7 @@
         <v>8</v>
       </c>
       <c r="F37">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G37">
         <v>8</v>
@@ -55187,7 +55187,7 @@
         <v>8</v>
       </c>
       <c r="X37">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y37">
         <v>8</v>
@@ -55210,7 +55210,7 @@
         <v>5</v>
       </c>
       <c r="F38">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G38">
         <v>-1</v>
@@ -55264,7 +55264,7 @@
         <v>5</v>
       </c>
       <c r="X38">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y38">
         <v>-1</v>
@@ -55287,7 +55287,7 @@
         <v>9</v>
       </c>
       <c r="F39">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="G39">
         <v>9</v>
@@ -55341,7 +55341,7 @@
         <v>9</v>
       </c>
       <c r="X39">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Y39">
         <v>9</v>
@@ -55364,7 +55364,7 @@
         <v>9</v>
       </c>
       <c r="F40">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G40">
         <v>8</v>
@@ -55418,7 +55418,7 @@
         <v>9</v>
       </c>
       <c r="X40">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y40">
         <v>8</v>
@@ -55518,7 +55518,7 @@
         <v>9</v>
       </c>
       <c r="F42">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="G42">
         <v>9</v>
@@ -55572,7 +55572,7 @@
         <v>9</v>
       </c>
       <c r="X42">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Y42">
         <v>9</v>
@@ -57847,7 +57847,7 @@
         <v>7</v>
       </c>
       <c r="E4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="F4">
         <v>9</v>
@@ -57901,7 +57901,7 @@
         <v>7</v>
       </c>
       <c r="W4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="X4">
         <v>9</v>
@@ -57924,7 +57924,7 @@
         <v>8</v>
       </c>
       <c r="E5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F5">
         <v>8</v>
@@ -57978,7 +57978,7 @@
         <v>8</v>
       </c>
       <c r="W5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X5">
         <v>8</v>
@@ -58001,7 +58001,7 @@
         <v>10</v>
       </c>
       <c r="E6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F6">
         <v>10</v>
@@ -58055,7 +58055,7 @@
         <v>10</v>
       </c>
       <c r="W6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X6">
         <v>10</v>
@@ -58078,7 +58078,7 @@
         <v>-1</v>
       </c>
       <c r="E7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="F7">
         <v>6</v>
@@ -58132,7 +58132,7 @@
         <v>-1</v>
       </c>
       <c r="W7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="X7">
         <v>6</v>
@@ -58155,7 +58155,7 @@
         <v>8</v>
       </c>
       <c r="E8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F8">
         <v>8</v>
@@ -58209,7 +58209,7 @@
         <v>8</v>
       </c>
       <c r="W8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X8">
         <v>8</v>
@@ -58232,7 +58232,7 @@
         <v>-1</v>
       </c>
       <c r="E9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="F9">
         <v>8</v>
@@ -58286,7 +58286,7 @@
         <v>-1</v>
       </c>
       <c r="W9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="X9">
         <v>8</v>
@@ -58309,7 +58309,7 @@
         <v>-1</v>
       </c>
       <c r="E10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="F10">
         <v>7</v>
@@ -58363,7 +58363,7 @@
         <v>-1</v>
       </c>
       <c r="W10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="X10">
         <v>7</v>
@@ -58386,7 +58386,7 @@
         <v>9</v>
       </c>
       <c r="E11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F11">
         <v>10</v>
@@ -58440,7 +58440,7 @@
         <v>9</v>
       </c>
       <c r="W11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X11">
         <v>10</v>
@@ -58463,7 +58463,7 @@
         <v>8</v>
       </c>
       <c r="E12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F12">
         <v>10</v>
@@ -58517,7 +58517,7 @@
         <v>8</v>
       </c>
       <c r="W12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X12">
         <v>10</v>
@@ -58540,7 +58540,7 @@
         <v>9</v>
       </c>
       <c r="E13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F13">
         <v>8</v>
@@ -58594,7 +58594,7 @@
         <v>9</v>
       </c>
       <c r="W13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X13">
         <v>8</v>
@@ -58617,7 +58617,7 @@
         <v>8</v>
       </c>
       <c r="E14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="F14">
         <v>9</v>
@@ -58671,7 +58671,7 @@
         <v>8</v>
       </c>
       <c r="W14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="X14">
         <v>9</v>
@@ -58694,7 +58694,7 @@
         <v>10</v>
       </c>
       <c r="E15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F15">
         <v>9</v>
@@ -58748,7 +58748,7 @@
         <v>10</v>
       </c>
       <c r="W15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X15">
         <v>9</v>
@@ -58771,7 +58771,7 @@
         <v>8</v>
       </c>
       <c r="E16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="F16">
         <v>10</v>
@@ -58825,7 +58825,7 @@
         <v>8</v>
       </c>
       <c r="W16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="X16">
         <v>10</v>
@@ -58848,7 +58848,7 @@
         <v>7</v>
       </c>
       <c r="E17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="F17">
         <v>8</v>
@@ -58902,7 +58902,7 @@
         <v>7</v>
       </c>
       <c r="W17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="X17">
         <v>8</v>
@@ -58925,7 +58925,7 @@
         <v>10</v>
       </c>
       <c r="E18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F18">
         <v>10</v>
@@ -58979,7 +58979,7 @@
         <v>10</v>
       </c>
       <c r="W18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X18">
         <v>10</v>
@@ -59002,7 +59002,7 @@
         <v>7</v>
       </c>
       <c r="E19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F19">
         <v>8</v>
@@ -59056,7 +59056,7 @@
         <v>7</v>
       </c>
       <c r="W19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X19">
         <v>8</v>
@@ -59079,7 +59079,7 @@
         <v>9</v>
       </c>
       <c r="E20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F20">
         <v>10</v>
@@ -59133,7 +59133,7 @@
         <v>9</v>
       </c>
       <c r="W20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X20">
         <v>10</v>
@@ -59156,7 +59156,7 @@
         <v>9</v>
       </c>
       <c r="E21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F21">
         <v>8</v>
@@ -59210,7 +59210,7 @@
         <v>9</v>
       </c>
       <c r="W21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X21">
         <v>8</v>
@@ -59310,7 +59310,7 @@
         <v>9</v>
       </c>
       <c r="E23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F23">
         <v>9</v>
@@ -59364,7 +59364,7 @@
         <v>9</v>
       </c>
       <c r="W23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X23">
         <v>9</v>
@@ -59387,7 +59387,7 @@
         <v>8</v>
       </c>
       <c r="E24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F24">
         <v>10</v>
@@ -59441,7 +59441,7 @@
         <v>8</v>
       </c>
       <c r="W24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X24">
         <v>10</v>
@@ -59464,7 +59464,7 @@
         <v>9</v>
       </c>
       <c r="E25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F25">
         <v>10</v>
@@ -59518,7 +59518,7 @@
         <v>9</v>
       </c>
       <c r="W25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X25">
         <v>10</v>
@@ -59541,7 +59541,7 @@
         <v>-1</v>
       </c>
       <c r="E26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F26">
         <v>6</v>
@@ -59595,7 +59595,7 @@
         <v>-1</v>
       </c>
       <c r="W26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X26">
         <v>6</v>
@@ -59618,7 +59618,7 @@
         <v>7</v>
       </c>
       <c r="E27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F27">
         <v>9</v>
@@ -59672,7 +59672,7 @@
         <v>7</v>
       </c>
       <c r="W27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X27">
         <v>9</v>
@@ -59695,7 +59695,7 @@
         <v>6</v>
       </c>
       <c r="E28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F28">
         <v>8</v>
@@ -59749,7 +59749,7 @@
         <v>6</v>
       </c>
       <c r="W28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X28">
         <v>8</v>
@@ -59772,7 +59772,7 @@
         <v>9</v>
       </c>
       <c r="E29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F29">
         <v>10</v>
@@ -59826,7 +59826,7 @@
         <v>9</v>
       </c>
       <c r="W29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X29">
         <v>10</v>
@@ -59849,7 +59849,7 @@
         <v>7</v>
       </c>
       <c r="E30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F30">
         <v>8</v>
@@ -59903,7 +59903,7 @@
         <v>7</v>
       </c>
       <c r="W30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X30">
         <v>8</v>
@@ -59926,7 +59926,7 @@
         <v>6</v>
       </c>
       <c r="E31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F31">
         <v>8</v>
@@ -59980,7 +59980,7 @@
         <v>6</v>
       </c>
       <c r="W31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X31">
         <v>8</v>
@@ -60080,7 +60080,7 @@
         <v>8</v>
       </c>
       <c r="E33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F33">
         <v>10</v>
@@ -60134,7 +60134,7 @@
         <v>8</v>
       </c>
       <c r="W33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X33">
         <v>10</v>
@@ -60157,7 +60157,7 @@
         <v>7</v>
       </c>
       <c r="E34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="F34">
         <v>10</v>
@@ -60211,7 +60211,7 @@
         <v>7</v>
       </c>
       <c r="W34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="X34">
         <v>10</v>
@@ -60234,7 +60234,7 @@
         <v>-1</v>
       </c>
       <c r="E35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="F35">
         <v>5</v>
@@ -60288,7 +60288,7 @@
         <v>-1</v>
       </c>
       <c r="W35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="X35">
         <v>5</v>
@@ -61760,7 +61760,7 @@
         <v>9</v>
       </c>
       <c r="G4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="H4">
         <v>7</v>
@@ -61823,7 +61823,7 @@
         <v>9</v>
       </c>
       <c r="AB4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AC4">
         <v>7</v>
@@ -61849,7 +61849,7 @@
         <v>9</v>
       </c>
       <c r="G5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="H5">
         <v>5</v>
@@ -61912,7 +61912,7 @@
         <v>9</v>
       </c>
       <c r="AB5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="AC5">
         <v>5</v>
@@ -61938,7 +61938,7 @@
         <v>10</v>
       </c>
       <c r="G6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H6">
         <v>7</v>
@@ -62001,7 +62001,7 @@
         <v>10</v>
       </c>
       <c r="AB6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="AC6">
         <v>7</v>
@@ -62027,7 +62027,7 @@
         <v>10</v>
       </c>
       <c r="G7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="H7">
         <v>10</v>
@@ -62090,7 +62090,7 @@
         <v>10</v>
       </c>
       <c r="AB7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AC7">
         <v>10</v>
@@ -62101,7 +62101,7 @@
         <v>1020</v>
       </c>
       <c r="B8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="C8">
         <v>5</v>
@@ -62164,7 +62164,7 @@
         <v>-1</v>
       </c>
       <c r="W8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="X8">
         <v>5</v>
@@ -62279,7 +62279,7 @@
         <v>1022</v>
       </c>
       <c r="B10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="C10">
         <v>7</v>
@@ -62342,7 +62342,7 @@
         <v>-1</v>
       </c>
       <c r="W10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="X10">
         <v>7</v>
@@ -62472,7 +62472,7 @@
         <v>9</v>
       </c>
       <c r="G12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="H12">
         <v>7</v>
@@ -62535,7 +62535,7 @@
         <v>9</v>
       </c>
       <c r="AB12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AC12">
         <v>7</v>
@@ -62561,7 +62561,7 @@
         <v>6</v>
       </c>
       <c r="G13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H13">
         <v>8</v>
@@ -62624,7 +62624,7 @@
         <v>6</v>
       </c>
       <c r="AB13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="AC13">
         <v>8</v>
@@ -62650,7 +62650,7 @@
         <v>10</v>
       </c>
       <c r="G14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="H14">
         <v>7</v>
@@ -62713,7 +62713,7 @@
         <v>10</v>
       </c>
       <c r="AB14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AC14">
         <v>7</v>
@@ -62828,7 +62828,7 @@
         <v>6</v>
       </c>
       <c r="G16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H16">
         <v>5</v>
@@ -62891,7 +62891,7 @@
         <v>6</v>
       </c>
       <c r="AB16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="AC16">
         <v>5</v>
@@ -62917,7 +62917,7 @@
         <v>-1</v>
       </c>
       <c r="G17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H17">
         <v>7</v>
@@ -62980,7 +62980,7 @@
         <v>-1</v>
       </c>
       <c r="AB17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="AC17">
         <v>7</v>
@@ -63095,7 +63095,7 @@
         <v>6</v>
       </c>
       <c r="G19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="H19">
         <v>8</v>
@@ -63158,7 +63158,7 @@
         <v>6</v>
       </c>
       <c r="AB19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AC19">
         <v>8</v>
@@ -63184,7 +63184,7 @@
         <v>-1</v>
       </c>
       <c r="G20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H20">
         <v>5</v>
@@ -63247,7 +63247,7 @@
         <v>-1</v>
       </c>
       <c r="AB20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="AC20">
         <v>5</v>
@@ -63273,7 +63273,7 @@
         <v>-1</v>
       </c>
       <c r="G21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="H21">
         <v>5</v>
@@ -63336,7 +63336,7 @@
         <v>-1</v>
       </c>
       <c r="AB21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AC21">
         <v>5</v>
@@ -63362,7 +63362,7 @@
         <v>9</v>
       </c>
       <c r="G22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="H22">
         <v>8</v>
@@ -63425,7 +63425,7 @@
         <v>9</v>
       </c>
       <c r="AB22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AC22">
         <v>8</v>
@@ -63451,7 +63451,7 @@
         <v>10</v>
       </c>
       <c r="G23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="H23">
         <v>10</v>
@@ -63514,7 +63514,7 @@
         <v>10</v>
       </c>
       <c r="AB23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="AC23">
         <v>10</v>
@@ -63540,7 +63540,7 @@
         <v>10</v>
       </c>
       <c r="G24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H24">
         <v>7</v>
@@ -63603,7 +63603,7 @@
         <v>10</v>
       </c>
       <c r="AB24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="AC24">
         <v>7</v>
@@ -63614,7 +63614,7 @@
         <v>1037</v>
       </c>
       <c r="B25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="C25">
         <v>5</v>
@@ -63677,7 +63677,7 @@
         <v>-1</v>
       </c>
       <c r="W25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="X25">
         <v>5</v>
@@ -63703,7 +63703,7 @@
         <v>1038</v>
       </c>
       <c r="B26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="C26">
         <v>6</v>
@@ -63766,7 +63766,7 @@
         <v>-1</v>
       </c>
       <c r="W26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="X26">
         <v>6</v>
@@ -63807,7 +63807,7 @@
         <v>6</v>
       </c>
       <c r="G27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="H27">
         <v>8</v>
@@ -63870,7 +63870,7 @@
         <v>6</v>
       </c>
       <c r="AB27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="AC27">
         <v>8</v>
@@ -63985,7 +63985,7 @@
         <v>6</v>
       </c>
       <c r="G29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="H29">
         <v>5</v>
@@ -64048,7 +64048,7 @@
         <v>6</v>
       </c>
       <c r="AB29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AC29">
         <v>5</v>
@@ -71244,7 +71244,7 @@
         <v>6</v>
       </c>
       <c r="E6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F6">
         <v>-1</v>
@@ -71298,7 +71298,7 @@
         <v>6</v>
       </c>
       <c r="W6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X6">
         <v>-1</v>
@@ -71321,7 +71321,7 @@
         <v>7</v>
       </c>
       <c r="E7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F7">
         <v>8</v>
@@ -71375,7 +71375,7 @@
         <v>7</v>
       </c>
       <c r="W7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X7">
         <v>8</v>
@@ -71398,7 +71398,7 @@
         <v>7</v>
       </c>
       <c r="E8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F8">
         <v>8</v>
@@ -71452,7 +71452,7 @@
         <v>7</v>
       </c>
       <c r="W8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X8">
         <v>8</v>
@@ -71475,7 +71475,7 @@
         <v>-1</v>
       </c>
       <c r="E9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F9">
         <v>7</v>
@@ -71529,7 +71529,7 @@
         <v>-1</v>
       </c>
       <c r="W9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X9">
         <v>7</v>
@@ -71552,7 +71552,7 @@
         <v>-1</v>
       </c>
       <c r="E10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F10">
         <v>7</v>
@@ -71606,7 +71606,7 @@
         <v>-1</v>
       </c>
       <c r="W10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X10">
         <v>7</v>
@@ -71783,7 +71783,7 @@
         <v>6</v>
       </c>
       <c r="E13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F13">
         <v>-1</v>
@@ -71837,7 +71837,7 @@
         <v>6</v>
       </c>
       <c r="W13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X13">
         <v>-1</v>
@@ -71860,7 +71860,7 @@
         <v>-1</v>
       </c>
       <c r="E14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F14">
         <v>-1</v>
@@ -71914,7 +71914,7 @@
         <v>-1</v>
       </c>
       <c r="W14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X14">
         <v>-1</v>
@@ -71937,7 +71937,7 @@
         <v>-1</v>
       </c>
       <c r="E15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F15">
         <v>-1</v>
@@ -71991,7 +71991,7 @@
         <v>-1</v>
       </c>
       <c r="W15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X15">
         <v>-1</v>
@@ -72091,7 +72091,7 @@
         <v>-1</v>
       </c>
       <c r="E17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="F17">
         <v>-1</v>
@@ -72145,7 +72145,7 @@
         <v>-1</v>
       </c>
       <c r="W17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="X17">
         <v>-1</v>
@@ -72168,7 +72168,7 @@
         <v>6</v>
       </c>
       <c r="E18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F18">
         <v>-1</v>
@@ -72222,7 +72222,7 @@
         <v>6</v>
       </c>
       <c r="W18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X18">
         <v>-1</v>
@@ -72322,7 +72322,7 @@
         <v>-1</v>
       </c>
       <c r="E20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F20">
         <v>-1</v>
@@ -72376,7 +72376,7 @@
         <v>-1</v>
       </c>
       <c r="W20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X20">
         <v>-1</v>
@@ -72476,7 +72476,7 @@
         <v>-1</v>
       </c>
       <c r="E22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F22">
         <v>-1</v>
@@ -72530,7 +72530,7 @@
         <v>-1</v>
       </c>
       <c r="W22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X22">
         <v>-1</v>
@@ -72553,7 +72553,7 @@
         <v>-1</v>
       </c>
       <c r="E23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F23">
         <v>-1</v>
@@ -72607,7 +72607,7 @@
         <v>-1</v>
       </c>
       <c r="W23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X23">
         <v>-1</v>
@@ -72630,7 +72630,7 @@
         <v>-1</v>
       </c>
       <c r="E24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F24">
         <v>-1</v>
@@ -72684,7 +72684,7 @@
         <v>-1</v>
       </c>
       <c r="W24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X24">
         <v>-1</v>
@@ -72707,7 +72707,7 @@
         <v>-1</v>
       </c>
       <c r="E25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F25">
         <v>-1</v>
@@ -72761,7 +72761,7 @@
         <v>-1</v>
       </c>
       <c r="W25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X25">
         <v>-1</v>
@@ -72784,7 +72784,7 @@
         <v>-1</v>
       </c>
       <c r="E26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="F26">
         <v>-1</v>
@@ -72838,7 +72838,7 @@
         <v>-1</v>
       </c>
       <c r="W26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="X26">
         <v>-1</v>
@@ -72902,7 +72902,7 @@
         <v>6</v>
       </c>
       <c r="E28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F28">
         <v>-1</v>
@@ -72956,7 +72956,7 @@
         <v>6</v>
       </c>
       <c r="W28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X28">
         <v>-1</v>
@@ -72979,7 +72979,7 @@
         <v>-1</v>
       </c>
       <c r="E29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F29">
         <v>-1</v>
@@ -73033,7 +73033,7 @@
         <v>-1</v>
       </c>
       <c r="W29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X29">
         <v>-1</v>
@@ -73056,7 +73056,7 @@
         <v>7</v>
       </c>
       <c r="E30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F30">
         <v>-1</v>
@@ -73110,7 +73110,7 @@
         <v>7</v>
       </c>
       <c r="W30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X30">
         <v>-1</v>
@@ -73133,7 +73133,7 @@
         <v>-1</v>
       </c>
       <c r="E31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F31">
         <v>-1</v>
@@ -73187,7 +73187,7 @@
         <v>-1</v>
       </c>
       <c r="W31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X31">
         <v>-1</v>
@@ -73210,7 +73210,7 @@
         <v>-1</v>
       </c>
       <c r="E32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F32">
         <v>-1</v>
@@ -73264,7 +73264,7 @@
         <v>-1</v>
       </c>
       <c r="W32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X32">
         <v>-1</v>
@@ -73287,7 +73287,7 @@
         <v>10</v>
       </c>
       <c r="E33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F33">
         <v>10</v>
@@ -73341,7 +73341,7 @@
         <v>10</v>
       </c>
       <c r="W33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X33">
         <v>10</v>
@@ -73364,7 +73364,7 @@
         <v>7</v>
       </c>
       <c r="E34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F34">
         <v>8</v>
@@ -73418,7 +73418,7 @@
         <v>7</v>
       </c>
       <c r="W34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X34">
         <v>8</v>
@@ -73441,7 +73441,7 @@
         <v>-1</v>
       </c>
       <c r="E35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F35">
         <v>-1</v>
@@ -73495,7 +73495,7 @@
         <v>-1</v>
       </c>
       <c r="W35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="X35">
         <v>-1</v>
@@ -73547,7 +73547,7 @@
         <v>-1</v>
       </c>
       <c r="E37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="F37">
         <v>-1</v>
@@ -73601,7 +73601,7 @@
         <v>-1</v>
       </c>
       <c r="W37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="X37">
         <v>-1</v>
@@ -73624,7 +73624,7 @@
         <v>9</v>
       </c>
       <c r="E38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="F38">
         <v>8</v>
@@ -73678,7 +73678,7 @@
         <v>9</v>
       </c>
       <c r="W38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="X38">
         <v>8</v>
@@ -74031,7 +74031,7 @@
         <v>7</v>
       </c>
       <c r="C4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D4">
         <v>8</v>
@@ -74085,7 +74085,7 @@
         <v>7</v>
       </c>
       <c r="U4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="V4">
         <v>8</v>
@@ -74339,7 +74339,7 @@
         <v>10</v>
       </c>
       <c r="C8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="D8">
         <v>9</v>
@@ -74393,7 +74393,7 @@
         <v>10</v>
       </c>
       <c r="U8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V8">
         <v>9</v>
@@ -74493,7 +74493,7 @@
         <v>10</v>
       </c>
       <c r="C10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="D10">
         <v>9</v>
@@ -74547,7 +74547,7 @@
         <v>10</v>
       </c>
       <c r="U10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V10">
         <v>9</v>
@@ -74878,7 +74878,7 @@
         <v>10</v>
       </c>
       <c r="C15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="D15">
         <v>7</v>
@@ -74932,7 +74932,7 @@
         <v>10</v>
       </c>
       <c r="U15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V15">
         <v>7</v>
@@ -79080,7 +79080,7 @@
         <v>10</v>
       </c>
       <c r="D4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E4">
         <v>6</v>
@@ -79134,7 +79134,7 @@
         <v>10</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W4">
         <v>6</v>
@@ -79311,7 +79311,7 @@
         <v>10</v>
       </c>
       <c r="D7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E7">
         <v>9</v>
@@ -79365,7 +79365,7 @@
         <v>10</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W7">
         <v>9</v>
@@ -79388,7 +79388,7 @@
         <v>8</v>
       </c>
       <c r="D8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E8">
         <v>9</v>
@@ -79442,7 +79442,7 @@
         <v>8</v>
       </c>
       <c r="V8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W8">
         <v>9</v>
@@ -79465,7 +79465,7 @@
         <v>10</v>
       </c>
       <c r="D9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E9">
         <v>6</v>
@@ -79519,7 +79519,7 @@
         <v>10</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W9">
         <v>6</v>
@@ -79773,7 +79773,7 @@
         <v>10</v>
       </c>
       <c r="D13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E13">
         <v>8</v>
@@ -79827,7 +79827,7 @@
         <v>10</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W13">
         <v>8</v>
@@ -79850,7 +79850,7 @@
         <v>10</v>
       </c>
       <c r="D14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E14">
         <v>6</v>
@@ -79904,7 +79904,7 @@
         <v>10</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W14">
         <v>6</v>
@@ -79927,7 +79927,7 @@
         <v>10</v>
       </c>
       <c r="D15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="E15">
         <v>6</v>
@@ -79981,7 +79981,7 @@
         <v>10</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W15">
         <v>6</v>
@@ -80004,7 +80004,7 @@
         <v>8</v>
       </c>
       <c r="D16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E16">
         <v>6</v>
@@ -80058,7 +80058,7 @@
         <v>8</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W16">
         <v>6</v>
@@ -80235,7 +80235,7 @@
         <v>10</v>
       </c>
       <c r="D19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E19">
         <v>8</v>
@@ -80289,7 +80289,7 @@
         <v>10</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W19">
         <v>8</v>
@@ -80697,7 +80697,7 @@
         <v>8</v>
       </c>
       <c r="D25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E25">
         <v>7</v>
@@ -80751,7 +80751,7 @@
         <v>8</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W25">
         <v>7</v>
@@ -80928,7 +80928,7 @@
         <v>10</v>
       </c>
       <c r="D28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="E28">
         <v>9</v>
@@ -80982,7 +80982,7 @@
         <v>10</v>
       </c>
       <c r="V28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W28">
         <v>9</v>
@@ -81005,7 +81005,7 @@
         <v>9</v>
       </c>
       <c r="D29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E29">
         <v>6</v>
@@ -81059,7 +81059,7 @@
         <v>9</v>
       </c>
       <c r="V29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W29">
         <v>6</v>
@@ -81159,7 +81159,7 @@
         <v>7</v>
       </c>
       <c r="D31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="E31">
         <v>6</v>
@@ -81213,7 +81213,7 @@
         <v>7</v>
       </c>
       <c r="V31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W31">
         <v>6</v>
@@ -81236,7 +81236,7 @@
         <v>10</v>
       </c>
       <c r="D32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E32">
         <v>6</v>
@@ -81290,7 +81290,7 @@
         <v>10</v>
       </c>
       <c r="V32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W32">
         <v>6</v>
@@ -81390,7 +81390,7 @@
         <v>10</v>
       </c>
       <c r="D34">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E34">
         <v>8</v>
@@ -81444,7 +81444,7 @@
         <v>10</v>
       </c>
       <c r="V34">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W34">
         <v>8</v>
@@ -81467,7 +81467,7 @@
         <v>9</v>
       </c>
       <c r="D35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E35">
         <v>6</v>
@@ -81521,7 +81521,7 @@
         <v>9</v>
       </c>
       <c r="V35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W35">
         <v>6</v>
@@ -81544,7 +81544,7 @@
         <v>5</v>
       </c>
       <c r="D36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E36">
         <v>5</v>
@@ -81598,7 +81598,7 @@
         <v>5</v>
       </c>
       <c r="V36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W36">
         <v>5</v>
@@ -81698,7 +81698,7 @@
         <v>7</v>
       </c>
       <c r="D38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="E38">
         <v>7</v>
@@ -81752,7 +81752,7 @@
         <v>7</v>
       </c>
       <c r="V38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W38">
         <v>7</v>
@@ -81775,7 +81775,7 @@
         <v>10</v>
       </c>
       <c r="D39">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E39">
         <v>8</v>
@@ -81829,7 +81829,7 @@
         <v>10</v>
       </c>
       <c r="V39">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W39">
         <v>8</v>
@@ -81929,7 +81929,7 @@
         <v>10</v>
       </c>
       <c r="D41">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="E41">
         <v>8</v>
@@ -81983,7 +81983,7 @@
         <v>10</v>
       </c>
       <c r="V41">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W41">
         <v>8</v>
@@ -82006,7 +82006,7 @@
         <v>10</v>
       </c>
       <c r="D42">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E42">
         <v>6</v>
@@ -82060,7 +82060,7 @@
         <v>10</v>
       </c>
       <c r="V42">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W42">
         <v>6</v>
@@ -82083,7 +82083,7 @@
         <v>10</v>
       </c>
       <c r="D43">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="E43">
         <v>9</v>
@@ -82137,7 +82137,7 @@
         <v>10</v>
       </c>
       <c r="V43">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W43">
         <v>9</v>

</xml_diff>

<commit_message>
Segundo Parcial 8 noviembre
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -6750,7 +6750,7 @@
         <v>10</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -6827,7 +6827,7 @@
         <v>10</v>
       </c>
       <c r="M5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N5">
         <v>-1</v>
@@ -6863,7 +6863,7 @@
         <v>10</v>
       </c>
       <c r="Y5">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -6904,7 +6904,7 @@
         <v>10</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -6981,7 +6981,7 @@
         <v>10</v>
       </c>
       <c r="M7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N7">
         <v>-1</v>
@@ -7058,7 +7058,7 @@
         <v>10</v>
       </c>
       <c r="M8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -7135,7 +7135,7 @@
         <v>10</v>
       </c>
       <c r="M9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N9">
         <v>-1</v>
@@ -7212,7 +7212,7 @@
         <v>10</v>
       </c>
       <c r="M10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N10">
         <v>-1</v>
@@ -7248,7 +7248,7 @@
         <v>10</v>
       </c>
       <c r="Y10">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -7289,7 +7289,7 @@
         <v>10</v>
       </c>
       <c r="M11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N11">
         <v>-1</v>
@@ -7366,7 +7366,7 @@
         <v>8</v>
       </c>
       <c r="M12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N12">
         <v>-1</v>
@@ -7443,7 +7443,7 @@
         <v>10</v>
       </c>
       <c r="M13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N13">
         <v>-1</v>
@@ -7520,7 +7520,7 @@
         <v>10</v>
       </c>
       <c r="M14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -7597,7 +7597,7 @@
         <v>10</v>
       </c>
       <c r="M15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N15">
         <v>-1</v>
@@ -7633,7 +7633,7 @@
         <v>10</v>
       </c>
       <c r="Y15">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:25">
@@ -7674,7 +7674,7 @@
         <v>10</v>
       </c>
       <c r="M16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N16">
         <v>-1</v>
@@ -7751,7 +7751,7 @@
         <v>8</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N17">
         <v>-1</v>
@@ -7828,7 +7828,7 @@
         <v>6</v>
       </c>
       <c r="M18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N18">
         <v>-1</v>
@@ -7864,7 +7864,7 @@
         <v>7</v>
       </c>
       <c r="Y18">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:25">
@@ -7905,7 +7905,7 @@
         <v>6</v>
       </c>
       <c r="M19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N19">
         <v>-1</v>
@@ -7941,7 +7941,7 @@
         <v>7</v>
       </c>
       <c r="Y19">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:25">
@@ -7982,7 +7982,7 @@
         <v>10</v>
       </c>
       <c r="M20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N20">
         <v>-1</v>
@@ -8059,7 +8059,7 @@
         <v>5</v>
       </c>
       <c r="M21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N21">
         <v>-1</v>
@@ -8095,7 +8095,7 @@
         <v>5</v>
       </c>
       <c r="Y21">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" spans="1:25">
@@ -8136,7 +8136,7 @@
         <v>10</v>
       </c>
       <c r="M22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N22">
         <v>-1</v>
@@ -8172,7 +8172,7 @@
         <v>9</v>
       </c>
       <c r="Y22">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23" spans="1:25">
@@ -8213,7 +8213,7 @@
         <v>5</v>
       </c>
       <c r="M23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N23">
         <v>-1</v>
@@ -8249,7 +8249,7 @@
         <v>6</v>
       </c>
       <c r="Y23">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:25">
@@ -8290,7 +8290,7 @@
         <v>6</v>
       </c>
       <c r="M24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N24">
         <v>-1</v>
@@ -8326,7 +8326,7 @@
         <v>6</v>
       </c>
       <c r="Y24">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -8367,7 +8367,7 @@
         <v>10</v>
       </c>
       <c r="M25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N25">
         <v>-1</v>
@@ -8444,7 +8444,7 @@
         <v>8</v>
       </c>
       <c r="M26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N26">
         <v>-1</v>
@@ -8521,7 +8521,7 @@
         <v>5</v>
       </c>
       <c r="M27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N27">
         <v>-1</v>
@@ -8557,7 +8557,7 @@
         <v>8</v>
       </c>
       <c r="Y27">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:25">
@@ -8598,7 +8598,7 @@
         <v>10</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -8675,7 +8675,7 @@
         <v>10</v>
       </c>
       <c r="M29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N29">
         <v>-1</v>
@@ -8752,7 +8752,7 @@
         <v>10</v>
       </c>
       <c r="M30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N30">
         <v>-1</v>
@@ -8829,7 +8829,7 @@
         <v>10</v>
       </c>
       <c r="M31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N31">
         <v>-1</v>
@@ -8906,7 +8906,7 @@
         <v>10</v>
       </c>
       <c r="M32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N32">
         <v>-1</v>
@@ -8983,7 +8983,7 @@
         <v>10</v>
       </c>
       <c r="M33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N33">
         <v>-1</v>
@@ -9060,7 +9060,7 @@
         <v>10</v>
       </c>
       <c r="M34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N34">
         <v>-1</v>
@@ -9096,7 +9096,7 @@
         <v>10</v>
       </c>
       <c r="Y34">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:25">
@@ -9137,7 +9137,7 @@
         <v>10</v>
       </c>
       <c r="M35">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N35">
         <v>-1</v>
@@ -9214,7 +9214,7 @@
         <v>10</v>
       </c>
       <c r="M36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N36">
         <v>-1</v>
@@ -9250,7 +9250,7 @@
         <v>10</v>
       </c>
       <c r="Y36">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:25">
@@ -9291,7 +9291,7 @@
         <v>10</v>
       </c>
       <c r="M37">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N37">
         <v>-1</v>
@@ -9368,7 +9368,7 @@
         <v>10</v>
       </c>
       <c r="M38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N38">
         <v>-1</v>
@@ -9445,7 +9445,7 @@
         <v>6</v>
       </c>
       <c r="M39">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N39">
         <v>-1</v>
@@ -9481,7 +9481,7 @@
         <v>5</v>
       </c>
       <c r="Y39">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:25">
@@ -9522,7 +9522,7 @@
         <v>10</v>
       </c>
       <c r="M40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N40">
         <v>-1</v>
@@ -9558,7 +9558,7 @@
         <v>10</v>
       </c>
       <c r="Y40">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:25">
@@ -9599,7 +9599,7 @@
         <v>10</v>
       </c>
       <c r="M41">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N41">
         <v>-1</v>
@@ -9635,7 +9635,7 @@
         <v>10</v>
       </c>
       <c r="Y41">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:25">
@@ -9676,7 +9676,7 @@
         <v>8</v>
       </c>
       <c r="M42">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N42">
         <v>-1</v>
@@ -9712,7 +9712,7 @@
         <v>8</v>
       </c>
       <c r="Y42">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -23614,7 +23614,7 @@
         <v>-1</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -23650,7 +23650,7 @@
         <v>7</v>
       </c>
       <c r="Y6">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -23768,7 +23768,7 @@
         <v>8</v>
       </c>
       <c r="M8">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -23804,7 +23804,7 @@
         <v>8</v>
       </c>
       <c r="Y8">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -24920,7 +24920,7 @@
         <v>9</v>
       </c>
       <c r="L23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M23">
         <v>9</v>
@@ -24956,7 +24956,7 @@
         <v>9</v>
       </c>
       <c r="X23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Y23">
         <v>10</v>
@@ -25000,7 +25000,7 @@
         <v>8</v>
       </c>
       <c r="M24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N24">
         <v>-1</v>
@@ -25036,7 +25036,7 @@
         <v>9</v>
       </c>
       <c r="Y24">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -25308,7 +25308,7 @@
         <v>8</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -25385,7 +25385,7 @@
         <v>8</v>
       </c>
       <c r="M29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N29">
         <v>-1</v>
@@ -25421,7 +25421,7 @@
         <v>8</v>
       </c>
       <c r="Y29">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:25">
@@ -26232,7 +26232,7 @@
         <v>9</v>
       </c>
       <c r="M40">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N40">
         <v>-1</v>
@@ -26268,7 +26268,7 @@
         <v>9</v>
       </c>
       <c r="Y40">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -30629,7 +30629,7 @@
         <v>8</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J23">
         <v>7</v>
@@ -30665,7 +30665,7 @@
         <v>8</v>
       </c>
       <c r="U23">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V23">
         <v>7</v>
@@ -30783,7 +30783,7 @@
         <v>8</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J25">
         <v>-1</v>
@@ -30819,7 +30819,7 @@
         <v>8</v>
       </c>
       <c r="U25">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V25">
         <v>-1</v>
@@ -31014,7 +31014,7 @@
         <v>7</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J28">
         <v>-1</v>
@@ -31050,7 +31050,7 @@
         <v>7</v>
       </c>
       <c r="U28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V28">
         <v>-1</v>
@@ -40034,7 +40034,7 @@
         <v>4</v>
       </c>
       <c r="K4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L4">
         <v>8</v>
@@ -40111,7 +40111,7 @@
         <v>7</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L5">
         <v>10</v>
@@ -40147,7 +40147,7 @@
         <v>7</v>
       </c>
       <c r="W5">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X5">
         <v>10</v>
@@ -40188,7 +40188,7 @@
         <v>9</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L6">
         <v>-1</v>
@@ -40224,7 +40224,7 @@
         <v>8</v>
       </c>
       <c r="W6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X6">
         <v>-1</v>
@@ -40265,7 +40265,7 @@
         <v>8</v>
       </c>
       <c r="K7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L7">
         <v>9</v>
@@ -40342,7 +40342,7 @@
         <v>4</v>
       </c>
       <c r="K8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L8">
         <v>-1</v>
@@ -40419,7 +40419,7 @@
         <v>4</v>
       </c>
       <c r="K9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L9">
         <v>10</v>
@@ -40455,7 +40455,7 @@
         <v>6</v>
       </c>
       <c r="W9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X9">
         <v>10</v>
@@ -40496,7 +40496,7 @@
         <v>8</v>
       </c>
       <c r="K10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L10">
         <v>10</v>
@@ -40532,7 +40532,7 @@
         <v>7</v>
       </c>
       <c r="W10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X10">
         <v>10</v>
@@ -40573,7 +40573,7 @@
         <v>6</v>
       </c>
       <c r="K11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L11">
         <v>9</v>
@@ -40609,7 +40609,7 @@
         <v>6</v>
       </c>
       <c r="W11">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X11">
         <v>9</v>
@@ -40650,7 +40650,7 @@
         <v>8</v>
       </c>
       <c r="K12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L12">
         <v>9</v>
@@ -40686,7 +40686,7 @@
         <v>8</v>
       </c>
       <c r="W12">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="X12">
         <v>9</v>
@@ -40727,7 +40727,7 @@
         <v>7</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L13">
         <v>10</v>
@@ -40763,7 +40763,7 @@
         <v>8</v>
       </c>
       <c r="W13">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X13">
         <v>10</v>
@@ -40804,7 +40804,7 @@
         <v>5</v>
       </c>
       <c r="K14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L14">
         <v>-1</v>
@@ -40881,7 +40881,7 @@
         <v>6</v>
       </c>
       <c r="K15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L15">
         <v>9</v>
@@ -40958,7 +40958,7 @@
         <v>8</v>
       </c>
       <c r="K16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L16">
         <v>9</v>
@@ -41035,7 +41035,7 @@
         <v>9</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L17">
         <v>9</v>
@@ -41071,7 +41071,7 @@
         <v>8</v>
       </c>
       <c r="W17">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="X17">
         <v>9</v>
@@ -41112,7 +41112,7 @@
         <v>6</v>
       </c>
       <c r="K18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L18">
         <v>9</v>
@@ -41148,7 +41148,7 @@
         <v>7</v>
       </c>
       <c r="W18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X18">
         <v>9</v>
@@ -41189,7 +41189,7 @@
         <v>4</v>
       </c>
       <c r="K19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L19">
         <v>8</v>
@@ -41225,7 +41225,7 @@
         <v>5</v>
       </c>
       <c r="W19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X19">
         <v>8</v>
@@ -41266,7 +41266,7 @@
         <v>9</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L20">
         <v>8</v>
@@ -41343,7 +41343,7 @@
         <v>9</v>
       </c>
       <c r="K21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L21">
         <v>10</v>
@@ -41420,7 +41420,7 @@
         <v>9</v>
       </c>
       <c r="K22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L22">
         <v>10</v>
@@ -41456,7 +41456,7 @@
         <v>8</v>
       </c>
       <c r="W22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X22">
         <v>10</v>
@@ -41497,7 +41497,7 @@
         <v>5</v>
       </c>
       <c r="K23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L23">
         <v>9</v>
@@ -41533,7 +41533,7 @@
         <v>6</v>
       </c>
       <c r="W23">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X23">
         <v>9</v>
@@ -41574,7 +41574,7 @@
         <v>7</v>
       </c>
       <c r="K24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L24">
         <v>9</v>
@@ -41610,7 +41610,7 @@
         <v>7</v>
       </c>
       <c r="W24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X24">
         <v>9</v>
@@ -41651,7 +41651,7 @@
         <v>9</v>
       </c>
       <c r="K25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L25">
         <v>10</v>
@@ -41687,7 +41687,7 @@
         <v>9</v>
       </c>
       <c r="W25">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X25">
         <v>10</v>
@@ -41728,7 +41728,7 @@
         <v>9</v>
       </c>
       <c r="K26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L26">
         <v>9</v>
@@ -41805,7 +41805,7 @@
         <v>7</v>
       </c>
       <c r="K27">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L27">
         <v>9</v>
@@ -41841,7 +41841,7 @@
         <v>8</v>
       </c>
       <c r="W27">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X27">
         <v>9</v>
@@ -41882,7 +41882,7 @@
         <v>7</v>
       </c>
       <c r="K28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L28">
         <v>9</v>
@@ -41959,7 +41959,7 @@
         <v>9</v>
       </c>
       <c r="K29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L29">
         <v>10</v>
@@ -41995,7 +41995,7 @@
         <v>9</v>
       </c>
       <c r="W29">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X29">
         <v>10</v>
@@ -42036,7 +42036,7 @@
         <v>8</v>
       </c>
       <c r="K30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L30">
         <v>9</v>
@@ -42072,7 +42072,7 @@
         <v>7</v>
       </c>
       <c r="W30">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="X30">
         <v>9</v>
@@ -42113,7 +42113,7 @@
         <v>7</v>
       </c>
       <c r="K31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L31">
         <v>10</v>
@@ -42190,7 +42190,7 @@
         <v>7</v>
       </c>
       <c r="K32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L32">
         <v>10</v>
@@ -42226,7 +42226,7 @@
         <v>7</v>
       </c>
       <c r="W32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X32">
         <v>9</v>
@@ -42267,7 +42267,7 @@
         <v>4</v>
       </c>
       <c r="K33">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L33">
         <v>-1</v>
@@ -42344,7 +42344,7 @@
         <v>7</v>
       </c>
       <c r="K34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L34">
         <v>10</v>
@@ -42421,7 +42421,7 @@
         <v>8</v>
       </c>
       <c r="K35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L35">
         <v>10</v>
@@ -42498,7 +42498,7 @@
         <v>8</v>
       </c>
       <c r="K36">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L36">
         <v>9</v>
@@ -42575,7 +42575,7 @@
         <v>7</v>
       </c>
       <c r="K37">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L37">
         <v>9</v>
@@ -42611,7 +42611,7 @@
         <v>7</v>
       </c>
       <c r="W37">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X37">
         <v>9</v>
@@ -42652,7 +42652,7 @@
         <v>6</v>
       </c>
       <c r="K38">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L38">
         <v>10</v>
@@ -42688,7 +42688,7 @@
         <v>6</v>
       </c>
       <c r="W38">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X38">
         <v>10</v>
@@ -42729,7 +42729,7 @@
         <v>9</v>
       </c>
       <c r="K39">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L39">
         <v>10</v>
@@ -42765,7 +42765,7 @@
         <v>9</v>
       </c>
       <c r="W39">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X39">
         <v>10</v>
@@ -42806,7 +42806,7 @@
         <v>4</v>
       </c>
       <c r="K40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L40">
         <v>-1</v>
@@ -42883,7 +42883,7 @@
         <v>8</v>
       </c>
       <c r="K41">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L41">
         <v>9</v>
@@ -42960,7 +42960,7 @@
         <v>8</v>
       </c>
       <c r="K42">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L42">
         <v>9</v>
@@ -42996,7 +42996,7 @@
         <v>7</v>
       </c>
       <c r="W42">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="X42">
         <v>9</v>
@@ -43037,7 +43037,7 @@
         <v>9</v>
       </c>
       <c r="K43">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L43">
         <v>9</v>
@@ -43073,7 +43073,7 @@
         <v>9</v>
       </c>
       <c r="W43">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X43">
         <v>9</v>
@@ -43114,7 +43114,7 @@
         <v>8</v>
       </c>
       <c r="K44">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L44">
         <v>10</v>
@@ -43150,7 +43150,7 @@
         <v>9</v>
       </c>
       <c r="W44">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X44">
         <v>10</v>
@@ -43404,7 +43404,7 @@
         <v>7</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L5">
         <v>8</v>
@@ -43440,7 +43440,7 @@
         <v>7</v>
       </c>
       <c r="W5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="X5">
         <v>7</v>
@@ -43481,7 +43481,7 @@
         <v>6</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L6">
         <v>7</v>
@@ -43517,7 +43517,7 @@
         <v>6</v>
       </c>
       <c r="W6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X6">
         <v>7</v>
@@ -44020,7 +44020,7 @@
         <v>4</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L13">
         <v>7</v>
@@ -44328,7 +44328,7 @@
         <v>4</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -44364,7 +44364,7 @@
         <v>5</v>
       </c>
       <c r="W17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X17">
         <v>5</v>
@@ -44636,7 +44636,7 @@
         <v>4</v>
       </c>
       <c r="K21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L21">
         <v>-1</v>
@@ -44790,7 +44790,7 @@
         <v>7</v>
       </c>
       <c r="K23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L23">
         <v>10</v>
@@ -45560,7 +45560,7 @@
         <v>6</v>
       </c>
       <c r="K33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L33">
         <v>7</v>
@@ -45868,7 +45868,7 @@
         <v>7</v>
       </c>
       <c r="K37">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L37">
         <v>5</v>
@@ -70951,7 +70951,7 @@
         <v>-1</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -70987,7 +70987,7 @@
         <v>-1</v>
       </c>
       <c r="Y6">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -71721,7 +71721,7 @@
         <v>-1</v>
       </c>
       <c r="M16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N16">
         <v>-1</v>
@@ -71757,7 +71757,7 @@
         <v>-1</v>
       </c>
       <c r="Y16">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:25">
@@ -71798,7 +71798,7 @@
         <v>-1</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="N17">
         <v>-1</v>
@@ -71834,7 +71834,7 @@
         <v>-1</v>
       </c>
       <c r="Y17">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:25">
@@ -72106,7 +72106,7 @@
         <v>-1</v>
       </c>
       <c r="M21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N21">
         <v>-1</v>
@@ -72142,7 +72142,7 @@
         <v>-1</v>
       </c>
       <c r="Y21">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:25">
@@ -72337,7 +72337,7 @@
         <v>-1</v>
       </c>
       <c r="M24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N24">
         <v>-1</v>
@@ -72491,7 +72491,7 @@
         <v>-1</v>
       </c>
       <c r="M26">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="N26">
         <v>-1</v>
@@ -72527,7 +72527,7 @@
         <v>-1</v>
       </c>
       <c r="Y26">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:25">
@@ -73148,7 +73148,7 @@
         <v>-1</v>
       </c>
       <c r="M35">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="N35">
         <v>-1</v>
@@ -73184,7 +73184,7 @@
         <v>-1</v>
       </c>
       <c r="Y35">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:25">
@@ -73254,7 +73254,7 @@
         <v>-1</v>
       </c>
       <c r="M37">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N37">
         <v>-1</v>
@@ -73290,7 +73290,7 @@
         <v>-1</v>
       </c>
       <c r="Y37">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38" spans="1:25">
@@ -73408,7 +73408,7 @@
         <v>-1</v>
       </c>
       <c r="M39">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N39">
         <v>-1</v>
@@ -73461,7 +73461,7 @@
         <v>-1</v>
       </c>
       <c r="M40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="R40">
         <v>-1</v>
@@ -73473,7 +73473,7 @@
         <v>8</v>
       </c>
       <c r="Y40">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41" spans="1:25">
@@ -73555,7 +73555,7 @@
         <v>-1</v>
       </c>
       <c r="M42">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="R42">
         <v>-1</v>
@@ -85684,7 +85684,7 @@
         <v>9</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -85761,7 +85761,7 @@
         <v>9</v>
       </c>
       <c r="M5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N5">
         <v>-1</v>
@@ -85838,7 +85838,7 @@
         <v>7</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -85874,7 +85874,7 @@
         <v>8</v>
       </c>
       <c r="Y6">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -85915,7 +85915,7 @@
         <v>8</v>
       </c>
       <c r="M7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N7">
         <v>-1</v>
@@ -85951,7 +85951,7 @@
         <v>7</v>
       </c>
       <c r="Y7">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -85992,7 +85992,7 @@
         <v>9</v>
       </c>
       <c r="M8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -86028,7 +86028,7 @@
         <v>9</v>
       </c>
       <c r="Y8">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -86069,7 +86069,7 @@
         <v>5</v>
       </c>
       <c r="M9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N9">
         <v>-1</v>
@@ -86146,7 +86146,7 @@
         <v>7</v>
       </c>
       <c r="M10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N10">
         <v>-1</v>
@@ -86182,7 +86182,7 @@
         <v>7</v>
       </c>
       <c r="Y10">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -86223,7 +86223,7 @@
         <v>9</v>
       </c>
       <c r="M11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N11">
         <v>-1</v>
@@ -86300,7 +86300,7 @@
         <v>5</v>
       </c>
       <c r="M12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N12">
         <v>-1</v>
@@ -86336,7 +86336,7 @@
         <v>5</v>
       </c>
       <c r="Y12">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -86377,7 +86377,7 @@
         <v>9</v>
       </c>
       <c r="M13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N13">
         <v>-1</v>
@@ -86454,7 +86454,7 @@
         <v>9</v>
       </c>
       <c r="M14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -86531,7 +86531,7 @@
         <v>9</v>
       </c>
       <c r="M15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N15">
         <v>-1</v>
@@ -86567,7 +86567,7 @@
         <v>7</v>
       </c>
       <c r="Y15">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:25">
@@ -86608,7 +86608,7 @@
         <v>8</v>
       </c>
       <c r="M16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N16">
         <v>-1</v>
@@ -86685,7 +86685,7 @@
         <v>5</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N17">
         <v>-1</v>
@@ -86762,7 +86762,7 @@
         <v>7</v>
       </c>
       <c r="M18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N18">
         <v>-1</v>
@@ -86798,7 +86798,7 @@
         <v>6</v>
       </c>
       <c r="Y18">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:25">
@@ -86839,7 +86839,7 @@
         <v>5</v>
       </c>
       <c r="M19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N19">
         <v>-1</v>
@@ -86916,7 +86916,7 @@
         <v>9</v>
       </c>
       <c r="M20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N20">
         <v>-1</v>
@@ -86952,7 +86952,7 @@
         <v>8</v>
       </c>
       <c r="Y20">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:25">
@@ -86993,7 +86993,7 @@
         <v>5</v>
       </c>
       <c r="M21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N21">
         <v>-1</v>
@@ -87029,7 +87029,7 @@
         <v>5</v>
       </c>
       <c r="Y21">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:25">
@@ -87070,7 +87070,7 @@
         <v>5</v>
       </c>
       <c r="M22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N22">
         <v>-1</v>
@@ -87147,7 +87147,7 @@
         <v>9</v>
       </c>
       <c r="M23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N23">
         <v>-1</v>
@@ -87183,7 +87183,7 @@
         <v>8</v>
       </c>
       <c r="Y23">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:25">
@@ -87224,7 +87224,7 @@
         <v>5</v>
       </c>
       <c r="M24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N24">
         <v>-1</v>
@@ -87260,7 +87260,7 @@
         <v>6</v>
       </c>
       <c r="Y24">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -87301,7 +87301,7 @@
         <v>8</v>
       </c>
       <c r="M25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N25">
         <v>-1</v>
@@ -87378,7 +87378,7 @@
         <v>9</v>
       </c>
       <c r="M26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N26">
         <v>-1</v>
@@ -87455,7 +87455,7 @@
         <v>7</v>
       </c>
       <c r="M27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N27">
         <v>-1</v>
@@ -87532,7 +87532,7 @@
         <v>9</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -87568,7 +87568,7 @@
         <v>8</v>
       </c>
       <c r="Y28">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -87609,7 +87609,7 @@
         <v>9</v>
       </c>
       <c r="M29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N29">
         <v>-1</v>
@@ -87686,7 +87686,7 @@
         <v>9</v>
       </c>
       <c r="M30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N30">
         <v>-1</v>
@@ -87763,7 +87763,7 @@
         <v>8</v>
       </c>
       <c r="M31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N31">
         <v>-1</v>
@@ -87840,7 +87840,7 @@
         <v>9</v>
       </c>
       <c r="M32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N32">
         <v>-1</v>
@@ -87876,7 +87876,7 @@
         <v>9</v>
       </c>
       <c r="Y32">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:25">
@@ -87917,7 +87917,7 @@
         <v>7</v>
       </c>
       <c r="M33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N33">
         <v>-1</v>
@@ -87953,7 +87953,7 @@
         <v>7</v>
       </c>
       <c r="Y33">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="34" spans="1:25">
@@ -87994,7 +87994,7 @@
         <v>9</v>
       </c>
       <c r="M34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N34">
         <v>-1</v>
@@ -88071,7 +88071,7 @@
         <v>8</v>
       </c>
       <c r="M35">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N35">
         <v>-1</v>
@@ -88107,7 +88107,7 @@
         <v>8</v>
       </c>
       <c r="Y35">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -88284,7 +88284,7 @@
         <v>7</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -88361,7 +88361,7 @@
         <v>9</v>
       </c>
       <c r="M5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N5">
         <v>-1</v>
@@ -88438,7 +88438,7 @@
         <v>8</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -88515,7 +88515,7 @@
         <v>10</v>
       </c>
       <c r="M7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N7">
         <v>-1</v>
@@ -88592,7 +88592,7 @@
         <v>9</v>
       </c>
       <c r="M8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -88669,7 +88669,7 @@
         <v>5</v>
       </c>
       <c r="M9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N9">
         <v>-1</v>
@@ -88705,7 +88705,7 @@
         <v>5</v>
       </c>
       <c r="Y9">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -88746,7 +88746,7 @@
         <v>8</v>
       </c>
       <c r="M10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N10">
         <v>-1</v>
@@ -88823,7 +88823,7 @@
         <v>8</v>
       </c>
       <c r="M11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N11">
         <v>-1</v>
@@ -88859,7 +88859,7 @@
         <v>8</v>
       </c>
       <c r="Y11">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -88900,7 +88900,7 @@
         <v>8</v>
       </c>
       <c r="M12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N12">
         <v>-1</v>
@@ -88977,7 +88977,7 @@
         <v>10</v>
       </c>
       <c r="M13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N13">
         <v>-1</v>
@@ -89054,7 +89054,7 @@
         <v>8</v>
       </c>
       <c r="M14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -89131,7 +89131,7 @@
         <v>5</v>
       </c>
       <c r="M15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N15">
         <v>-1</v>
@@ -89167,7 +89167,7 @@
         <v>5</v>
       </c>
       <c r="Y15">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:25">
@@ -89208,7 +89208,7 @@
         <v>8</v>
       </c>
       <c r="M16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N16">
         <v>-1</v>
@@ -89285,7 +89285,7 @@
         <v>9</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N17">
         <v>-1</v>
@@ -89362,7 +89362,7 @@
         <v>10</v>
       </c>
       <c r="M18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N18">
         <v>-1</v>
@@ -89439,7 +89439,7 @@
         <v>7</v>
       </c>
       <c r="M19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N19">
         <v>-1</v>
@@ -89475,7 +89475,7 @@
         <v>8</v>
       </c>
       <c r="Y19">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:25">
@@ -89516,7 +89516,7 @@
         <v>8</v>
       </c>
       <c r="M20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N20">
         <v>-1</v>
@@ -89593,7 +89593,7 @@
         <v>9</v>
       </c>
       <c r="M21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N21">
         <v>-1</v>
@@ -89670,7 +89670,7 @@
         <v>10</v>
       </c>
       <c r="M22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N22">
         <v>-1</v>
@@ -89747,7 +89747,7 @@
         <v>10</v>
       </c>
       <c r="M23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N23">
         <v>-1</v>
@@ -89824,7 +89824,7 @@
         <v>9</v>
       </c>
       <c r="M24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N24">
         <v>-1</v>
@@ -89860,7 +89860,7 @@
         <v>8</v>
       </c>
       <c r="Y24">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -89901,7 +89901,7 @@
         <v>10</v>
       </c>
       <c r="M25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N25">
         <v>-1</v>
@@ -89978,7 +89978,7 @@
         <v>10</v>
       </c>
       <c r="M26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N26">
         <v>-1</v>
@@ -90014,7 +90014,7 @@
         <v>10</v>
       </c>
       <c r="Y26">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:25">
@@ -90055,7 +90055,7 @@
         <v>8</v>
       </c>
       <c r="M27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N27">
         <v>-1</v>
@@ -90091,7 +90091,7 @@
         <v>9</v>
       </c>
       <c r="Y27">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28" spans="1:25">
@@ -90132,7 +90132,7 @@
         <v>8</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -90168,7 +90168,7 @@
         <v>9</v>
       </c>
       <c r="Y28">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -90209,7 +90209,7 @@
         <v>10</v>
       </c>
       <c r="M29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N29">
         <v>-1</v>
@@ -90245,7 +90245,7 @@
         <v>10</v>
       </c>
       <c r="Y29">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:25">
@@ -90286,7 +90286,7 @@
         <v>8</v>
       </c>
       <c r="M30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N30">
         <v>-1</v>
@@ -90322,7 +90322,7 @@
         <v>9</v>
       </c>
       <c r="Y30">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:25">
@@ -90363,7 +90363,7 @@
         <v>8</v>
       </c>
       <c r="M31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N31">
         <v>-1</v>
@@ -90440,7 +90440,7 @@
         <v>10</v>
       </c>
       <c r="M32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N32">
         <v>-1</v>
@@ -90476,7 +90476,7 @@
         <v>10</v>
       </c>
       <c r="Y32">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33" spans="1:25">
@@ -90517,7 +90517,7 @@
         <v>10</v>
       </c>
       <c r="M33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N33">
         <v>-1</v>
@@ -90594,7 +90594,7 @@
         <v>10</v>
       </c>
       <c r="M34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N34">
         <v>-1</v>
@@ -90671,7 +90671,7 @@
         <v>9</v>
       </c>
       <c r="M35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N35">
         <v>-1</v>
@@ -90748,7 +90748,7 @@
         <v>8</v>
       </c>
       <c r="M36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N36">
         <v>-1</v>
@@ -90825,7 +90825,7 @@
         <v>7</v>
       </c>
       <c r="M37">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N37">
         <v>-1</v>
@@ -90902,7 +90902,7 @@
         <v>7</v>
       </c>
       <c r="M38">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N38">
         <v>-1</v>
@@ -90979,7 +90979,7 @@
         <v>7</v>
       </c>
       <c r="M39">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N39">
         <v>-1</v>
@@ -91015,7 +91015,7 @@
         <v>6</v>
       </c>
       <c r="Y39">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:25">
@@ -91056,7 +91056,7 @@
         <v>7</v>
       </c>
       <c r="M40">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N40">
         <v>-1</v>
@@ -91133,7 +91133,7 @@
         <v>8</v>
       </c>
       <c r="M41">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N41">
         <v>-1</v>
@@ -91169,7 +91169,7 @@
         <v>8</v>
       </c>
       <c r="Y41">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:25">
@@ -91210,7 +91210,7 @@
         <v>9</v>
       </c>
       <c r="M42">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N42">
         <v>-1</v>
@@ -91287,7 +91287,7 @@
         <v>7</v>
       </c>
       <c r="M43">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N43">
         <v>-1</v>
@@ -91323,7 +91323,7 @@
         <v>7</v>
       </c>
       <c r="Y43">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Segundo Parcial 8 noviembre noche
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -2154,7 +2154,7 @@
     <t>TZOMPOLE COLOHUA JOSE LEONARDO</t>
   </si>
   <si>
-    <t>VAZQUEZ COLOHUA NAHUM HIRAM</t>
+    <t>VASQUEZ COLOHUA NAHUM HIRAM</t>
   </si>
   <si>
     <t>VERA GONZALEZ ISRAEL</t>
@@ -3996,7 +3996,7 @@
         <v>10</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -4073,7 +4073,7 @@
         <v>6</v>
       </c>
       <c r="M5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N5">
         <v>-1</v>
@@ -4150,7 +4150,7 @@
         <v>6</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -4227,7 +4227,7 @@
         <v>10</v>
       </c>
       <c r="M7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N7">
         <v>-1</v>
@@ -4263,7 +4263,7 @@
         <v>10</v>
       </c>
       <c r="Y7">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -4304,7 +4304,7 @@
         <v>7</v>
       </c>
       <c r="M8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -4381,7 +4381,7 @@
         <v>6</v>
       </c>
       <c r="M9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N9">
         <v>-1</v>
@@ -4458,7 +4458,7 @@
         <v>6</v>
       </c>
       <c r="M10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N10">
         <v>-1</v>
@@ -4494,7 +4494,7 @@
         <v>5</v>
       </c>
       <c r="Y10">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -4535,7 +4535,7 @@
         <v>6</v>
       </c>
       <c r="M11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N11">
         <v>-1</v>
@@ -4612,7 +4612,7 @@
         <v>7</v>
       </c>
       <c r="M12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N12">
         <v>-1</v>
@@ -4648,7 +4648,7 @@
         <v>7</v>
       </c>
       <c r="Y12">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -4689,7 +4689,7 @@
         <v>-1</v>
       </c>
       <c r="M13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N13">
         <v>-1</v>
@@ -4766,7 +4766,7 @@
         <v>7</v>
       </c>
       <c r="M14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -4843,7 +4843,7 @@
         <v>7</v>
       </c>
       <c r="M15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N15">
         <v>-1</v>
@@ -4920,7 +4920,7 @@
         <v>6</v>
       </c>
       <c r="M16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N16">
         <v>-1</v>
@@ -4997,7 +4997,7 @@
         <v>7</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N17">
         <v>-1</v>
@@ -5074,7 +5074,7 @@
         <v>6</v>
       </c>
       <c r="M18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N18">
         <v>-1</v>
@@ -5151,7 +5151,7 @@
         <v>9</v>
       </c>
       <c r="M19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N19">
         <v>-1</v>
@@ -5187,7 +5187,7 @@
         <v>9</v>
       </c>
       <c r="Y19">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:25">
@@ -5228,7 +5228,7 @@
         <v>-1</v>
       </c>
       <c r="M20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N20">
         <v>-1</v>
@@ -5264,7 +5264,7 @@
         <v>6</v>
       </c>
       <c r="Y20">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:25">
@@ -5305,7 +5305,7 @@
         <v>6</v>
       </c>
       <c r="M21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N21">
         <v>-1</v>
@@ -5382,7 +5382,7 @@
         <v>-1</v>
       </c>
       <c r="M22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N22">
         <v>-1</v>
@@ -5459,7 +5459,7 @@
         <v>6</v>
       </c>
       <c r="M23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N23">
         <v>-1</v>
@@ -5536,7 +5536,7 @@
         <v>6</v>
       </c>
       <c r="M24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N24">
         <v>-1</v>
@@ -5572,7 +5572,7 @@
         <v>5</v>
       </c>
       <c r="Y24">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -5613,7 +5613,7 @@
         <v>10</v>
       </c>
       <c r="M25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N25">
         <v>-1</v>
@@ -5649,7 +5649,7 @@
         <v>10</v>
       </c>
       <c r="Y25">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:25">
@@ -5690,7 +5690,7 @@
         <v>6</v>
       </c>
       <c r="M26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N26">
         <v>-1</v>
@@ -5726,7 +5726,7 @@
         <v>5</v>
       </c>
       <c r="Y26">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:25">
@@ -5767,7 +5767,7 @@
         <v>6</v>
       </c>
       <c r="M27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N27">
         <v>-1</v>
@@ -5844,7 +5844,7 @@
         <v>6</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -5880,7 +5880,7 @@
         <v>5</v>
       </c>
       <c r="Y28">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -5921,7 +5921,7 @@
         <v>7</v>
       </c>
       <c r="M29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N29">
         <v>-1</v>
@@ -5957,7 +5957,7 @@
         <v>8</v>
       </c>
       <c r="Y29">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="30" spans="1:25">
@@ -5998,7 +5998,7 @@
         <v>7</v>
       </c>
       <c r="M30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N30">
         <v>-1</v>
@@ -6034,7 +6034,7 @@
         <v>8</v>
       </c>
       <c r="Y30">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:25">
@@ -6075,7 +6075,7 @@
         <v>8</v>
       </c>
       <c r="M31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N31">
         <v>-1</v>
@@ -6152,7 +6152,7 @@
         <v>9</v>
       </c>
       <c r="M32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N32">
         <v>-1</v>
@@ -6188,7 +6188,7 @@
         <v>8</v>
       </c>
       <c r="Y32">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:25">
@@ -6229,7 +6229,7 @@
         <v>9</v>
       </c>
       <c r="M33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N33">
         <v>-1</v>
@@ -6265,7 +6265,7 @@
         <v>8</v>
       </c>
       <c r="Y33">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:25">
@@ -6306,7 +6306,7 @@
         <v>10</v>
       </c>
       <c r="M34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N34">
         <v>-1</v>
@@ -6383,7 +6383,7 @@
         <v>8</v>
       </c>
       <c r="M35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N35">
         <v>-1</v>
@@ -6460,7 +6460,7 @@
         <v>-1</v>
       </c>
       <c r="M36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N36">
         <v>-1</v>
@@ -6496,7 +6496,7 @@
         <v>5</v>
       </c>
       <c r="Y36">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:25">
@@ -6537,7 +6537,7 @@
         <v>6</v>
       </c>
       <c r="M37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N37">
         <v>-1</v>
@@ -6573,7 +6573,7 @@
         <v>6</v>
       </c>
       <c r="Y37">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -9889,7 +9889,7 @@
         <v>10</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -9966,7 +9966,7 @@
         <v>10</v>
       </c>
       <c r="M5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N5">
         <v>-1</v>
@@ -10043,7 +10043,7 @@
         <v>10</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -10120,7 +10120,7 @@
         <v>10</v>
       </c>
       <c r="M7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N7">
         <v>-1</v>
@@ -10156,7 +10156,7 @@
         <v>10</v>
       </c>
       <c r="Y7">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -10197,7 +10197,7 @@
         <v>9</v>
       </c>
       <c r="M8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -10274,7 +10274,7 @@
         <v>10</v>
       </c>
       <c r="M9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N9">
         <v>-1</v>
@@ -10351,7 +10351,7 @@
         <v>10</v>
       </c>
       <c r="M10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N10">
         <v>-1</v>
@@ -10428,7 +10428,7 @@
         <v>10</v>
       </c>
       <c r="M11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N11">
         <v>-1</v>
@@ -10505,7 +10505,7 @@
         <v>5</v>
       </c>
       <c r="M12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N12">
         <v>-1</v>
@@ -10582,7 +10582,7 @@
         <v>10</v>
       </c>
       <c r="M13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N13">
         <v>-1</v>
@@ -10659,7 +10659,7 @@
         <v>10</v>
       </c>
       <c r="M14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -10736,7 +10736,7 @@
         <v>10</v>
       </c>
       <c r="M15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N15">
         <v>-1</v>
@@ -10813,7 +10813,7 @@
         <v>10</v>
       </c>
       <c r="M16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N16">
         <v>-1</v>
@@ -10890,7 +10890,7 @@
         <v>8</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N17">
         <v>-1</v>
@@ -10926,7 +10926,7 @@
         <v>9</v>
       </c>
       <c r="Y17">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:25">
@@ -10967,7 +10967,7 @@
         <v>5</v>
       </c>
       <c r="M18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N18">
         <v>-1</v>
@@ -11044,7 +11044,7 @@
         <v>10</v>
       </c>
       <c r="M19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N19">
         <v>-1</v>
@@ -11121,7 +11121,7 @@
         <v>5</v>
       </c>
       <c r="M20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N20">
         <v>-1</v>
@@ -11198,7 +11198,7 @@
         <v>10</v>
       </c>
       <c r="M21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N21">
         <v>-1</v>
@@ -11234,7 +11234,7 @@
         <v>9</v>
       </c>
       <c r="Y21">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:25">
@@ -11275,7 +11275,7 @@
         <v>8</v>
       </c>
       <c r="M22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N22">
         <v>-1</v>
@@ -11311,7 +11311,7 @@
         <v>8</v>
       </c>
       <c r="Y22">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" spans="1:25">
@@ -11352,7 +11352,7 @@
         <v>10</v>
       </c>
       <c r="M23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N23">
         <v>-1</v>
@@ -11388,7 +11388,7 @@
         <v>9</v>
       </c>
       <c r="Y23">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:25">
@@ -11429,7 +11429,7 @@
         <v>10</v>
       </c>
       <c r="M24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N24">
         <v>-1</v>
@@ -11506,7 +11506,7 @@
         <v>10</v>
       </c>
       <c r="M25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N25">
         <v>-1</v>
@@ -11583,7 +11583,7 @@
         <v>7</v>
       </c>
       <c r="M26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N26">
         <v>-1</v>
@@ -11660,7 +11660,7 @@
         <v>10</v>
       </c>
       <c r="M27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N27">
         <v>-1</v>
@@ -11737,7 +11737,7 @@
         <v>10</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -11814,7 +11814,7 @@
         <v>10</v>
       </c>
       <c r="M29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N29">
         <v>-1</v>
@@ -11891,7 +11891,7 @@
         <v>10</v>
       </c>
       <c r="M30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N30">
         <v>-1</v>
@@ -11968,7 +11968,7 @@
         <v>10</v>
       </c>
       <c r="M31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N31">
         <v>-1</v>
@@ -12045,7 +12045,7 @@
         <v>10</v>
       </c>
       <c r="M32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N32">
         <v>-1</v>
@@ -12122,7 +12122,7 @@
         <v>8</v>
       </c>
       <c r="M33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N33">
         <v>-1</v>
@@ -12199,7 +12199,7 @@
         <v>10</v>
       </c>
       <c r="M34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N34">
         <v>-1</v>
@@ -12235,7 +12235,7 @@
         <v>10</v>
       </c>
       <c r="Y34">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -12400,7 +12400,7 @@
         <v>9</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J4">
         <v>8</v>
@@ -12477,7 +12477,7 @@
         <v>9</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J5">
         <v>6</v>
@@ -12513,7 +12513,7 @@
         <v>9</v>
       </c>
       <c r="U5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V5">
         <v>7</v>
@@ -12554,7 +12554,7 @@
         <v>9</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J6">
         <v>7</v>
@@ -12631,7 +12631,7 @@
         <v>9</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J7">
         <v>7</v>
@@ -12667,7 +12667,7 @@
         <v>9</v>
       </c>
       <c r="U7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V7">
         <v>8</v>
@@ -12708,7 +12708,7 @@
         <v>9</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J8">
         <v>7</v>
@@ -12744,7 +12744,7 @@
         <v>9</v>
       </c>
       <c r="U8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V8">
         <v>9</v>
@@ -12785,7 +12785,7 @@
         <v>9</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J9">
         <v>8</v>
@@ -12862,7 +12862,7 @@
         <v>5</v>
       </c>
       <c r="I10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J10">
         <v>5</v>
@@ -12939,7 +12939,7 @@
         <v>10</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J11">
         <v>7</v>
@@ -13016,7 +13016,7 @@
         <v>6</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J12">
         <v>7</v>
@@ -13093,7 +13093,7 @@
         <v>6</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J13">
         <v>7</v>
@@ -13129,7 +13129,7 @@
         <v>8</v>
       </c>
       <c r="U13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V13">
         <v>7</v>
@@ -13170,7 +13170,7 @@
         <v>10</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J14">
         <v>8</v>
@@ -13247,7 +13247,7 @@
         <v>10</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J15">
         <v>7</v>
@@ -13324,7 +13324,7 @@
         <v>7</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J16">
         <v>6</v>
@@ -13360,7 +13360,7 @@
         <v>7</v>
       </c>
       <c r="U16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V16">
         <v>7</v>
@@ -13401,7 +13401,7 @@
         <v>9</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J17">
         <v>7</v>
@@ -13437,7 +13437,7 @@
         <v>10</v>
       </c>
       <c r="U17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V17">
         <v>8</v>
@@ -13478,7 +13478,7 @@
         <v>10</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J18">
         <v>8</v>
@@ -13514,7 +13514,7 @@
         <v>10</v>
       </c>
       <c r="U18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V18">
         <v>8</v>
@@ -13555,7 +13555,7 @@
         <v>8</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J19">
         <v>5</v>
@@ -13591,7 +13591,7 @@
         <v>9</v>
       </c>
       <c r="U19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V19">
         <v>5</v>
@@ -13632,7 +13632,7 @@
         <v>7</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J20">
         <v>7</v>
@@ -13709,7 +13709,7 @@
         <v>7</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J21">
         <v>6</v>
@@ -13786,7 +13786,7 @@
         <v>9</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J22">
         <v>5</v>
@@ -13822,7 +13822,7 @@
         <v>9</v>
       </c>
       <c r="U22">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V22">
         <v>5</v>
@@ -13863,7 +13863,7 @@
         <v>7</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J23">
         <v>8</v>
@@ -13940,7 +13940,7 @@
         <v>10</v>
       </c>
       <c r="I24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J24">
         <v>8</v>
@@ -13976,7 +13976,7 @@
         <v>10</v>
       </c>
       <c r="U24">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V24">
         <v>8</v>
@@ -14017,7 +14017,7 @@
         <v>9</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J25">
         <v>6</v>
@@ -14094,7 +14094,7 @@
         <v>8</v>
       </c>
       <c r="I26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J26">
         <v>7</v>
@@ -14130,7 +14130,7 @@
         <v>9</v>
       </c>
       <c r="U26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V26">
         <v>8</v>
@@ -14200,7 +14200,7 @@
         <v>5</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J28">
         <v>5</v>
@@ -14212,7 +14212,7 @@
         <v>10</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -14236,7 +14236,7 @@
         <v>7</v>
       </c>
       <c r="U28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V28">
         <v>5</v>
@@ -14248,7 +14248,7 @@
         <v>10</v>
       </c>
       <c r="Y28">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -14277,7 +14277,7 @@
         <v>8</v>
       </c>
       <c r="I29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J29">
         <v>-1</v>
@@ -14313,7 +14313,7 @@
         <v>7</v>
       </c>
       <c r="U29">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V29">
         <v>-1</v>
@@ -14354,7 +14354,7 @@
         <v>8</v>
       </c>
       <c r="I30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J30">
         <v>5</v>
@@ -14431,7 +14431,7 @@
         <v>9</v>
       </c>
       <c r="I31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J31">
         <v>8</v>
@@ -14467,7 +14467,7 @@
         <v>10</v>
       </c>
       <c r="U31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V31">
         <v>9</v>
@@ -14508,7 +14508,7 @@
         <v>10</v>
       </c>
       <c r="I32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J32">
         <v>8</v>
@@ -14544,7 +14544,7 @@
         <v>10</v>
       </c>
       <c r="U32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V32">
         <v>7</v>
@@ -14585,7 +14585,7 @@
         <v>8</v>
       </c>
       <c r="I33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J33">
         <v>6</v>
@@ -14621,7 +14621,7 @@
         <v>9</v>
       </c>
       <c r="U33">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V33">
         <v>6</v>
@@ -14662,7 +14662,7 @@
         <v>8</v>
       </c>
       <c r="I34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J34">
         <v>6</v>
@@ -14739,7 +14739,7 @@
         <v>10</v>
       </c>
       <c r="I35">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J35">
         <v>8</v>
@@ -14775,7 +14775,7 @@
         <v>10</v>
       </c>
       <c r="U35">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V35">
         <v>8</v>
@@ -14816,7 +14816,7 @@
         <v>8</v>
       </c>
       <c r="I36">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J36">
         <v>7</v>
@@ -14893,7 +14893,7 @@
         <v>10</v>
       </c>
       <c r="I37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J37">
         <v>7</v>
@@ -14929,7 +14929,7 @@
         <v>10</v>
       </c>
       <c r="U37">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V37">
         <v>8</v>
@@ -14970,7 +14970,7 @@
         <v>10</v>
       </c>
       <c r="I38">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J38">
         <v>8</v>
@@ -15006,7 +15006,7 @@
         <v>10</v>
       </c>
       <c r="U38">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V38">
         <v>9</v>
@@ -15047,7 +15047,7 @@
         <v>8</v>
       </c>
       <c r="I39">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J39">
         <v>6</v>
@@ -15124,7 +15124,7 @@
         <v>10</v>
       </c>
       <c r="I40">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J40">
         <v>7</v>
@@ -15160,7 +15160,7 @@
         <v>10</v>
       </c>
       <c r="U40">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V40">
         <v>8</v>
@@ -15201,7 +15201,7 @@
         <v>10</v>
       </c>
       <c r="I41">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J41">
         <v>8</v>
@@ -15237,7 +15237,7 @@
         <v>10</v>
       </c>
       <c r="U41">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V41">
         <v>8</v>
@@ -15278,7 +15278,7 @@
         <v>6</v>
       </c>
       <c r="I42">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J42">
         <v>6</v>
@@ -15355,7 +15355,7 @@
         <v>7</v>
       </c>
       <c r="I43">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J43">
         <v>6</v>
@@ -15391,7 +15391,7 @@
         <v>8</v>
       </c>
       <c r="U43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V43">
         <v>7</v>
@@ -15432,7 +15432,7 @@
         <v>10</v>
       </c>
       <c r="I44">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J44">
         <v>8</v>
@@ -15509,7 +15509,7 @@
         <v>10</v>
       </c>
       <c r="I45">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J45">
         <v>7</v>
@@ -15586,7 +15586,7 @@
         <v>9</v>
       </c>
       <c r="I46">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J46">
         <v>5</v>
@@ -15663,7 +15663,7 @@
         <v>9</v>
       </c>
       <c r="I47">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J47">
         <v>7</v>
@@ -15740,7 +15740,7 @@
         <v>9</v>
       </c>
       <c r="I48">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J48">
         <v>7</v>
@@ -19711,7 +19711,7 @@
         <v>10</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J15">
         <v>6</v>
@@ -19747,7 +19747,7 @@
         <v>10</v>
       </c>
       <c r="U15">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V15">
         <v>5</v>
@@ -32613,7 +32613,7 @@
         <v>9</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J15">
         <v>7</v>
@@ -33152,7 +33152,7 @@
         <v>6</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J22">
         <v>4</v>
@@ -33188,7 +33188,7 @@
         <v>8</v>
       </c>
       <c r="U22">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="V22">
         <v>5</v>
@@ -33229,7 +33229,7 @@
         <v>9</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J23">
         <v>9</v>
@@ -33768,7 +33768,7 @@
         <v>7</v>
       </c>
       <c r="I30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J30">
         <v>5</v>
@@ -33804,7 +33804,7 @@
         <v>8</v>
       </c>
       <c r="U30">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="V30">
         <v>5</v>
@@ -33845,7 +33845,7 @@
         <v>5</v>
       </c>
       <c r="I31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J31">
         <v>6</v>
@@ -33881,7 +33881,7 @@
         <v>6</v>
       </c>
       <c r="U31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V31">
         <v>6</v>
@@ -40336,7 +40336,7 @@
         <v>-1</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J8">
         <v>4</v>
@@ -40372,7 +40372,7 @@
         <v>6</v>
       </c>
       <c r="U8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V8">
         <v>6</v>
@@ -41722,7 +41722,7 @@
         <v>-1</v>
       </c>
       <c r="I26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J26">
         <v>9</v>
@@ -41758,7 +41758,7 @@
         <v>7</v>
       </c>
       <c r="U26">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V26">
         <v>8</v>
@@ -41953,7 +41953,7 @@
         <v>-1</v>
       </c>
       <c r="I29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J29">
         <v>9</v>
@@ -41989,7 +41989,7 @@
         <v>7</v>
       </c>
       <c r="U29">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V29">
         <v>9</v>
@@ -43333,7 +43333,7 @@
         <v>10</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -43410,7 +43410,7 @@
         <v>8</v>
       </c>
       <c r="M5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N5">
         <v>-1</v>
@@ -45862,7 +45862,7 @@
         <v>-1</v>
       </c>
       <c r="I37">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J37">
         <v>7</v>
@@ -45898,7 +45898,7 @@
         <v>-1</v>
       </c>
       <c r="U37">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V37">
         <v>7</v>
@@ -46691,7 +46691,7 @@
         <v>-1</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J6">
         <v>5</v>
@@ -46727,7 +46727,7 @@
         <v>5</v>
       </c>
       <c r="U6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V6">
         <v>6</v>
@@ -47461,7 +47461,7 @@
         <v>-1</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J16">
         <v>7</v>
@@ -47497,7 +47497,7 @@
         <v>6</v>
       </c>
       <c r="U16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V16">
         <v>7</v>
@@ -47615,7 +47615,7 @@
         <v>-1</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J18">
         <v>6</v>
@@ -47651,7 +47651,7 @@
         <v>6</v>
       </c>
       <c r="U18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V18">
         <v>6</v>
@@ -48539,7 +48539,7 @@
         <v>-1</v>
       </c>
       <c r="I30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J30">
         <v>7</v>
@@ -48575,7 +48575,7 @@
         <v>8</v>
       </c>
       <c r="U30">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="V30">
         <v>7</v>
@@ -57542,7 +57542,7 @@
         <v>9</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J4">
         <v>5</v>
@@ -57554,7 +57554,7 @@
         <v>8</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -57578,7 +57578,7 @@
         <v>8</v>
       </c>
       <c r="U4">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V4">
         <v>6</v>
@@ -57619,7 +57619,7 @@
         <v>10</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J5">
         <v>10</v>
@@ -57631,7 +57631,7 @@
         <v>10</v>
       </c>
       <c r="M5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N5">
         <v>-1</v>
@@ -57667,7 +57667,7 @@
         <v>9</v>
       </c>
       <c r="Y5">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -57696,7 +57696,7 @@
         <v>10</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J6">
         <v>10</v>
@@ -57708,7 +57708,7 @@
         <v>10</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -57744,7 +57744,7 @@
         <v>10</v>
       </c>
       <c r="Y6">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -57773,7 +57773,7 @@
         <v>9</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J7">
         <v>5</v>
@@ -57785,7 +57785,7 @@
         <v>5</v>
       </c>
       <c r="M7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N7">
         <v>-1</v>
@@ -57809,7 +57809,7 @@
         <v>7</v>
       </c>
       <c r="U7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V7">
         <v>5</v>
@@ -57821,7 +57821,7 @@
         <v>5</v>
       </c>
       <c r="Y7">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -57850,7 +57850,7 @@
         <v>8</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J8">
         <v>9</v>
@@ -57862,7 +57862,7 @@
         <v>6</v>
       </c>
       <c r="M8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -57886,7 +57886,7 @@
         <v>8</v>
       </c>
       <c r="U8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V8">
         <v>9</v>
@@ -57927,7 +57927,7 @@
         <v>8</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J9">
         <v>5</v>
@@ -57939,7 +57939,7 @@
         <v>8</v>
       </c>
       <c r="M9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N9">
         <v>-1</v>
@@ -57963,7 +57963,7 @@
         <v>9</v>
       </c>
       <c r="U9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V9">
         <v>5</v>
@@ -58004,7 +58004,7 @@
         <v>6</v>
       </c>
       <c r="I10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J10">
         <v>5</v>
@@ -58016,7 +58016,7 @@
         <v>6</v>
       </c>
       <c r="M10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N10">
         <v>-1</v>
@@ -58040,7 +58040,7 @@
         <v>6</v>
       </c>
       <c r="U10">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V10">
         <v>5</v>
@@ -58081,7 +58081,7 @@
         <v>10</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J11">
         <v>10</v>
@@ -58093,7 +58093,7 @@
         <v>10</v>
       </c>
       <c r="M11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N11">
         <v>-1</v>
@@ -58129,7 +58129,7 @@
         <v>10</v>
       </c>
       <c r="Y11">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -58158,7 +58158,7 @@
         <v>9</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J12">
         <v>10</v>
@@ -58170,7 +58170,7 @@
         <v>10</v>
       </c>
       <c r="M12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N12">
         <v>-1</v>
@@ -58194,7 +58194,7 @@
         <v>10</v>
       </c>
       <c r="U12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V12">
         <v>9</v>
@@ -58235,7 +58235,7 @@
         <v>9</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J13">
         <v>9</v>
@@ -58247,7 +58247,7 @@
         <v>9</v>
       </c>
       <c r="M13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N13">
         <v>-1</v>
@@ -58283,7 +58283,7 @@
         <v>9</v>
       </c>
       <c r="Y13">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -58312,7 +58312,7 @@
         <v>9</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J14">
         <v>9</v>
@@ -58324,7 +58324,7 @@
         <v>8</v>
       </c>
       <c r="M14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -58348,7 +58348,7 @@
         <v>9</v>
       </c>
       <c r="U14">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V14">
         <v>9</v>
@@ -58389,7 +58389,7 @@
         <v>10</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J15">
         <v>10</v>
@@ -58401,7 +58401,7 @@
         <v>10</v>
       </c>
       <c r="M15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N15">
         <v>-1</v>
@@ -58437,7 +58437,7 @@
         <v>10</v>
       </c>
       <c r="Y15">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:25">
@@ -58466,7 +58466,7 @@
         <v>9</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>5</v>
@@ -58478,7 +58478,7 @@
         <v>10</v>
       </c>
       <c r="M16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N16">
         <v>-1</v>
@@ -58502,7 +58502,7 @@
         <v>9</v>
       </c>
       <c r="U16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V16">
         <v>7</v>
@@ -58543,7 +58543,7 @@
         <v>9</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J17">
         <v>6</v>
@@ -58555,7 +58555,7 @@
         <v>8</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N17">
         <v>-1</v>
@@ -58579,7 +58579,7 @@
         <v>7</v>
       </c>
       <c r="U17">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V17">
         <v>7</v>
@@ -58620,7 +58620,7 @@
         <v>9</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J18">
         <v>10</v>
@@ -58632,7 +58632,7 @@
         <v>10</v>
       </c>
       <c r="M18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N18">
         <v>-1</v>
@@ -58656,7 +58656,7 @@
         <v>10</v>
       </c>
       <c r="U18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V18">
         <v>10</v>
@@ -58697,7 +58697,7 @@
         <v>8</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J19">
         <v>7</v>
@@ -58709,7 +58709,7 @@
         <v>8</v>
       </c>
       <c r="M19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N19">
         <v>-1</v>
@@ -58774,7 +58774,7 @@
         <v>10</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J20">
         <v>10</v>
@@ -58786,7 +58786,7 @@
         <v>10</v>
       </c>
       <c r="M20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N20">
         <v>-1</v>
@@ -58822,7 +58822,7 @@
         <v>10</v>
       </c>
       <c r="Y20">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="21" spans="1:25">
@@ -58851,7 +58851,7 @@
         <v>10</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J21">
         <v>10</v>
@@ -58863,7 +58863,7 @@
         <v>10</v>
       </c>
       <c r="M21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N21">
         <v>-1</v>
@@ -58928,7 +58928,7 @@
         <v>7</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J22">
         <v>5</v>
@@ -58940,7 +58940,7 @@
         <v>5</v>
       </c>
       <c r="M22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N22">
         <v>-1</v>
@@ -59005,7 +59005,7 @@
         <v>9</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J23">
         <v>9</v>
@@ -59017,7 +59017,7 @@
         <v>8</v>
       </c>
       <c r="M23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N23">
         <v>-1</v>
@@ -59041,7 +59041,7 @@
         <v>10</v>
       </c>
       <c r="U23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V23">
         <v>9</v>
@@ -59053,7 +59053,7 @@
         <v>9</v>
       </c>
       <c r="Y23">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:25">
@@ -59082,7 +59082,7 @@
         <v>10</v>
       </c>
       <c r="I24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J24">
         <v>10</v>
@@ -59094,7 +59094,7 @@
         <v>10</v>
       </c>
       <c r="M24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N24">
         <v>-1</v>
@@ -59130,7 +59130,7 @@
         <v>10</v>
       </c>
       <c r="Y24">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -59159,7 +59159,7 @@
         <v>10</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J25">
         <v>10</v>
@@ -59171,7 +59171,7 @@
         <v>10</v>
       </c>
       <c r="M25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N25">
         <v>-1</v>
@@ -59236,7 +59236,7 @@
         <v>7</v>
       </c>
       <c r="I26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J26">
         <v>5</v>
@@ -59248,7 +59248,7 @@
         <v>5</v>
       </c>
       <c r="M26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N26">
         <v>-1</v>
@@ -59272,7 +59272,7 @@
         <v>6</v>
       </c>
       <c r="U26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V26">
         <v>5</v>
@@ -59313,7 +59313,7 @@
         <v>9</v>
       </c>
       <c r="I27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J27">
         <v>9</v>
@@ -59325,7 +59325,7 @@
         <v>10</v>
       </c>
       <c r="M27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N27">
         <v>-1</v>
@@ -59390,7 +59390,7 @@
         <v>10</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J28">
         <v>9</v>
@@ -59402,7 +59402,7 @@
         <v>10</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -59426,7 +59426,7 @@
         <v>10</v>
       </c>
       <c r="U28">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="V28">
         <v>8</v>
@@ -59438,7 +59438,7 @@
         <v>9</v>
       </c>
       <c r="Y28">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -59467,7 +59467,7 @@
         <v>10</v>
       </c>
       <c r="I29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J29">
         <v>9</v>
@@ -59479,7 +59479,7 @@
         <v>10</v>
       </c>
       <c r="M29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N29">
         <v>-1</v>
@@ -59503,7 +59503,7 @@
         <v>10</v>
       </c>
       <c r="U29">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="V29">
         <v>9</v>
@@ -59515,7 +59515,7 @@
         <v>10</v>
       </c>
       <c r="Y29">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:25">
@@ -59544,7 +59544,7 @@
         <v>9</v>
       </c>
       <c r="I30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J30">
         <v>8</v>
@@ -59556,7 +59556,7 @@
         <v>7</v>
       </c>
       <c r="M30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N30">
         <v>-1</v>
@@ -59621,7 +59621,7 @@
         <v>8</v>
       </c>
       <c r="I31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J31">
         <v>10</v>
@@ -59633,7 +59633,7 @@
         <v>8</v>
       </c>
       <c r="M31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N31">
         <v>-1</v>
@@ -59669,7 +59669,7 @@
         <v>8</v>
       </c>
       <c r="Y31">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32" spans="1:25">
@@ -59698,7 +59698,7 @@
         <v>5</v>
       </c>
       <c r="I32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J32">
         <v>5</v>
@@ -59710,7 +59710,7 @@
         <v>5</v>
       </c>
       <c r="M32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N32">
         <v>-1</v>
@@ -59775,7 +59775,7 @@
         <v>9</v>
       </c>
       <c r="I33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J33">
         <v>10</v>
@@ -59787,7 +59787,7 @@
         <v>8</v>
       </c>
       <c r="M33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N33">
         <v>-1</v>
@@ -59852,7 +59852,7 @@
         <v>9</v>
       </c>
       <c r="I34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J34">
         <v>7</v>
@@ -59864,7 +59864,7 @@
         <v>10</v>
       </c>
       <c r="M34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N34">
         <v>-1</v>
@@ -59888,7 +59888,7 @@
         <v>9</v>
       </c>
       <c r="U34">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V34">
         <v>7</v>
@@ -59929,7 +59929,7 @@
         <v>7</v>
       </c>
       <c r="I35">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J35">
         <v>6</v>
@@ -59941,7 +59941,7 @@
         <v>5</v>
       </c>
       <c r="M35">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N35">
         <v>-1</v>
@@ -59977,7 +59977,7 @@
         <v>5</v>
       </c>
       <c r="Y35">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -60142,7 +60142,7 @@
         <v>7</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J4">
         <v>5</v>
@@ -60219,7 +60219,7 @@
         <v>9</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J5">
         <v>10</v>
@@ -60296,7 +60296,7 @@
         <v>9</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J6">
         <v>6</v>
@@ -60332,7 +60332,7 @@
         <v>9</v>
       </c>
       <c r="U6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="V6">
         <v>6</v>
@@ -60373,7 +60373,7 @@
         <v>9</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J7">
         <v>5</v>
@@ -60450,7 +60450,7 @@
         <v>9</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J8">
         <v>6</v>
@@ -60486,7 +60486,7 @@
         <v>10</v>
       </c>
       <c r="U8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V8">
         <v>7</v>
@@ -60527,7 +60527,7 @@
         <v>7</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J9">
         <v>6</v>
@@ -60604,7 +60604,7 @@
         <v>7</v>
       </c>
       <c r="I10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J10">
         <v>6</v>
@@ -60640,7 +60640,7 @@
         <v>7</v>
       </c>
       <c r="U10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V10">
         <v>7</v>
@@ -60681,7 +60681,7 @@
         <v>5</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J11">
         <v>5</v>
@@ -60717,7 +60717,7 @@
         <v>6</v>
       </c>
       <c r="U11">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V11">
         <v>5</v>
@@ -60758,7 +60758,7 @@
         <v>9</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="J12">
         <v>6</v>
@@ -60794,7 +60794,7 @@
         <v>10</v>
       </c>
       <c r="U12">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V12">
         <v>8</v>
@@ -60835,7 +60835,7 @@
         <v>7</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J13">
         <v>5</v>
@@ -60871,7 +60871,7 @@
         <v>8</v>
       </c>
       <c r="U13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V13">
         <v>5</v>
@@ -60912,7 +60912,7 @@
         <v>7</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J14">
         <v>5</v>
@@ -60989,7 +60989,7 @@
         <v>10</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J15">
         <v>6</v>
@@ -61025,7 +61025,7 @@
         <v>9</v>
       </c>
       <c r="U15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V15">
         <v>5</v>
@@ -61066,7 +61066,7 @@
         <v>10</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J16">
         <v>9</v>
@@ -61102,7 +61102,7 @@
         <v>10</v>
       </c>
       <c r="U16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V16">
         <v>9</v>
@@ -61143,7 +61143,7 @@
         <v>8</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J17">
         <v>5</v>
@@ -61220,7 +61220,7 @@
         <v>10</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J18">
         <v>6</v>
@@ -84923,7 +84923,7 @@
         <v>8</v>
       </c>
       <c r="J39">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K39">
         <v>7</v>
@@ -91494,7 +91494,7 @@
         <v>9</v>
       </c>
       <c r="K4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L4">
         <v>8</v>
@@ -91530,7 +91530,7 @@
         <v>10</v>
       </c>
       <c r="W4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X4">
         <v>7</v>
@@ -91571,7 +91571,7 @@
         <v>10</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L5">
         <v>10</v>
@@ -91648,7 +91648,7 @@
         <v>10</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L6">
         <v>9</v>
@@ -91725,7 +91725,7 @@
         <v>7</v>
       </c>
       <c r="K7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -91802,7 +91802,7 @@
         <v>10</v>
       </c>
       <c r="K8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L8">
         <v>9</v>
@@ -91879,7 +91879,7 @@
         <v>9</v>
       </c>
       <c r="K9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L9">
         <v>7</v>
@@ -91956,7 +91956,7 @@
         <v>9</v>
       </c>
       <c r="K10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L10">
         <v>10</v>
@@ -92033,7 +92033,7 @@
         <v>9</v>
       </c>
       <c r="K11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L11">
         <v>9</v>
@@ -92110,7 +92110,7 @@
         <v>10</v>
       </c>
       <c r="K12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L12">
         <v>10</v>
@@ -92187,7 +92187,7 @@
         <v>9</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L13">
         <v>10</v>
@@ -92264,7 +92264,7 @@
         <v>10</v>
       </c>
       <c r="K14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L14">
         <v>7</v>
@@ -92300,7 +92300,7 @@
         <v>10</v>
       </c>
       <c r="W14">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X14">
         <v>9</v>
@@ -92341,7 +92341,7 @@
         <v>9</v>
       </c>
       <c r="K15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L15">
         <v>7</v>
@@ -92418,7 +92418,7 @@
         <v>9</v>
       </c>
       <c r="K16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L16">
         <v>9</v>
@@ -92454,7 +92454,7 @@
         <v>9</v>
       </c>
       <c r="W16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X16">
         <v>9</v>
@@ -92495,7 +92495,7 @@
         <v>9</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L17">
         <v>10</v>
@@ -92572,7 +92572,7 @@
         <v>10</v>
       </c>
       <c r="K18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L18">
         <v>10</v>
@@ -92608,7 +92608,7 @@
         <v>10</v>
       </c>
       <c r="W18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X18">
         <v>10</v>
@@ -92649,7 +92649,7 @@
         <v>10</v>
       </c>
       <c r="K19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L19">
         <v>9</v>
@@ -92726,7 +92726,7 @@
         <v>9</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L20">
         <v>6</v>
@@ -92803,7 +92803,7 @@
         <v>10</v>
       </c>
       <c r="K21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L21">
         <v>9</v>
@@ -92880,7 +92880,7 @@
         <v>9</v>
       </c>
       <c r="K22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L22">
         <v>10</v>
@@ -92916,7 +92916,7 @@
         <v>10</v>
       </c>
       <c r="W22">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X22">
         <v>10</v>
@@ -92957,7 +92957,7 @@
         <v>9</v>
       </c>
       <c r="K23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L23">
         <v>9</v>
@@ -92993,7 +92993,7 @@
         <v>10</v>
       </c>
       <c r="W23">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X23">
         <v>10</v>
@@ -93034,7 +93034,7 @@
         <v>7</v>
       </c>
       <c r="K24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L24">
         <v>5</v>
@@ -93111,7 +93111,7 @@
         <v>8</v>
       </c>
       <c r="K25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L25">
         <v>8</v>
@@ -93188,7 +93188,7 @@
         <v>10</v>
       </c>
       <c r="K26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L26">
         <v>10</v>
@@ -93224,7 +93224,7 @@
         <v>10</v>
       </c>
       <c r="W26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X26">
         <v>10</v>
@@ -93265,7 +93265,7 @@
         <v>10</v>
       </c>
       <c r="K27">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L27">
         <v>10</v>
@@ -93342,7 +93342,7 @@
         <v>10</v>
       </c>
       <c r="K28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L28">
         <v>10</v>
@@ -93419,7 +93419,7 @@
         <v>7</v>
       </c>
       <c r="K29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L29">
         <v>7</v>
@@ -93496,7 +93496,7 @@
         <v>10</v>
       </c>
       <c r="K30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L30">
         <v>10</v>

</xml_diff>

<commit_message>
Segundo Parcial 9 noviembre
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -18870,7 +18870,7 @@
         <v>9</v>
       </c>
       <c r="K4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L4">
         <v>9</v>
@@ -18947,7 +18947,7 @@
         <v>7</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L5">
         <v>-1</v>
@@ -18983,7 +18983,7 @@
         <v>7</v>
       </c>
       <c r="W5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X5">
         <v>-1</v>
@@ -19024,7 +19024,7 @@
         <v>6</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L6">
         <v>9</v>
@@ -19101,7 +19101,7 @@
         <v>6</v>
       </c>
       <c r="K7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L7">
         <v>9</v>
@@ -19178,7 +19178,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L8">
         <v>9</v>
@@ -19214,7 +19214,7 @@
         <v>8</v>
       </c>
       <c r="W8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X8">
         <v>9</v>
@@ -19255,7 +19255,7 @@
         <v>7</v>
       </c>
       <c r="K9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L9">
         <v>9</v>
@@ -19332,7 +19332,7 @@
         <v>7</v>
       </c>
       <c r="K10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L10">
         <v>9</v>
@@ -19409,7 +19409,7 @@
         <v>5</v>
       </c>
       <c r="K11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L11">
         <v>9</v>
@@ -19486,7 +19486,7 @@
         <v>7</v>
       </c>
       <c r="K12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L12">
         <v>9</v>
@@ -19522,7 +19522,7 @@
         <v>7</v>
       </c>
       <c r="W12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X12">
         <v>8</v>
@@ -19563,7 +19563,7 @@
         <v>7</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L13">
         <v>9</v>
@@ -19599,7 +19599,7 @@
         <v>7</v>
       </c>
       <c r="W13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X13">
         <v>9</v>
@@ -19640,7 +19640,7 @@
         <v>10</v>
       </c>
       <c r="K14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L14">
         <v>10</v>
@@ -19717,7 +19717,7 @@
         <v>6</v>
       </c>
       <c r="K15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L15">
         <v>9</v>
@@ -19794,7 +19794,7 @@
         <v>7</v>
       </c>
       <c r="K16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L16">
         <v>9</v>
@@ -19830,7 +19830,7 @@
         <v>7</v>
       </c>
       <c r="W16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X16">
         <v>9</v>
@@ -19871,7 +19871,7 @@
         <v>7</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L17">
         <v>9</v>
@@ -19948,7 +19948,7 @@
         <v>8</v>
       </c>
       <c r="K18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L18">
         <v>9</v>
@@ -20025,7 +20025,7 @@
         <v>7</v>
       </c>
       <c r="K19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L19">
         <v>9</v>
@@ -20102,7 +20102,7 @@
         <v>7</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L20">
         <v>9</v>
@@ -20179,7 +20179,7 @@
         <v>8</v>
       </c>
       <c r="K21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L21">
         <v>9</v>
@@ -20256,7 +20256,7 @@
         <v>10</v>
       </c>
       <c r="K22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L22">
         <v>9</v>
@@ -20333,7 +20333,7 @@
         <v>7</v>
       </c>
       <c r="K23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L23">
         <v>9</v>
@@ -20369,7 +20369,7 @@
         <v>7</v>
       </c>
       <c r="W23">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X23">
         <v>8</v>
@@ -20410,7 +20410,7 @@
         <v>5</v>
       </c>
       <c r="K24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L24">
         <v>9</v>
@@ -20487,7 +20487,7 @@
         <v>9</v>
       </c>
       <c r="K25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L25">
         <v>9</v>
@@ -20564,7 +20564,7 @@
         <v>5</v>
       </c>
       <c r="K26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L26">
         <v>-1</v>
@@ -20641,7 +20641,7 @@
         <v>5</v>
       </c>
       <c r="K27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L27">
         <v>9</v>
@@ -20718,7 +20718,7 @@
         <v>5</v>
       </c>
       <c r="K28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L28">
         <v>9</v>
@@ -20754,7 +20754,7 @@
         <v>5</v>
       </c>
       <c r="W28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X28">
         <v>9</v>
@@ -20795,7 +20795,7 @@
         <v>6</v>
       </c>
       <c r="K29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L29">
         <v>9</v>
@@ -20872,7 +20872,7 @@
         <v>5</v>
       </c>
       <c r="K30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L30">
         <v>9</v>
@@ -20949,7 +20949,7 @@
         <v>10</v>
       </c>
       <c r="K31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L31">
         <v>9</v>
@@ -21026,7 +21026,7 @@
         <v>8</v>
       </c>
       <c r="K32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L32">
         <v>9</v>
@@ -21103,7 +21103,7 @@
         <v>8</v>
       </c>
       <c r="K33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L33">
         <v>9</v>
@@ -21180,7 +21180,7 @@
         <v>7</v>
       </c>
       <c r="K34">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L34">
         <v>9</v>
@@ -21257,7 +21257,7 @@
         <v>7</v>
       </c>
       <c r="K35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L35">
         <v>9</v>
@@ -21334,7 +21334,7 @@
         <v>8</v>
       </c>
       <c r="K36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L36">
         <v>9</v>
@@ -21411,7 +21411,7 @@
         <v>7</v>
       </c>
       <c r="K37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L37">
         <v>9</v>
@@ -21447,7 +21447,7 @@
         <v>7</v>
       </c>
       <c r="W37">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X37">
         <v>9</v>
@@ -21488,7 +21488,7 @@
         <v>8</v>
       </c>
       <c r="K38">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L38">
         <v>9</v>
@@ -21704,7 +21704,7 @@
         <v>9</v>
       </c>
       <c r="L4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M4">
         <v>7</v>
@@ -21740,7 +21740,7 @@
         <v>7</v>
       </c>
       <c r="X4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y4">
         <v>7</v>
@@ -21781,7 +21781,7 @@
         <v>9</v>
       </c>
       <c r="L5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M5">
         <v>6</v>
@@ -21858,7 +21858,7 @@
         <v>9</v>
       </c>
       <c r="L6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M6">
         <v>9</v>
@@ -21935,7 +21935,7 @@
         <v>7</v>
       </c>
       <c r="L7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M7">
         <v>7</v>
@@ -21971,7 +21971,7 @@
         <v>7</v>
       </c>
       <c r="X7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y7">
         <v>7</v>
@@ -22012,7 +22012,7 @@
         <v>9</v>
       </c>
       <c r="L8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M8">
         <v>9</v>
@@ -22089,7 +22089,7 @@
         <v>9</v>
       </c>
       <c r="L9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="M9">
         <v>8</v>
@@ -22166,7 +22166,7 @@
         <v>9</v>
       </c>
       <c r="L10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M10">
         <v>8</v>
@@ -22243,7 +22243,7 @@
         <v>6</v>
       </c>
       <c r="L11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M11">
         <v>8</v>
@@ -22279,7 +22279,7 @@
         <v>7</v>
       </c>
       <c r="X11">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y11">
         <v>8</v>
@@ -22320,7 +22320,7 @@
         <v>5</v>
       </c>
       <c r="L12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M12">
         <v>6</v>
@@ -22356,7 +22356,7 @@
         <v>7</v>
       </c>
       <c r="X12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y12">
         <v>7</v>
@@ -22397,7 +22397,7 @@
         <v>6</v>
       </c>
       <c r="L13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M13">
         <v>10</v>
@@ -22474,7 +22474,7 @@
         <v>7</v>
       </c>
       <c r="L14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M14">
         <v>10</v>
@@ -22510,7 +22510,7 @@
         <v>7</v>
       </c>
       <c r="X14">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y14">
         <v>10</v>
@@ -22551,7 +22551,7 @@
         <v>9</v>
       </c>
       <c r="L15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M15">
         <v>9</v>
@@ -22628,7 +22628,7 @@
         <v>9</v>
       </c>
       <c r="L16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M16">
         <v>10</v>
@@ -22705,7 +22705,7 @@
         <v>-1</v>
       </c>
       <c r="L17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M17">
         <v>5</v>
@@ -22782,7 +22782,7 @@
         <v>6</v>
       </c>
       <c r="L18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M18">
         <v>6</v>
@@ -22859,7 +22859,7 @@
         <v>9</v>
       </c>
       <c r="L19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="M19">
         <v>9</v>
@@ -22936,7 +22936,7 @@
         <v>10</v>
       </c>
       <c r="L20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M20">
         <v>10</v>
@@ -23013,7 +23013,7 @@
         <v>9</v>
       </c>
       <c r="L21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M21">
         <v>7</v>
@@ -23090,7 +23090,7 @@
         <v>-1</v>
       </c>
       <c r="L22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M22">
         <v>7</v>
@@ -23126,7 +23126,7 @@
         <v>-1</v>
       </c>
       <c r="X22">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y22">
         <v>8</v>
@@ -23167,7 +23167,7 @@
         <v>10</v>
       </c>
       <c r="L23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M23">
         <v>9</v>
@@ -23244,7 +23244,7 @@
         <v>-1</v>
       </c>
       <c r="L24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M24">
         <v>8</v>
@@ -23280,7 +23280,7 @@
         <v>-1</v>
       </c>
       <c r="X24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y24">
         <v>7</v>
@@ -23451,7 +23451,7 @@
         <v>9</v>
       </c>
       <c r="J4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K4">
         <v>9</v>
@@ -23528,7 +23528,7 @@
         <v>7</v>
       </c>
       <c r="J5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K5">
         <v>9</v>
@@ -23605,7 +23605,7 @@
         <v>7</v>
       </c>
       <c r="J6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K6">
         <v>9</v>
@@ -23682,7 +23682,7 @@
         <v>8</v>
       </c>
       <c r="J7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K7">
         <v>9</v>
@@ -23759,7 +23759,7 @@
         <v>6</v>
       </c>
       <c r="J8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K8">
         <v>9</v>
@@ -23836,7 +23836,7 @@
         <v>9</v>
       </c>
       <c r="J9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K9">
         <v>9</v>
@@ -23872,7 +23872,7 @@
         <v>8</v>
       </c>
       <c r="V9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W9">
         <v>9</v>
@@ -23913,7 +23913,7 @@
         <v>6</v>
       </c>
       <c r="J10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K10">
         <v>9</v>
@@ -23990,7 +23990,7 @@
         <v>9</v>
       </c>
       <c r="J11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K11">
         <v>9</v>
@@ -24026,7 +24026,7 @@
         <v>9</v>
       </c>
       <c r="V11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W11">
         <v>9</v>
@@ -24067,7 +24067,7 @@
         <v>8</v>
       </c>
       <c r="J12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K12">
         <v>9</v>
@@ -24144,7 +24144,7 @@
         <v>6</v>
       </c>
       <c r="J13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K13">
         <v>9</v>
@@ -24221,7 +24221,7 @@
         <v>9</v>
       </c>
       <c r="J14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K14">
         <v>9</v>
@@ -24298,7 +24298,7 @@
         <v>8</v>
       </c>
       <c r="J15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K15">
         <v>9</v>
@@ -24334,7 +24334,7 @@
         <v>8</v>
       </c>
       <c r="V15">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W15">
         <v>9</v>
@@ -24375,7 +24375,7 @@
         <v>8</v>
       </c>
       <c r="J16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K16">
         <v>9</v>
@@ -24452,7 +24452,7 @@
         <v>7</v>
       </c>
       <c r="J17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K17">
         <v>9</v>
@@ -24488,7 +24488,7 @@
         <v>7</v>
       </c>
       <c r="V17">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W17">
         <v>9</v>
@@ -24529,7 +24529,7 @@
         <v>7</v>
       </c>
       <c r="J18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K18">
         <v>9</v>
@@ -24565,7 +24565,7 @@
         <v>7</v>
       </c>
       <c r="V18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W18">
         <v>9</v>
@@ -24606,7 +24606,7 @@
         <v>7</v>
       </c>
       <c r="J19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K19">
         <v>9</v>
@@ -24683,7 +24683,7 @@
         <v>8</v>
       </c>
       <c r="J20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K20">
         <v>9</v>
@@ -24760,7 +24760,7 @@
         <v>8</v>
       </c>
       <c r="J21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K21">
         <v>9</v>
@@ -24837,7 +24837,7 @@
         <v>6</v>
       </c>
       <c r="J22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K22">
         <v>9</v>
@@ -24914,7 +24914,7 @@
         <v>-1</v>
       </c>
       <c r="J23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K23">
         <v>9</v>
@@ -24991,7 +24991,7 @@
         <v>7</v>
       </c>
       <c r="J24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K24">
         <v>9</v>
@@ -25068,7 +25068,7 @@
         <v>7</v>
       </c>
       <c r="J25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K25">
         <v>9</v>
@@ -25104,7 +25104,7 @@
         <v>7</v>
       </c>
       <c r="V25">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W25">
         <v>9</v>
@@ -25145,7 +25145,7 @@
         <v>7</v>
       </c>
       <c r="J26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K26">
         <v>9</v>
@@ -25222,7 +25222,7 @@
         <v>-1</v>
       </c>
       <c r="J27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K27">
         <v>9</v>
@@ -25299,7 +25299,7 @@
         <v>7</v>
       </c>
       <c r="J28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K28">
         <v>9</v>
@@ -25376,7 +25376,7 @@
         <v>7</v>
       </c>
       <c r="J29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K29">
         <v>9</v>
@@ -25453,7 +25453,7 @@
         <v>7</v>
       </c>
       <c r="J30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K30">
         <v>9</v>
@@ -25530,7 +25530,7 @@
         <v>6</v>
       </c>
       <c r="J31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K31">
         <v>9</v>
@@ -25607,7 +25607,7 @@
         <v>9</v>
       </c>
       <c r="J32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K32">
         <v>9</v>
@@ -25684,7 +25684,7 @@
         <v>7</v>
       </c>
       <c r="J33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K33">
         <v>9</v>
@@ -25720,7 +25720,7 @@
         <v>7</v>
       </c>
       <c r="V33">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W33">
         <v>8</v>
@@ -25761,7 +25761,7 @@
         <v>7</v>
       </c>
       <c r="J34">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K34">
         <v>9</v>
@@ -25797,7 +25797,7 @@
         <v>7</v>
       </c>
       <c r="V34">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W34">
         <v>9</v>
@@ -25838,7 +25838,7 @@
         <v>7</v>
       </c>
       <c r="J35">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K35">
         <v>9</v>
@@ -25915,7 +25915,7 @@
         <v>7</v>
       </c>
       <c r="J36">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K36">
         <v>9</v>
@@ -25951,7 +25951,7 @@
         <v>8</v>
       </c>
       <c r="V36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W36">
         <v>9</v>
@@ -25992,7 +25992,7 @@
         <v>9</v>
       </c>
       <c r="J37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="K37">
         <v>9</v>
@@ -26069,7 +26069,7 @@
         <v>8</v>
       </c>
       <c r="J38">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K38">
         <v>9</v>
@@ -26146,7 +26146,7 @@
         <v>8</v>
       </c>
       <c r="J39">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K39">
         <v>9</v>
@@ -26223,7 +26223,7 @@
         <v>6</v>
       </c>
       <c r="J40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K40">
         <v>9</v>
@@ -29172,7 +29172,7 @@
         <v>-1</v>
       </c>
       <c r="K4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -29249,7 +29249,7 @@
         <v>8</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L5">
         <v>10</v>
@@ -29326,7 +29326,7 @@
         <v>-1</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L6">
         <v>10</v>
@@ -29362,7 +29362,7 @@
         <v>-1</v>
       </c>
       <c r="W6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X6">
         <v>10</v>
@@ -29403,7 +29403,7 @@
         <v>7</v>
       </c>
       <c r="K7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L7">
         <v>6</v>
@@ -29480,7 +29480,7 @@
         <v>8</v>
       </c>
       <c r="K8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L8">
         <v>10</v>
@@ -29516,7 +29516,7 @@
         <v>8</v>
       </c>
       <c r="W8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X8">
         <v>10</v>
@@ -29557,7 +29557,7 @@
         <v>8</v>
       </c>
       <c r="K9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L9">
         <v>10</v>
@@ -29634,7 +29634,7 @@
         <v>7</v>
       </c>
       <c r="K10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L10">
         <v>10</v>
@@ -29670,7 +29670,7 @@
         <v>7</v>
       </c>
       <c r="W10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X10">
         <v>10</v>
@@ -29711,7 +29711,7 @@
         <v>8</v>
       </c>
       <c r="K11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L11">
         <v>10</v>
@@ -29788,7 +29788,7 @@
         <v>7</v>
       </c>
       <c r="K12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L12">
         <v>10</v>
@@ -29824,7 +29824,7 @@
         <v>8</v>
       </c>
       <c r="W12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X12">
         <v>10</v>
@@ -29865,7 +29865,7 @@
         <v>7</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L13">
         <v>10</v>
@@ -29901,7 +29901,7 @@
         <v>7</v>
       </c>
       <c r="W13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X13">
         <v>10</v>
@@ -29942,7 +29942,7 @@
         <v>-1</v>
       </c>
       <c r="K14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L14">
         <v>10</v>
@@ -29978,7 +29978,7 @@
         <v>-1</v>
       </c>
       <c r="W14">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="X14">
         <v>10</v>
@@ -30019,7 +30019,7 @@
         <v>-1</v>
       </c>
       <c r="K15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L15">
         <v>7</v>
@@ -30055,7 +30055,7 @@
         <v>-1</v>
       </c>
       <c r="W15">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X15">
         <v>6</v>
@@ -30096,7 +30096,7 @@
         <v>8</v>
       </c>
       <c r="K16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L16">
         <v>9</v>
@@ -30132,7 +30132,7 @@
         <v>8</v>
       </c>
       <c r="W16">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X16">
         <v>10</v>
@@ -30173,7 +30173,7 @@
         <v>-1</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L17">
         <v>10</v>
@@ -30250,7 +30250,7 @@
         <v>7</v>
       </c>
       <c r="K18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L18">
         <v>10</v>
@@ -30286,7 +30286,7 @@
         <v>7</v>
       </c>
       <c r="W18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X18">
         <v>10</v>
@@ -30327,7 +30327,7 @@
         <v>-1</v>
       </c>
       <c r="K19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L19">
         <v>10</v>
@@ -30363,7 +30363,7 @@
         <v>-1</v>
       </c>
       <c r="W19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X19">
         <v>8</v>
@@ -30404,7 +30404,7 @@
         <v>7</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L20">
         <v>10</v>
@@ -30481,7 +30481,7 @@
         <v>-1</v>
       </c>
       <c r="K21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L21">
         <v>10</v>
@@ -30558,7 +30558,7 @@
         <v>7</v>
       </c>
       <c r="K22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L22">
         <v>10</v>
@@ -30594,7 +30594,7 @@
         <v>7</v>
       </c>
       <c r="W22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X22">
         <v>10</v>
@@ -30635,7 +30635,7 @@
         <v>7</v>
       </c>
       <c r="K23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L23">
         <v>10</v>
@@ -30671,7 +30671,7 @@
         <v>7</v>
       </c>
       <c r="W23">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X23">
         <v>10</v>
@@ -30712,7 +30712,7 @@
         <v>7</v>
       </c>
       <c r="K24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L24">
         <v>10</v>
@@ -30748,7 +30748,7 @@
         <v>7</v>
       </c>
       <c r="W24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X24">
         <v>9</v>
@@ -30789,7 +30789,7 @@
         <v>-1</v>
       </c>
       <c r="K25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L25">
         <v>10</v>
@@ -30825,7 +30825,7 @@
         <v>-1</v>
       </c>
       <c r="W25">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X25">
         <v>8</v>
@@ -30866,7 +30866,7 @@
         <v>7</v>
       </c>
       <c r="K26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L26">
         <v>10</v>
@@ -30902,7 +30902,7 @@
         <v>7</v>
       </c>
       <c r="W26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X26">
         <v>8</v>
@@ -30943,7 +30943,7 @@
         <v>-1</v>
       </c>
       <c r="K27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L27">
         <v>8</v>
@@ -31020,7 +31020,7 @@
         <v>-1</v>
       </c>
       <c r="K28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L28">
         <v>10</v>
@@ -31056,7 +31056,7 @@
         <v>-1</v>
       </c>
       <c r="W28">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X28">
         <v>8</v>
@@ -31097,7 +31097,7 @@
         <v>8</v>
       </c>
       <c r="K29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L29">
         <v>10</v>
@@ -31174,7 +31174,7 @@
         <v>8</v>
       </c>
       <c r="K30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L30">
         <v>10</v>
@@ -31251,7 +31251,7 @@
         <v>6</v>
       </c>
       <c r="K31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L31">
         <v>10</v>
@@ -31287,7 +31287,7 @@
         <v>6</v>
       </c>
       <c r="W31">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X31">
         <v>10</v>
@@ -31328,7 +31328,7 @@
         <v>7</v>
       </c>
       <c r="K32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L32">
         <v>10</v>
@@ -31405,7 +31405,7 @@
         <v>8</v>
       </c>
       <c r="K33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L33">
         <v>10</v>
@@ -31441,7 +31441,7 @@
         <v>8</v>
       </c>
       <c r="W33">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X33">
         <v>10</v>
@@ -31482,7 +31482,7 @@
         <v>7</v>
       </c>
       <c r="K34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L34">
         <v>10</v>
@@ -31559,7 +31559,7 @@
         <v>8</v>
       </c>
       <c r="K35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L35">
         <v>10</v>
@@ -31595,7 +31595,7 @@
         <v>8</v>
       </c>
       <c r="W35">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X35">
         <v>10</v>
@@ -43318,7 +43318,7 @@
         <v>7</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I4">
         <v>6</v>
@@ -43395,7 +43395,7 @@
         <v>6</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I5">
         <v>6</v>
@@ -43472,7 +43472,7 @@
         <v>-1</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I6">
         <v>-1</v>
@@ -43508,7 +43508,7 @@
         <v>-1</v>
       </c>
       <c r="T6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U6">
         <v>-1</v>
@@ -43549,7 +43549,7 @@
         <v>9</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I7">
         <v>10</v>
@@ -43585,7 +43585,7 @@
         <v>-1</v>
       </c>
       <c r="T7">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U7">
         <v>8</v>
@@ -43703,7 +43703,7 @@
         <v>6</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I9">
         <v>6</v>
@@ -43780,7 +43780,7 @@
         <v>-1</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I10">
         <v>6</v>
@@ -43816,7 +43816,7 @@
         <v>-1</v>
       </c>
       <c r="T10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U10">
         <v>6</v>
@@ -43857,7 +43857,7 @@
         <v>7</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I11">
         <v>6</v>
@@ -43893,7 +43893,7 @@
         <v>-1</v>
       </c>
       <c r="T11">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U11">
         <v>7</v>
@@ -43934,7 +43934,7 @@
         <v>7</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I12">
         <v>7</v>
@@ -44088,7 +44088,7 @@
         <v>6</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I14">
         <v>6</v>
@@ -44124,7 +44124,7 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U14">
         <v>7</v>
@@ -44165,7 +44165,7 @@
         <v>8</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I15">
         <v>6</v>
@@ -44201,7 +44201,7 @@
         <v>-1</v>
       </c>
       <c r="T15">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U15">
         <v>6</v>
@@ -44396,7 +44396,7 @@
         <v>6</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I18">
         <v>6</v>
@@ -44473,7 +44473,7 @@
         <v>7</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I19">
         <v>6</v>
@@ -44509,7 +44509,7 @@
         <v>-1</v>
       </c>
       <c r="T19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U19">
         <v>7</v>
@@ -44550,7 +44550,7 @@
         <v>6</v>
       </c>
       <c r="H20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I20">
         <v>-1</v>
@@ -44627,7 +44627,7 @@
         <v>-1</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I21">
         <v>6</v>
@@ -44704,7 +44704,7 @@
         <v>9</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I22">
         <v>6</v>
@@ -44740,7 +44740,7 @@
         <v>-1</v>
       </c>
       <c r="T22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U22">
         <v>8</v>
@@ -44781,7 +44781,7 @@
         <v>7</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I23">
         <v>7</v>
@@ -44817,7 +44817,7 @@
         <v>-1</v>
       </c>
       <c r="T23">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U23">
         <v>7</v>
@@ -44858,7 +44858,7 @@
         <v>6</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I24">
         <v>6</v>
@@ -44935,7 +44935,7 @@
         <v>8</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I25">
         <v>6</v>
@@ -45012,7 +45012,7 @@
         <v>7</v>
       </c>
       <c r="H26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I26">
         <v>7</v>
@@ -45089,7 +45089,7 @@
         <v>6</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I27">
         <v>6</v>
@@ -45166,7 +45166,7 @@
         <v>6</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I28">
         <v>6</v>
@@ -45243,7 +45243,7 @@
         <v>6</v>
       </c>
       <c r="H29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I29">
         <v>6</v>
@@ -45279,7 +45279,7 @@
         <v>-1</v>
       </c>
       <c r="T29">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U29">
         <v>7</v>
@@ -45320,7 +45320,7 @@
         <v>8</v>
       </c>
       <c r="H30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I30">
         <v>6</v>
@@ -45397,7 +45397,7 @@
         <v>6</v>
       </c>
       <c r="H31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I31">
         <v>6</v>
@@ -45433,7 +45433,7 @@
         <v>-1</v>
       </c>
       <c r="T31">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U31">
         <v>6</v>
@@ -45474,7 +45474,7 @@
         <v>9</v>
       </c>
       <c r="H32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I32">
         <v>7</v>
@@ -45510,7 +45510,7 @@
         <v>-1</v>
       </c>
       <c r="T32">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U32">
         <v>7</v>
@@ -45551,7 +45551,7 @@
         <v>6</v>
       </c>
       <c r="H33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I33">
         <v>6</v>
@@ -45628,7 +45628,7 @@
         <v>-1</v>
       </c>
       <c r="H34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I34">
         <v>6</v>
@@ -45705,7 +45705,7 @@
         <v>7</v>
       </c>
       <c r="H35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I35">
         <v>6</v>
@@ -45782,7 +45782,7 @@
         <v>-1</v>
       </c>
       <c r="H36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I36">
         <v>-1</v>
@@ -45936,7 +45936,7 @@
         <v>8</v>
       </c>
       <c r="H38">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I38">
         <v>5</v>
@@ -46013,7 +46013,7 @@
         <v>6</v>
       </c>
       <c r="H39">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I39">
         <v>6</v>
@@ -46090,7 +46090,7 @@
         <v>6</v>
       </c>
       <c r="H40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I40">
         <v>6</v>
@@ -46126,7 +46126,7 @@
         <v>-1</v>
       </c>
       <c r="T40">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U40">
         <v>6</v>
@@ -46167,7 +46167,7 @@
         <v>8</v>
       </c>
       <c r="H41">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I41">
         <v>6</v>
@@ -46244,7 +46244,7 @@
         <v>8</v>
       </c>
       <c r="H42">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I42">
         <v>6</v>
@@ -46280,7 +46280,7 @@
         <v>-1</v>
       </c>
       <c r="T42">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U42">
         <v>7</v>
@@ -46321,7 +46321,7 @@
         <v>6</v>
       </c>
       <c r="H43">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I43">
         <v>6</v>
@@ -49365,7 +49365,7 @@
         <v>5</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I4">
         <v>5</v>
@@ -49401,7 +49401,7 @@
         <v>-1</v>
       </c>
       <c r="T4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="U4">
         <v>5</v>
@@ -49439,7 +49439,7 @@
         <v>7</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I5">
         <v>7</v>
@@ -49469,7 +49469,7 @@
         <v>-1</v>
       </c>
       <c r="T5">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U5">
         <v>8</v>
@@ -49507,7 +49507,7 @@
         <v>8</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I6">
         <v>8</v>
@@ -49584,7 +49584,7 @@
         <v>7</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I7">
         <v>5</v>
@@ -49620,7 +49620,7 @@
         <v>-1</v>
       </c>
       <c r="T7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U7">
         <v>5</v>
@@ -49767,7 +49767,7 @@
         <v>7</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I10">
         <v>6</v>
@@ -49803,7 +49803,7 @@
         <v>-1</v>
       </c>
       <c r="T10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U10">
         <v>5</v>
@@ -49844,7 +49844,7 @@
         <v>8</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I11">
         <v>9</v>
@@ -49880,7 +49880,7 @@
         <v>-1</v>
       </c>
       <c r="T11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U11">
         <v>9</v>
@@ -49921,7 +49921,7 @@
         <v>8</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I12">
         <v>5</v>
@@ -49957,7 +49957,7 @@
         <v>-1</v>
       </c>
       <c r="T12">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="U12">
         <v>7</v>
@@ -49998,7 +49998,7 @@
         <v>5</v>
       </c>
       <c r="H13">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I13">
         <v>7</v>
@@ -50034,7 +50034,7 @@
         <v>-1</v>
       </c>
       <c r="T13">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="U13">
         <v>8</v>
@@ -50075,7 +50075,7 @@
         <v>5</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I14">
         <v>5</v>
@@ -50111,7 +50111,7 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U14">
         <v>5</v>
@@ -50152,7 +50152,7 @@
         <v>7</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I15">
         <v>7</v>
@@ -50188,7 +50188,7 @@
         <v>-1</v>
       </c>
       <c r="T15">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U15">
         <v>7</v>
@@ -50229,7 +50229,7 @@
         <v>6</v>
       </c>
       <c r="H16">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I16">
         <v>6</v>
@@ -50265,7 +50265,7 @@
         <v>-1</v>
       </c>
       <c r="T16">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="U16">
         <v>7</v>
@@ -50306,7 +50306,7 @@
         <v>9</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I17">
         <v>9</v>
@@ -50342,7 +50342,7 @@
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U17">
         <v>10</v>
@@ -50383,7 +50383,7 @@
         <v>6</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I18">
         <v>5</v>
@@ -50460,7 +50460,7 @@
         <v>7</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I19">
         <v>8</v>
@@ -50496,7 +50496,7 @@
         <v>-1</v>
       </c>
       <c r="T19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U19">
         <v>7</v>
@@ -50554,7 +50554,7 @@
         <v>7</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I21">
         <v>9</v>
@@ -50631,7 +50631,7 @@
         <v>6</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I22">
         <v>9</v>
@@ -50667,7 +50667,7 @@
         <v>-1</v>
       </c>
       <c r="T22">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U22">
         <v>8</v>
@@ -50708,7 +50708,7 @@
         <v>7</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I23">
         <v>5</v>
@@ -50785,7 +50785,7 @@
         <v>8</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I24">
         <v>10</v>
@@ -50862,7 +50862,7 @@
         <v>6</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I25">
         <v>9</v>
@@ -50939,7 +50939,7 @@
         <v>8</v>
       </c>
       <c r="H26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I26">
         <v>9</v>
@@ -50975,7 +50975,7 @@
         <v>-1</v>
       </c>
       <c r="T26">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U26">
         <v>10</v>
@@ -51016,7 +51016,7 @@
         <v>9</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I27">
         <v>10</v>
@@ -51134,7 +51134,7 @@
         <v>10</v>
       </c>
       <c r="H29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I29">
         <v>7</v>
@@ -51170,7 +51170,7 @@
         <v>-1</v>
       </c>
       <c r="T29">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U29">
         <v>8</v>
@@ -51288,7 +51288,7 @@
         <v>5</v>
       </c>
       <c r="H31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I31">
         <v>5</v>
@@ -51324,7 +51324,7 @@
         <v>-1</v>
       </c>
       <c r="T31">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U31">
         <v>5</v>
@@ -51365,7 +51365,7 @@
         <v>6</v>
       </c>
       <c r="H32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I32">
         <v>5</v>
@@ -51442,7 +51442,7 @@
         <v>7</v>
       </c>
       <c r="H33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I33">
         <v>8</v>
@@ -51548,7 +51548,7 @@
         <v>7</v>
       </c>
       <c r="H35">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I35">
         <v>9</v>
@@ -51625,7 +51625,7 @@
         <v>7</v>
       </c>
       <c r="H36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I36">
         <v>8</v>
@@ -51661,7 +51661,7 @@
         <v>-1</v>
       </c>
       <c r="T36">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U36">
         <v>9</v>
@@ -51702,7 +51702,7 @@
         <v>7</v>
       </c>
       <c r="H37">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I37">
         <v>7</v>
@@ -51738,7 +51738,7 @@
         <v>-1</v>
       </c>
       <c r="T37">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U37">
         <v>8</v>
@@ -51779,7 +51779,7 @@
         <v>8</v>
       </c>
       <c r="H38">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I38">
         <v>10</v>
@@ -51856,7 +51856,7 @@
         <v>6</v>
       </c>
       <c r="H39">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I39">
         <v>5</v>
@@ -51892,7 +51892,7 @@
         <v>-1</v>
       </c>
       <c r="T39">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="U39">
         <v>5</v>
@@ -51933,7 +51933,7 @@
         <v>7</v>
       </c>
       <c r="H40">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I40">
         <v>5</v>
@@ -52010,7 +52010,7 @@
         <v>8</v>
       </c>
       <c r="H41">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I41">
         <v>9</v>
@@ -52087,7 +52087,7 @@
         <v>7</v>
       </c>
       <c r="H42">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I42">
         <v>5</v>
@@ -52123,7 +52123,7 @@
         <v>-1</v>
       </c>
       <c r="T42">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U42">
         <v>5</v>
@@ -61458,7 +61458,7 @@
         <v>9</v>
       </c>
       <c r="L4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M4">
         <v>10</v>
@@ -61500,7 +61500,7 @@
         <v>9</v>
       </c>
       <c r="Z4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA4">
         <v>10</v>
@@ -61636,7 +61636,7 @@
         <v>5</v>
       </c>
       <c r="L6">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="M6">
         <v>6</v>
@@ -61678,7 +61678,7 @@
         <v>5</v>
       </c>
       <c r="Z6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA6">
         <v>8</v>
@@ -61725,7 +61725,7 @@
         <v>9</v>
       </c>
       <c r="L7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M7">
         <v>10</v>
@@ -62081,7 +62081,7 @@
         <v>7</v>
       </c>
       <c r="L11">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="M11">
         <v>6</v>
@@ -62123,7 +62123,7 @@
         <v>7</v>
       </c>
       <c r="Z11">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AA11">
         <v>7</v>
@@ -62170,7 +62170,7 @@
         <v>8</v>
       </c>
       <c r="L12">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="M12">
         <v>10</v>
@@ -62212,7 +62212,7 @@
         <v>8</v>
       </c>
       <c r="Z12">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AA12">
         <v>10</v>
@@ -63149,7 +63149,7 @@
         <v>10</v>
       </c>
       <c r="L23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M23">
         <v>10</v>
@@ -63238,7 +63238,7 @@
         <v>5</v>
       </c>
       <c r="L24">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="M24">
         <v>7</v>
@@ -63280,7 +63280,7 @@
         <v>7</v>
       </c>
       <c r="Z24">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AA24">
         <v>9</v>
@@ -67275,7 +67275,7 @@
         <v>8</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L6">
         <v>9</v>
@@ -68122,7 +68122,7 @@
         <v>8</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L17">
         <v>10</v>
@@ -68158,7 +68158,7 @@
         <v>8</v>
       </c>
       <c r="W17">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X17">
         <v>10</v>
@@ -68199,7 +68199,7 @@
         <v>10</v>
       </c>
       <c r="K18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L18">
         <v>10</v>
@@ -68353,7 +68353,7 @@
         <v>8</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L20">
         <v>10</v>
@@ -68507,7 +68507,7 @@
         <v>9</v>
       </c>
       <c r="K22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L22">
         <v>9</v>
@@ -68543,7 +68543,7 @@
         <v>9</v>
       </c>
       <c r="W22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X22">
         <v>10</v>
@@ -68969,7 +68969,7 @@
         <v>9</v>
       </c>
       <c r="K28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L28">
         <v>10</v>
@@ -69005,7 +69005,7 @@
         <v>9</v>
       </c>
       <c r="W28">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X28">
         <v>10</v>
@@ -70860,7 +70860,7 @@
         <v>-1</v>
       </c>
       <c r="L4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="M4">
         <v>6</v>
@@ -70878,7 +70878,7 @@
         <v>-1</v>
       </c>
       <c r="X4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Y4">
         <v>6</v>
@@ -70942,7 +70942,7 @@
         <v>6</v>
       </c>
       <c r="J6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="K6">
         <v>9</v>
@@ -70978,7 +70978,7 @@
         <v>5</v>
       </c>
       <c r="V6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="W6">
         <v>9</v>
@@ -71019,13 +71019,13 @@
         <v>9</v>
       </c>
       <c r="J7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K7">
         <v>6</v>
       </c>
       <c r="L7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="M7">
         <v>9</v>
@@ -71055,13 +71055,13 @@
         <v>9</v>
       </c>
       <c r="V7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W7">
         <v>7</v>
       </c>
       <c r="X7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y7">
         <v>9</v>
@@ -71096,13 +71096,13 @@
         <v>10</v>
       </c>
       <c r="J8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="K8">
         <v>10</v>
       </c>
       <c r="L8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="M8">
         <v>10</v>
@@ -71132,13 +71132,13 @@
         <v>9</v>
       </c>
       <c r="V8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W8">
         <v>10</v>
       </c>
       <c r="X8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y8">
         <v>10</v>
@@ -71179,7 +71179,7 @@
         <v>9</v>
       </c>
       <c r="L9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="M9">
         <v>8</v>
@@ -71215,7 +71215,7 @@
         <v>10</v>
       </c>
       <c r="X9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Y9">
         <v>8</v>
@@ -71256,7 +71256,7 @@
         <v>10</v>
       </c>
       <c r="L10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M10">
         <v>9</v>
@@ -71292,7 +71292,7 @@
         <v>9</v>
       </c>
       <c r="X10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y10">
         <v>8</v>
@@ -71481,7 +71481,7 @@
         <v>6</v>
       </c>
       <c r="J13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K13">
         <v>10</v>
@@ -71517,7 +71517,7 @@
         <v>5</v>
       </c>
       <c r="V13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W13">
         <v>10</v>
@@ -71866,7 +71866,7 @@
         <v>6</v>
       </c>
       <c r="J18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K18">
         <v>10</v>
@@ -71902,7 +71902,7 @@
         <v>7</v>
       </c>
       <c r="V18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W18">
         <v>10</v>
@@ -72600,7 +72600,7 @@
         <v>6</v>
       </c>
       <c r="J28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K28">
         <v>10</v>
@@ -72636,7 +72636,7 @@
         <v>6</v>
       </c>
       <c r="V28">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W28">
         <v>10</v>
@@ -72754,7 +72754,7 @@
         <v>6</v>
       </c>
       <c r="J30">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K30">
         <v>10</v>
@@ -72985,13 +72985,13 @@
         <v>10</v>
       </c>
       <c r="J33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="K33">
         <v>10</v>
       </c>
       <c r="L33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="M33">
         <v>10</v>
@@ -73062,13 +73062,13 @@
         <v>9</v>
       </c>
       <c r="J34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="K34">
         <v>10</v>
       </c>
       <c r="L34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="M34">
         <v>10</v>
@@ -73098,13 +73098,13 @@
         <v>7</v>
       </c>
       <c r="V34">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="W34">
         <v>10</v>
       </c>
       <c r="X34">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y34">
         <v>10</v>
@@ -73198,7 +73198,7 @@
         <v>8</v>
       </c>
       <c r="L36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="M36">
         <v>6</v>
@@ -73210,7 +73210,7 @@
         <v>-1</v>
       </c>
       <c r="X36">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Y36">
         <v>7</v>
@@ -73322,13 +73322,13 @@
         <v>9</v>
       </c>
       <c r="J38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="K38">
         <v>10</v>
       </c>
       <c r="L38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="M38">
         <v>9</v>
@@ -73358,13 +73358,13 @@
         <v>9</v>
       </c>
       <c r="V38">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W38">
         <v>10</v>
       </c>
       <c r="X38">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y38">
         <v>10</v>
@@ -73399,7 +73399,7 @@
         <v>-1</v>
       </c>
       <c r="J39">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K39">
         <v>-1</v>
@@ -73435,7 +73435,7 @@
         <v>-1</v>
       </c>
       <c r="V39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W39">
         <v>-1</v>
@@ -73458,7 +73458,7 @@
         <v>8</v>
       </c>
       <c r="L40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="M40">
         <v>5</v>
@@ -73470,7 +73470,7 @@
         <v>-1</v>
       </c>
       <c r="X40">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y40">
         <v>7</v>
@@ -73741,7 +73741,7 @@
         <v>10</v>
       </c>
       <c r="L4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M4">
         <v>10</v>
@@ -73895,7 +73895,7 @@
         <v>10</v>
       </c>
       <c r="L6">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="M6">
         <v>8</v>
@@ -73931,7 +73931,7 @@
         <v>10</v>
       </c>
       <c r="X6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y6">
         <v>9</v>
@@ -73972,7 +73972,7 @@
         <v>8</v>
       </c>
       <c r="L7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M7">
         <v>7</v>
@@ -74049,7 +74049,7 @@
         <v>10</v>
       </c>
       <c r="L8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M8">
         <v>9</v>
@@ -74203,7 +74203,7 @@
         <v>10</v>
       </c>
       <c r="L10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M10">
         <v>10</v>
@@ -74280,7 +74280,7 @@
         <v>10</v>
       </c>
       <c r="L11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M11">
         <v>8</v>
@@ -74588,7 +74588,7 @@
         <v>10</v>
       </c>
       <c r="L15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M15">
         <v>8</v>
@@ -74665,7 +74665,7 @@
         <v>10</v>
       </c>
       <c r="L16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M16">
         <v>6</v>
@@ -74701,7 +74701,7 @@
         <v>10</v>
       </c>
       <c r="X16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y16">
         <v>7</v>
@@ -74973,7 +74973,7 @@
         <v>9</v>
       </c>
       <c r="L20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M20">
         <v>6</v>
@@ -75009,7 +75009,7 @@
         <v>9</v>
       </c>
       <c r="X20">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y20">
         <v>7</v>

</xml_diff>

<commit_message>
Segundo Parcial 14 noviembre
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -4351,7 +4351,7 @@
         <v>7</v>
       </c>
       <c r="C9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="D9">
         <v>8</v>
@@ -4369,7 +4369,7 @@
         <v>8</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J9">
         <v>6</v>
@@ -4405,7 +4405,7 @@
         <v>8</v>
       </c>
       <c r="U9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V9">
         <v>7</v>
@@ -4505,7 +4505,7 @@
         <v>7</v>
       </c>
       <c r="C11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D11">
         <v>5</v>
@@ -4523,7 +4523,7 @@
         <v>6</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J11">
         <v>5</v>
@@ -4559,7 +4559,7 @@
         <v>7</v>
       </c>
       <c r="U11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="V11">
         <v>5</v>
@@ -4659,7 +4659,7 @@
         <v>9</v>
       </c>
       <c r="C13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D13">
         <v>6</v>
@@ -4677,7 +4677,7 @@
         <v>6</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J13">
         <v>5</v>
@@ -4713,7 +4713,7 @@
         <v>8</v>
       </c>
       <c r="U13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V13">
         <v>5</v>
@@ -4736,7 +4736,7 @@
         <v>7</v>
       </c>
       <c r="C14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="D14">
         <v>6</v>
@@ -4754,7 +4754,7 @@
         <v>6</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J14">
         <v>5</v>
@@ -4790,7 +4790,7 @@
         <v>7</v>
       </c>
       <c r="U14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V14">
         <v>5</v>
@@ -4890,7 +4890,7 @@
         <v>7</v>
       </c>
       <c r="C16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="D16">
         <v>5</v>
@@ -4908,7 +4908,7 @@
         <v>6</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>5</v>
@@ -4944,7 +4944,7 @@
         <v>7</v>
       </c>
       <c r="U16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V16">
         <v>5</v>
@@ -5044,7 +5044,7 @@
         <v>7</v>
       </c>
       <c r="C18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D18">
         <v>5</v>
@@ -5062,7 +5062,7 @@
         <v>6</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J18">
         <v>6</v>
@@ -5098,7 +5098,7 @@
         <v>7</v>
       </c>
       <c r="U18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V18">
         <v>5</v>
@@ -5275,7 +5275,7 @@
         <v>7</v>
       </c>
       <c r="C21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="D21">
         <v>8</v>
@@ -5293,7 +5293,7 @@
         <v>7</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J21">
         <v>6</v>
@@ -5329,7 +5329,7 @@
         <v>7</v>
       </c>
       <c r="U21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V21">
         <v>7</v>
@@ -5506,7 +5506,7 @@
         <v>7</v>
       </c>
       <c r="C24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D24">
         <v>5</v>
@@ -5524,7 +5524,7 @@
         <v>6</v>
       </c>
       <c r="I24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J24">
         <v>5</v>
@@ -5560,7 +5560,7 @@
         <v>7</v>
       </c>
       <c r="U24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V24">
         <v>5</v>
@@ -5814,7 +5814,7 @@
         <v>7</v>
       </c>
       <c r="C28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D28">
         <v>6</v>
@@ -5832,7 +5832,7 @@
         <v>7</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J28">
         <v>6</v>
@@ -5868,7 +5868,7 @@
         <v>7</v>
       </c>
       <c r="U28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V28">
         <v>6</v>
@@ -6199,7 +6199,7 @@
         <v>6</v>
       </c>
       <c r="C33">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D33">
         <v>5</v>
@@ -6217,7 +6217,7 @@
         <v>9</v>
       </c>
       <c r="I33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J33">
         <v>6</v>
@@ -6253,7 +6253,7 @@
         <v>8</v>
       </c>
       <c r="U33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V33">
         <v>5</v>
@@ -6430,7 +6430,7 @@
         <v>8</v>
       </c>
       <c r="C36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D36">
         <v>5</v>
@@ -6448,7 +6448,7 @@
         <v>7</v>
       </c>
       <c r="I36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J36">
         <v>5</v>
@@ -6484,7 +6484,7 @@
         <v>8</v>
       </c>
       <c r="U36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V36">
         <v>5</v>
@@ -24893,7 +24893,7 @@
         <v>6</v>
       </c>
       <c r="C23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D23">
         <v>5</v>
@@ -24911,7 +24911,7 @@
         <v>6</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J23">
         <v>6</v>
@@ -24947,7 +24947,7 @@
         <v>6</v>
       </c>
       <c r="U23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V23">
         <v>5</v>
@@ -25201,7 +25201,7 @@
         <v>5</v>
       </c>
       <c r="C27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D27">
         <v>6</v>
@@ -25219,7 +25219,7 @@
         <v>6</v>
       </c>
       <c r="I27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J27">
         <v>6</v>
@@ -25255,7 +25255,7 @@
         <v>5</v>
       </c>
       <c r="U27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="V27">
         <v>6</v>
@@ -29151,7 +29151,7 @@
         <v>6</v>
       </c>
       <c r="D4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E4">
         <v>4</v>
@@ -29169,7 +29169,7 @@
         <v>9</v>
       </c>
       <c r="J4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K4">
         <v>7</v>
@@ -29205,7 +29205,7 @@
         <v>8</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W4">
         <v>5</v>
@@ -29305,7 +29305,7 @@
         <v>7</v>
       </c>
       <c r="D6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E6">
         <v>7</v>
@@ -29323,7 +29323,7 @@
         <v>9</v>
       </c>
       <c r="J6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K6">
         <v>9</v>
@@ -29359,7 +29359,7 @@
         <v>8</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>8</v>
@@ -29921,7 +29921,7 @@
         <v>7</v>
       </c>
       <c r="D14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E14">
         <v>6</v>
@@ -29939,7 +29939,7 @@
         <v>9</v>
       </c>
       <c r="J14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K14">
         <v>9</v>
@@ -29975,7 +29975,7 @@
         <v>8</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W14">
         <v>8</v>
@@ -29998,7 +29998,7 @@
         <v>5</v>
       </c>
       <c r="D15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E15">
         <v>6</v>
@@ -30016,7 +30016,7 @@
         <v>8</v>
       </c>
       <c r="J15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K15">
         <v>7</v>
@@ -30052,7 +30052,7 @@
         <v>7</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W15">
         <v>7</v>
@@ -30152,7 +30152,7 @@
         <v>7</v>
       </c>
       <c r="D17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E17">
         <v>4</v>
@@ -30170,7 +30170,7 @@
         <v>7</v>
       </c>
       <c r="J17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K17">
         <v>6</v>
@@ -30206,7 +30206,7 @@
         <v>7</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W17">
         <v>5</v>
@@ -30306,7 +30306,7 @@
         <v>7</v>
       </c>
       <c r="D19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E19">
         <v>6</v>
@@ -30324,7 +30324,7 @@
         <v>5</v>
       </c>
       <c r="J19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K19">
         <v>7</v>
@@ -30360,7 +30360,7 @@
         <v>6</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W19">
         <v>7</v>
@@ -30460,7 +30460,7 @@
         <v>7</v>
       </c>
       <c r="D21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E21">
         <v>4</v>
@@ -30478,7 +30478,7 @@
         <v>6</v>
       </c>
       <c r="J21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K21">
         <v>6</v>
@@ -30514,7 +30514,7 @@
         <v>7</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W21">
         <v>5</v>
@@ -30768,7 +30768,7 @@
         <v>7</v>
       </c>
       <c r="D25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E25">
         <v>8</v>
@@ -30786,7 +30786,7 @@
         <v>5</v>
       </c>
       <c r="J25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K25">
         <v>9</v>
@@ -30822,7 +30822,7 @@
         <v>6</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W25">
         <v>9</v>
@@ -30922,7 +30922,7 @@
         <v>8</v>
       </c>
       <c r="D27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E27">
         <v>4</v>
@@ -30940,7 +30940,7 @@
         <v>6</v>
       </c>
       <c r="J27">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K27">
         <v>6</v>
@@ -30976,7 +30976,7 @@
         <v>7</v>
       </c>
       <c r="V27">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W27">
         <v>5</v>
@@ -30999,7 +30999,7 @@
         <v>6</v>
       </c>
       <c r="D28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="E28">
         <v>6</v>
@@ -31017,7 +31017,7 @@
         <v>5</v>
       </c>
       <c r="J28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K28">
         <v>7</v>
@@ -31053,7 +31053,7 @@
         <v>5</v>
       </c>
       <c r="V28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W28">
         <v>7</v>
@@ -37256,7 +37256,7 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D4">
         <v>7</v>
@@ -37274,7 +37274,7 @@
         <v>5</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J4">
         <v>6</v>
@@ -37310,7 +37310,7 @@
         <v>5</v>
       </c>
       <c r="U4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V4">
         <v>7</v>
@@ -37641,7 +37641,7 @@
         <v>6</v>
       </c>
       <c r="C9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="D9">
         <v>6</v>
@@ -37659,7 +37659,7 @@
         <v>8</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J9">
         <v>8</v>
@@ -37695,7 +37695,7 @@
         <v>7</v>
       </c>
       <c r="U9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="V9">
         <v>7</v>
@@ -37795,7 +37795,7 @@
         <v>5</v>
       </c>
       <c r="C11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D11">
         <v>6</v>
@@ -37813,7 +37813,7 @@
         <v>5</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J11">
         <v>4</v>
@@ -37849,7 +37849,7 @@
         <v>5</v>
       </c>
       <c r="U11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V11">
         <v>5</v>
@@ -37872,7 +37872,7 @@
         <v>7</v>
       </c>
       <c r="C12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D12">
         <v>7</v>
@@ -37890,7 +37890,7 @@
         <v>6</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J12">
         <v>8</v>
@@ -37926,7 +37926,7 @@
         <v>7</v>
       </c>
       <c r="U12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V12">
         <v>8</v>
@@ -38026,7 +38026,7 @@
         <v>-1</v>
       </c>
       <c r="C14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D14">
         <v>7</v>
@@ -38044,7 +38044,7 @@
         <v>-1</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -38080,7 +38080,7 @@
         <v>-1</v>
       </c>
       <c r="U14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V14">
         <v>5</v>
@@ -38180,7 +38180,7 @@
         <v>6</v>
       </c>
       <c r="C16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="D16">
         <v>4</v>
@@ -38198,7 +38198,7 @@
         <v>6</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J16">
         <v>7</v>
@@ -38234,7 +38234,7 @@
         <v>6</v>
       </c>
       <c r="U16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V16">
         <v>5</v>
@@ -38257,7 +38257,7 @@
         <v>5</v>
       </c>
       <c r="C17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D17">
         <v>8</v>
@@ -38275,7 +38275,7 @@
         <v>5</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J17">
         <v>4</v>
@@ -38311,7 +38311,7 @@
         <v>5</v>
       </c>
       <c r="U17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V17">
         <v>6</v>
@@ -38488,7 +38488,7 @@
         <v>6</v>
       </c>
       <c r="C20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D20">
         <v>7</v>
@@ -38506,7 +38506,7 @@
         <v>6</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J20">
         <v>5</v>
@@ -38542,7 +38542,7 @@
         <v>6</v>
       </c>
       <c r="U20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V20">
         <v>6</v>
@@ -38642,7 +38642,7 @@
         <v>8</v>
       </c>
       <c r="C22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="D22">
         <v>8</v>
@@ -38660,7 +38660,7 @@
         <v>6</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J22">
         <v>9</v>
@@ -38696,7 +38696,7 @@
         <v>7</v>
       </c>
       <c r="U22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V22">
         <v>9</v>
@@ -38719,7 +38719,7 @@
         <v>5</v>
       </c>
       <c r="C23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D23">
         <v>8</v>
@@ -38737,7 +38737,7 @@
         <v>6</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J23">
         <v>7</v>
@@ -38773,7 +38773,7 @@
         <v>5</v>
       </c>
       <c r="U23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V23">
         <v>8</v>
@@ -39566,7 +39566,7 @@
         <v>5</v>
       </c>
       <c r="C34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D34">
         <v>7</v>
@@ -39584,7 +39584,7 @@
         <v>5</v>
       </c>
       <c r="I34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J34">
         <v>5</v>
@@ -39620,7 +39620,7 @@
         <v>5</v>
       </c>
       <c r="U34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V34">
         <v>6</v>
@@ -39797,7 +39797,7 @@
         <v>6</v>
       </c>
       <c r="C37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="D37">
         <v>6</v>
@@ -39815,7 +39815,7 @@
         <v>6</v>
       </c>
       <c r="I37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J37">
         <v>8</v>
@@ -39851,7 +39851,7 @@
         <v>6</v>
       </c>
       <c r="U37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V37">
         <v>7</v>
@@ -49672,7 +49672,7 @@
         <v>863</v>
       </c>
       <c r="B9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="C9">
         <v>6</v>
@@ -49690,7 +49690,7 @@
         <v>5</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I9">
         <v>5</v>
@@ -49726,7 +49726,7 @@
         <v>-1</v>
       </c>
       <c r="T9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="U9">
         <v>5</v>
@@ -51075,7 +51075,7 @@
         <v>882</v>
       </c>
       <c r="B28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="E28">
         <v>5</v>
@@ -51084,7 +51084,7 @@
         <v>5</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="K28">
         <v>5</v>
@@ -51102,7 +51102,7 @@
         <v>-1</v>
       </c>
       <c r="T28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W28">
         <v>5</v>
@@ -51193,7 +51193,7 @@
         <v>884</v>
       </c>
       <c r="B30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="C30">
         <v>5</v>
@@ -51211,7 +51211,7 @@
         <v>5</v>
       </c>
       <c r="H30">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="I30">
         <v>5</v>
@@ -51247,7 +51247,7 @@
         <v>-1</v>
       </c>
       <c r="T30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="U30">
         <v>5</v>
@@ -52397,7 +52397,7 @@
         <v>5</v>
       </c>
       <c r="E5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -52415,7 +52415,7 @@
         <v>5</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -52451,7 +52451,7 @@
         <v>5</v>
       </c>
       <c r="W5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="X5">
         <v>5</v>
@@ -55417,7 +55417,7 @@
         <v>6</v>
       </c>
       <c r="G4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="H4">
         <v>7</v>
@@ -55435,7 +55435,7 @@
         <v>6</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -55471,7 +55471,7 @@
         <v>6</v>
       </c>
       <c r="Y4">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -55482,7 +55482,7 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D5">
         <v>6</v>
@@ -55494,13 +55494,13 @@
         <v>5</v>
       </c>
       <c r="G5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H5">
         <v>7</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J5">
         <v>6</v>
@@ -55512,7 +55512,7 @@
         <v>5</v>
       </c>
       <c r="M5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N5">
         <v>-1</v>
@@ -55536,7 +55536,7 @@
         <v>7</v>
       </c>
       <c r="U5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V5">
         <v>6</v>
@@ -55548,7 +55548,7 @@
         <v>5</v>
       </c>
       <c r="Y5">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -55636,7 +55636,7 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D7">
         <v>6</v>
@@ -55654,7 +55654,7 @@
         <v>7</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J7">
         <v>8</v>
@@ -55690,7 +55690,7 @@
         <v>7</v>
       </c>
       <c r="U7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V7">
         <v>7</v>
@@ -55713,7 +55713,7 @@
         <v>5</v>
       </c>
       <c r="C8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -55725,13 +55725,13 @@
         <v>5</v>
       </c>
       <c r="G8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H8">
         <v>5</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J8">
         <v>5</v>
@@ -55743,7 +55743,7 @@
         <v>5</v>
       </c>
       <c r="M8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -55767,7 +55767,7 @@
         <v>5</v>
       </c>
       <c r="U8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V8">
         <v>5</v>
@@ -55779,7 +55779,7 @@
         <v>5</v>
       </c>
       <c r="Y8">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -56021,7 +56021,7 @@
         <v>6</v>
       </c>
       <c r="C12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D12">
         <v>5</v>
@@ -56033,13 +56033,13 @@
         <v>6</v>
       </c>
       <c r="G12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="H12">
         <v>7</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J12">
         <v>8</v>
@@ -56051,7 +56051,7 @@
         <v>6</v>
       </c>
       <c r="M12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N12">
         <v>-1</v>
@@ -56075,7 +56075,7 @@
         <v>7</v>
       </c>
       <c r="U12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V12">
         <v>7</v>
@@ -56087,7 +56087,7 @@
         <v>6</v>
       </c>
       <c r="Y12">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -56175,7 +56175,7 @@
         <v>6</v>
       </c>
       <c r="C14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D14">
         <v>7</v>
@@ -56187,13 +56187,13 @@
         <v>6</v>
       </c>
       <c r="G14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="H14">
         <v>7</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J14">
         <v>8</v>
@@ -56205,7 +56205,7 @@
         <v>5</v>
       </c>
       <c r="M14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -56229,7 +56229,7 @@
         <v>7</v>
       </c>
       <c r="U14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="V14">
         <v>8</v>
@@ -56241,7 +56241,7 @@
         <v>5</v>
       </c>
       <c r="Y14">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -56329,7 +56329,7 @@
         <v>6</v>
       </c>
       <c r="C16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D16">
         <v>5</v>
@@ -56341,13 +56341,13 @@
         <v>5</v>
       </c>
       <c r="G16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H16">
         <v>7</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J16">
         <v>9</v>
@@ -56359,7 +56359,7 @@
         <v>5</v>
       </c>
       <c r="M16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N16">
         <v>-1</v>
@@ -56383,7 +56383,7 @@
         <v>7</v>
       </c>
       <c r="U16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V16">
         <v>7</v>
@@ -56395,7 +56395,7 @@
         <v>5</v>
       </c>
       <c r="Y16">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:25">
@@ -56560,7 +56560,7 @@
         <v>6</v>
       </c>
       <c r="C19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D19">
         <v>7</v>
@@ -56572,13 +56572,13 @@
         <v>8</v>
       </c>
       <c r="G19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="H19">
         <v>7</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J19">
         <v>5</v>
@@ -56590,7 +56590,7 @@
         <v>5</v>
       </c>
       <c r="M19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N19">
         <v>-1</v>
@@ -56614,7 +56614,7 @@
         <v>7</v>
       </c>
       <c r="U19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V19">
         <v>6</v>
@@ -56626,7 +56626,7 @@
         <v>7</v>
       </c>
       <c r="Y19">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:25">
@@ -56637,7 +56637,7 @@
         <v>6</v>
       </c>
       <c r="C20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D20">
         <v>9</v>
@@ -56649,13 +56649,13 @@
         <v>7</v>
       </c>
       <c r="G20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H20">
         <v>7</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J20">
         <v>6</v>
@@ -56667,7 +56667,7 @@
         <v>5</v>
       </c>
       <c r="M20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N20">
         <v>-1</v>
@@ -56691,7 +56691,7 @@
         <v>7</v>
       </c>
       <c r="U20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V20">
         <v>8</v>
@@ -56703,7 +56703,7 @@
         <v>6</v>
       </c>
       <c r="Y20">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:25">
@@ -56714,7 +56714,7 @@
         <v>6</v>
       </c>
       <c r="C21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="D21">
         <v>8</v>
@@ -56726,13 +56726,13 @@
         <v>6</v>
       </c>
       <c r="G21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H21">
         <v>7</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J21">
         <v>6</v>
@@ -56744,7 +56744,7 @@
         <v>5</v>
       </c>
       <c r="M21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N21">
         <v>-1</v>
@@ -56768,7 +56768,7 @@
         <v>7</v>
       </c>
       <c r="U21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V21">
         <v>7</v>
@@ -56780,7 +56780,7 @@
         <v>5</v>
       </c>
       <c r="Y21">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:25">
@@ -57169,7 +57169,7 @@
         <v>6</v>
       </c>
       <c r="G28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="H28">
         <v>7</v>
@@ -57187,7 +57187,7 @@
         <v>6</v>
       </c>
       <c r="M28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N28">
         <v>-1</v>
@@ -57223,7 +57223,7 @@
         <v>6</v>
       </c>
       <c r="Y28">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -57246,7 +57246,7 @@
         <v>6</v>
       </c>
       <c r="G29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H29">
         <v>6</v>
@@ -57264,7 +57264,7 @@
         <v>5</v>
       </c>
       <c r="M29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="N29">
         <v>-1</v>
@@ -57300,7 +57300,7 @@
         <v>5</v>
       </c>
       <c r="Y29">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:25">
@@ -57323,7 +57323,7 @@
         <v>5</v>
       </c>
       <c r="G30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H30">
         <v>5</v>
@@ -57341,7 +57341,7 @@
         <v>5</v>
       </c>
       <c r="M30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N30">
         <v>-1</v>
@@ -57377,7 +57377,7 @@
         <v>5</v>
       </c>
       <c r="Y30">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -60136,7 +60136,7 @@
         <v>6</v>
       </c>
       <c r="G4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H4">
         <v>7</v>
@@ -60154,7 +60154,7 @@
         <v>8</v>
       </c>
       <c r="M4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N4">
         <v>-1</v>
@@ -60190,7 +60190,7 @@
         <v>7</v>
       </c>
       <c r="Y4">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -60367,7 +60367,7 @@
         <v>9</v>
       </c>
       <c r="G7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H7">
         <v>9</v>
@@ -60385,7 +60385,7 @@
         <v>10</v>
       </c>
       <c r="M7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="N7">
         <v>-1</v>
@@ -60421,7 +60421,7 @@
         <v>10</v>
       </c>
       <c r="Y7">
-        <v>-1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -60521,7 +60521,7 @@
         <v>10</v>
       </c>
       <c r="G9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H9">
         <v>7</v>
@@ -60539,7 +60539,7 @@
         <v>8</v>
       </c>
       <c r="M9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="N9">
         <v>-1</v>
@@ -60575,7 +60575,7 @@
         <v>9</v>
       </c>
       <c r="Y9">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -60829,7 +60829,7 @@
         <v>8</v>
       </c>
       <c r="G13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H13">
         <v>7</v>
@@ -60847,7 +60847,7 @@
         <v>6</v>
       </c>
       <c r="M13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N13">
         <v>-1</v>
@@ -60883,7 +60883,7 @@
         <v>7</v>
       </c>
       <c r="Y13">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -60906,7 +60906,7 @@
         <v>6</v>
       </c>
       <c r="G14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H14">
         <v>7</v>
@@ -60924,7 +60924,7 @@
         <v>6</v>
       </c>
       <c r="M14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -60960,7 +60960,7 @@
         <v>6</v>
       </c>
       <c r="Y14">
-        <v>-1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -61137,7 +61137,7 @@
         <v>6</v>
       </c>
       <c r="G17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H17">
         <v>8</v>
@@ -61155,7 +61155,7 @@
         <v>5</v>
       </c>
       <c r="M17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="N17">
         <v>-1</v>
@@ -61191,7 +61191,7 @@
         <v>5</v>
       </c>
       <c r="Y17">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:25">
@@ -69501,7 +69501,7 @@
         <v>5</v>
       </c>
       <c r="E7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="F7">
         <v>5</v>
@@ -69519,7 +69519,7 @@
         <v>5</v>
       </c>
       <c r="K7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -69555,7 +69555,7 @@
         <v>5</v>
       </c>
       <c r="W7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="X7">
         <v>5</v>

</xml_diff>

<commit_message>
7 dic noche 2
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -12436,7 +12436,7 @@
         <v>10</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T4">
         <v>9</v>
@@ -12454,7 +12454,7 @@
         <v>8</v>
       </c>
       <c r="Y4">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -12513,7 +12513,7 @@
         <v>6</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T5">
         <v>9</v>
@@ -12531,7 +12531,7 @@
         <v>7</v>
       </c>
       <c r="Y5">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -12590,7 +12590,7 @@
         <v>9</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T6">
         <v>10</v>
@@ -12608,7 +12608,7 @@
         <v>9</v>
       </c>
       <c r="Y6">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -12667,7 +12667,7 @@
         <v>8</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T7">
         <v>9</v>
@@ -12744,7 +12744,7 @@
         <v>9</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T8">
         <v>9</v>
@@ -12821,7 +12821,7 @@
         <v>10</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T9">
         <v>10</v>
@@ -12898,7 +12898,7 @@
         <v>5</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T10">
         <v>5</v>
@@ -12975,7 +12975,7 @@
         <v>10</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T11">
         <v>10</v>
@@ -13052,7 +13052,7 @@
         <v>8</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T12">
         <v>8</v>
@@ -13070,7 +13070,7 @@
         <v>8</v>
       </c>
       <c r="Y12">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -13129,7 +13129,7 @@
         <v>9</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T13">
         <v>8</v>
@@ -13147,7 +13147,7 @@
         <v>8</v>
       </c>
       <c r="Y13">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -13206,7 +13206,7 @@
         <v>7</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T14">
         <v>10</v>
@@ -13224,7 +13224,7 @@
         <v>8</v>
       </c>
       <c r="Y14">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -13283,7 +13283,7 @@
         <v>8</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T15">
         <v>10</v>
@@ -13360,7 +13360,7 @@
         <v>7</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T16">
         <v>7</v>
@@ -13437,7 +13437,7 @@
         <v>10</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T17">
         <v>10</v>
@@ -13514,7 +13514,7 @@
         <v>7</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T18">
         <v>10</v>
@@ -13591,7 +13591,7 @@
         <v>8</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T19">
         <v>9</v>
@@ -13668,7 +13668,7 @@
         <v>7</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T20">
         <v>9</v>
@@ -13745,7 +13745,7 @@
         <v>7</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T21">
         <v>8</v>
@@ -13822,7 +13822,7 @@
         <v>7</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T22">
         <v>9</v>
@@ -13899,7 +13899,7 @@
         <v>9</v>
       </c>
       <c r="S23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T23">
         <v>7</v>
@@ -13917,7 +13917,7 @@
         <v>7</v>
       </c>
       <c r="Y23">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:25">
@@ -13976,7 +13976,7 @@
         <v>9</v>
       </c>
       <c r="S24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T24">
         <v>10</v>
@@ -13994,7 +13994,7 @@
         <v>8</v>
       </c>
       <c r="Y24">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -14053,7 +14053,7 @@
         <v>6</v>
       </c>
       <c r="S25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T25">
         <v>9</v>
@@ -14130,7 +14130,7 @@
         <v>9</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T26">
         <v>9</v>
@@ -14148,7 +14148,7 @@
         <v>9</v>
       </c>
       <c r="Y26">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:25">
@@ -14236,7 +14236,7 @@
         <v>10</v>
       </c>
       <c r="S28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T28">
         <v>7</v>
@@ -14254,7 +14254,7 @@
         <v>10</v>
       </c>
       <c r="Y28">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -14313,7 +14313,7 @@
         <v>7</v>
       </c>
       <c r="S29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T29">
         <v>7</v>
@@ -14390,7 +14390,7 @@
         <v>5</v>
       </c>
       <c r="S30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T30">
         <v>8</v>
@@ -14467,7 +14467,7 @@
         <v>7</v>
       </c>
       <c r="S31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T31">
         <v>10</v>
@@ -14544,7 +14544,7 @@
         <v>6</v>
       </c>
       <c r="S32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T32">
         <v>10</v>
@@ -14621,7 +14621,7 @@
         <v>7</v>
       </c>
       <c r="S33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T33">
         <v>9</v>
@@ -14698,7 +14698,7 @@
         <v>8</v>
       </c>
       <c r="S34">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T34">
         <v>9</v>
@@ -14775,7 +14775,7 @@
         <v>10</v>
       </c>
       <c r="S35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T35">
         <v>10</v>
@@ -14852,7 +14852,7 @@
         <v>8</v>
       </c>
       <c r="S36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T36">
         <v>9</v>
@@ -14929,7 +14929,7 @@
         <v>10</v>
       </c>
       <c r="S37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T37">
         <v>10</v>
@@ -15006,7 +15006,7 @@
         <v>7</v>
       </c>
       <c r="S38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T38">
         <v>10</v>
@@ -15083,7 +15083,7 @@
         <v>6</v>
       </c>
       <c r="S39">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T39">
         <v>8</v>
@@ -15101,7 +15101,7 @@
         <v>7</v>
       </c>
       <c r="Y39">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:25">
@@ -15160,7 +15160,7 @@
         <v>10</v>
       </c>
       <c r="S40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T40">
         <v>10</v>
@@ -15237,7 +15237,7 @@
         <v>7</v>
       </c>
       <c r="S41">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T41">
         <v>10</v>
@@ -15255,7 +15255,7 @@
         <v>7</v>
       </c>
       <c r="Y41">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:25">
@@ -15314,7 +15314,7 @@
         <v>6</v>
       </c>
       <c r="S42">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T42">
         <v>5</v>
@@ -15391,7 +15391,7 @@
         <v>7</v>
       </c>
       <c r="S43">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T43">
         <v>8</v>
@@ -15409,7 +15409,7 @@
         <v>6</v>
       </c>
       <c r="Y43">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:25">
@@ -15468,7 +15468,7 @@
         <v>7</v>
       </c>
       <c r="S44">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T44">
         <v>10</v>
@@ -15486,7 +15486,7 @@
         <v>7</v>
       </c>
       <c r="Y44">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45" spans="1:25">
@@ -15545,7 +15545,7 @@
         <v>9</v>
       </c>
       <c r="S45">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T45">
         <v>10</v>
@@ -15563,7 +15563,7 @@
         <v>9</v>
       </c>
       <c r="Y45">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46" spans="1:25">
@@ -15622,7 +15622,7 @@
         <v>9</v>
       </c>
       <c r="S46">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T46">
         <v>9</v>
@@ -15699,7 +15699,7 @@
         <v>8</v>
       </c>
       <c r="S47">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T47">
         <v>9</v>
@@ -15776,7 +15776,7 @@
         <v>9</v>
       </c>
       <c r="S48">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T48">
         <v>9</v>
@@ -37295,7 +37295,7 @@
         <v>5</v>
       </c>
       <c r="N4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O4">
         <v>7</v>
@@ -37310,10 +37310,10 @@
         <v>7</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U4">
         <v>6</v>
@@ -37372,7 +37372,7 @@
         <v>6</v>
       </c>
       <c r="N5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O5">
         <v>7</v>
@@ -37387,10 +37387,10 @@
         <v>9</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U5">
         <v>7</v>
@@ -37405,7 +37405,7 @@
         <v>8</v>
       </c>
       <c r="Y5">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -37449,7 +37449,7 @@
         <v>8</v>
       </c>
       <c r="N6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O6">
         <v>10</v>
@@ -37464,7 +37464,7 @@
         <v>10</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T6">
         <v>8</v>
@@ -37526,7 +37526,7 @@
         <v>6</v>
       </c>
       <c r="N7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O7">
         <v>10</v>
@@ -37541,7 +37541,7 @@
         <v>9</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T7">
         <v>7</v>
@@ -37559,7 +37559,7 @@
         <v>7</v>
       </c>
       <c r="Y7">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -37603,7 +37603,7 @@
         <v>10</v>
       </c>
       <c r="N8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O8">
         <v>8</v>
@@ -37618,7 +37618,7 @@
         <v>10</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T8">
         <v>9</v>
@@ -37680,7 +37680,7 @@
         <v>5</v>
       </c>
       <c r="N9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O9">
         <v>8</v>
@@ -37695,10 +37695,10 @@
         <v>8</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U9">
         <v>8</v>
@@ -37713,7 +37713,7 @@
         <v>7</v>
       </c>
       <c r="Y9">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -37757,7 +37757,7 @@
         <v>6</v>
       </c>
       <c r="N10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O10">
         <v>10</v>
@@ -37772,7 +37772,7 @@
         <v>10</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T10">
         <v>7</v>
@@ -37790,7 +37790,7 @@
         <v>9</v>
       </c>
       <c r="Y10">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -37834,7 +37834,7 @@
         <v>5</v>
       </c>
       <c r="N11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O11">
         <v>10</v>
@@ -37849,10 +37849,10 @@
         <v>8</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U11">
         <v>7</v>
@@ -37867,7 +37867,7 @@
         <v>7</v>
       </c>
       <c r="Y11">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -37911,7 +37911,7 @@
         <v>6</v>
       </c>
       <c r="N12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O12">
         <v>9</v>
@@ -37926,7 +37926,7 @@
         <v>8</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T12">
         <v>7</v>
@@ -37988,7 +37988,7 @@
         <v>10</v>
       </c>
       <c r="N13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O13">
         <v>10</v>
@@ -38003,7 +38003,7 @@
         <v>10</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T13">
         <v>8</v>
@@ -38080,7 +38080,7 @@
         <v>5</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T14">
         <v>-1</v>
@@ -38142,7 +38142,7 @@
         <v>6</v>
       </c>
       <c r="N15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O15">
         <v>9</v>
@@ -38157,10 +38157,10 @@
         <v>9</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T15">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U15">
         <v>9</v>
@@ -38219,7 +38219,7 @@
         <v>6</v>
       </c>
       <c r="N16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O16">
         <v>9</v>
@@ -38234,7 +38234,7 @@
         <v>9</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T16">
         <v>6</v>
@@ -38252,7 +38252,7 @@
         <v>7</v>
       </c>
       <c r="Y16">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:25">
@@ -38296,7 +38296,7 @@
         <v>5</v>
       </c>
       <c r="N17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O17">
         <v>5</v>
@@ -38311,10 +38311,10 @@
         <v>9</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U17">
         <v>5</v>
@@ -38373,7 +38373,7 @@
         <v>6</v>
       </c>
       <c r="N18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O18">
         <v>7</v>
@@ -38388,10 +38388,10 @@
         <v>9</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U18">
         <v>8</v>
@@ -38450,7 +38450,7 @@
         <v>9</v>
       </c>
       <c r="N19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O19">
         <v>8</v>
@@ -38465,7 +38465,7 @@
         <v>9</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T19">
         <v>7</v>
@@ -38483,7 +38483,7 @@
         <v>8</v>
       </c>
       <c r="Y19">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:25">
@@ -38527,7 +38527,7 @@
         <v>5</v>
       </c>
       <c r="N20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O20">
         <v>7</v>
@@ -38542,10 +38542,10 @@
         <v>10</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T20">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U20">
         <v>7</v>
@@ -38560,7 +38560,7 @@
         <v>9</v>
       </c>
       <c r="Y20">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:25">
@@ -38604,7 +38604,7 @@
         <v>6</v>
       </c>
       <c r="N21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O21">
         <v>9</v>
@@ -38619,10 +38619,10 @@
         <v>8</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T21">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U21">
         <v>7</v>
@@ -38637,7 +38637,7 @@
         <v>7</v>
       </c>
       <c r="Y21">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:25">
@@ -38681,7 +38681,7 @@
         <v>8</v>
       </c>
       <c r="N22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O22">
         <v>8</v>
@@ -38696,10 +38696,10 @@
         <v>10</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U22">
         <v>9</v>
@@ -38758,7 +38758,7 @@
         <v>5</v>
       </c>
       <c r="N23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O23">
         <v>6</v>
@@ -38773,10 +38773,10 @@
         <v>7</v>
       </c>
       <c r="S23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U23">
         <v>6</v>
@@ -38835,7 +38835,7 @@
         <v>8</v>
       </c>
       <c r="N24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O24">
         <v>9</v>
@@ -38850,7 +38850,7 @@
         <v>10</v>
       </c>
       <c r="S24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T24">
         <v>9</v>
@@ -38868,7 +38868,7 @@
         <v>10</v>
       </c>
       <c r="Y24">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -38912,7 +38912,7 @@
         <v>5</v>
       </c>
       <c r="N25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O25">
         <v>8</v>
@@ -38927,10 +38927,10 @@
         <v>8</v>
       </c>
       <c r="S25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U25">
         <v>7</v>
@@ -38989,7 +38989,7 @@
         <v>8</v>
       </c>
       <c r="N26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O26">
         <v>8</v>
@@ -39004,7 +39004,7 @@
         <v>7</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T26">
         <v>7</v>
@@ -39066,7 +39066,7 @@
         <v>6</v>
       </c>
       <c r="N27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O27">
         <v>8</v>
@@ -39081,10 +39081,10 @@
         <v>8</v>
       </c>
       <c r="S27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T27">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U27">
         <v>8</v>
@@ -39099,7 +39099,7 @@
         <v>8</v>
       </c>
       <c r="Y27">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:25">
@@ -39143,7 +39143,7 @@
         <v>6</v>
       </c>
       <c r="N28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O28">
         <v>7</v>
@@ -39158,7 +39158,7 @@
         <v>8</v>
       </c>
       <c r="S28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T28">
         <v>7</v>
@@ -39176,7 +39176,7 @@
         <v>8</v>
       </c>
       <c r="Y28">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -39220,7 +39220,7 @@
         <v>8</v>
       </c>
       <c r="N29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O29">
         <v>10</v>
@@ -39235,7 +39235,7 @@
         <v>10</v>
       </c>
       <c r="S29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T29">
         <v>9</v>
@@ -39297,7 +39297,7 @@
         <v>8</v>
       </c>
       <c r="N30">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O30">
         <v>9</v>
@@ -39312,7 +39312,7 @@
         <v>10</v>
       </c>
       <c r="S30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T30">
         <v>6</v>
@@ -39374,7 +39374,7 @@
         <v>5</v>
       </c>
       <c r="N31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O31">
         <v>7</v>
@@ -39389,7 +39389,7 @@
         <v>7</v>
       </c>
       <c r="S31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T31">
         <v>6</v>
@@ -39407,7 +39407,7 @@
         <v>7</v>
       </c>
       <c r="Y31">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:25">
@@ -39451,7 +39451,7 @@
         <v>9</v>
       </c>
       <c r="N32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O32">
         <v>10</v>
@@ -39466,10 +39466,10 @@
         <v>10</v>
       </c>
       <c r="S32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T32">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U32">
         <v>10</v>
@@ -39484,7 +39484,7 @@
         <v>8</v>
       </c>
       <c r="Y32">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:25">
@@ -39528,7 +39528,7 @@
         <v>9</v>
       </c>
       <c r="N33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O33">
         <v>10</v>
@@ -39543,7 +39543,7 @@
         <v>10</v>
       </c>
       <c r="S33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T33">
         <v>9</v>
@@ -39561,7 +39561,7 @@
         <v>10</v>
       </c>
       <c r="Y33">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:25">
@@ -39605,7 +39605,7 @@
         <v>5</v>
       </c>
       <c r="N34">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O34">
         <v>7</v>
@@ -39620,10 +39620,10 @@
         <v>9</v>
       </c>
       <c r="S34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T34">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U34">
         <v>6</v>
@@ -39682,7 +39682,7 @@
         <v>7</v>
       </c>
       <c r="N35">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O35">
         <v>10</v>
@@ -39697,7 +39697,7 @@
         <v>10</v>
       </c>
       <c r="S35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T35">
         <v>10</v>
@@ -39759,7 +39759,7 @@
         <v>9</v>
       </c>
       <c r="N36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O36">
         <v>8</v>
@@ -39774,7 +39774,7 @@
         <v>10</v>
       </c>
       <c r="S36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T36">
         <v>8</v>
@@ -39836,7 +39836,7 @@
         <v>6</v>
       </c>
       <c r="N37">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O37">
         <v>8</v>
@@ -39851,7 +39851,7 @@
         <v>8</v>
       </c>
       <c r="S37">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T37">
         <v>6</v>
@@ -55456,7 +55456,7 @@
         <v>6</v>
       </c>
       <c r="R4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S4">
         <v>8</v>
@@ -55474,7 +55474,7 @@
         <v>6</v>
       </c>
       <c r="X4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y4">
         <v>7</v>
@@ -55533,7 +55533,7 @@
         <v>5</v>
       </c>
       <c r="R5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S5">
         <v>5</v>
@@ -55551,7 +55551,7 @@
         <v>5</v>
       </c>
       <c r="X5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y5">
         <v>5</v>
@@ -55610,7 +55610,7 @@
         <v>7</v>
       </c>
       <c r="R6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S6">
         <v>6</v>
@@ -55687,7 +55687,7 @@
         <v>7</v>
       </c>
       <c r="R7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S7">
         <v>6</v>
@@ -55764,7 +55764,7 @@
         <v>5</v>
       </c>
       <c r="R8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S8">
         <v>5</v>
@@ -55841,7 +55841,7 @@
         <v>10</v>
       </c>
       <c r="R9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S9">
         <v>10</v>
@@ -55918,7 +55918,7 @@
         <v>9</v>
       </c>
       <c r="R10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S10">
         <v>6</v>
@@ -55936,7 +55936,7 @@
         <v>7</v>
       </c>
       <c r="X10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y10">
         <v>8</v>
@@ -55995,7 +55995,7 @@
         <v>9</v>
       </c>
       <c r="R11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S11">
         <v>10</v>
@@ -56072,7 +56072,7 @@
         <v>8</v>
       </c>
       <c r="R12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S12">
         <v>6</v>
@@ -56149,7 +56149,7 @@
         <v>8</v>
       </c>
       <c r="R13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S13">
         <v>8</v>
@@ -56226,7 +56226,7 @@
         <v>8</v>
       </c>
       <c r="R14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S14">
         <v>6</v>
@@ -56244,7 +56244,7 @@
         <v>6</v>
       </c>
       <c r="X14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y14">
         <v>6</v>
@@ -56303,7 +56303,7 @@
         <v>7</v>
       </c>
       <c r="R15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S15">
         <v>10</v>
@@ -56380,7 +56380,7 @@
         <v>6</v>
       </c>
       <c r="R16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S16">
         <v>8</v>
@@ -56398,7 +56398,7 @@
         <v>5</v>
       </c>
       <c r="X16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y16">
         <v>6</v>
@@ -56457,7 +56457,7 @@
         <v>6</v>
       </c>
       <c r="R17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S17">
         <v>8</v>
@@ -56534,7 +56534,7 @@
         <v>8</v>
       </c>
       <c r="R18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S18">
         <v>9</v>
@@ -56611,7 +56611,7 @@
         <v>5</v>
       </c>
       <c r="R19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S19">
         <v>5</v>
@@ -56629,7 +56629,7 @@
         <v>6</v>
       </c>
       <c r="X19">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Y19">
         <v>6</v>
@@ -56688,7 +56688,7 @@
         <v>5</v>
       </c>
       <c r="R20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="S20">
         <v>5</v>
@@ -56765,7 +56765,7 @@
         <v>5</v>
       </c>
       <c r="R21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S21">
         <v>5</v>
@@ -56783,7 +56783,7 @@
         <v>5</v>
       </c>
       <c r="X21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y21">
         <v>5</v>
@@ -56842,7 +56842,7 @@
         <v>7</v>
       </c>
       <c r="R22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S22">
         <v>6</v>
@@ -56860,7 +56860,7 @@
         <v>6</v>
       </c>
       <c r="X22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y22">
         <v>6</v>
@@ -56919,7 +56919,7 @@
         <v>10</v>
       </c>
       <c r="R23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S23">
         <v>8</v>
@@ -56996,7 +56996,7 @@
         <v>7</v>
       </c>
       <c r="R24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S24">
         <v>7</v>
@@ -57014,7 +57014,7 @@
         <v>6</v>
       </c>
       <c r="X24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y24">
         <v>6</v>
@@ -57073,7 +57073,7 @@
         <v>8</v>
       </c>
       <c r="R25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S25">
         <v>10</v>
@@ -57208,7 +57208,7 @@
         <v>6</v>
       </c>
       <c r="R28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S28">
         <v>5</v>
@@ -57285,7 +57285,7 @@
         <v>8</v>
       </c>
       <c r="R29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S29">
         <v>5</v>
@@ -57303,7 +57303,7 @@
         <v>6</v>
       </c>
       <c r="X29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y29">
         <v>5</v>
@@ -57362,7 +57362,7 @@
         <v>5</v>
       </c>
       <c r="R30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S30">
         <v>5</v>
@@ -63926,7 +63926,7 @@
         <v>10</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q4">
         <v>-1</v>
@@ -63944,7 +63944,7 @@
         <v>10</v>
       </c>
       <c r="V4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W4">
         <v>9</v>
@@ -64003,7 +64003,7 @@
         <v>7</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q5">
         <v>-1</v>
@@ -64080,7 +64080,7 @@
         <v>5</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q6">
         <v>-1</v>
@@ -64098,7 +64098,7 @@
         <v>7</v>
       </c>
       <c r="V6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>7</v>
@@ -64157,7 +64157,7 @@
         <v>5</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q7">
         <v>-1</v>
@@ -64234,7 +64234,7 @@
         <v>10</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q8">
         <v>-1</v>
@@ -64311,7 +64311,7 @@
         <v>5</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q9">
         <v>-1</v>
@@ -64388,7 +64388,7 @@
         <v>10</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q10">
         <v>-1</v>
@@ -64465,7 +64465,7 @@
         <v>10</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q11">
         <v>-1</v>
@@ -64542,7 +64542,7 @@
         <v>10</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q12">
         <v>-1</v>
@@ -64560,7 +64560,7 @@
         <v>9</v>
       </c>
       <c r="V12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W12">
         <v>8</v>
@@ -64619,7 +64619,7 @@
         <v>5</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q13">
         <v>-1</v>
@@ -64696,7 +64696,7 @@
         <v>10</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q14">
         <v>-1</v>
@@ -64714,7 +64714,7 @@
         <v>10</v>
       </c>
       <c r="V14">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W14">
         <v>9</v>
@@ -64773,7 +64773,7 @@
         <v>5</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q15">
         <v>-1</v>
@@ -64850,7 +64850,7 @@
         <v>10</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q16">
         <v>-1</v>
@@ -64868,7 +64868,7 @@
         <v>10</v>
       </c>
       <c r="V16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W16">
         <v>9</v>
@@ -64927,7 +64927,7 @@
         <v>10</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q17">
         <v>-1</v>
@@ -65004,7 +65004,7 @@
         <v>7</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q18">
         <v>-1</v>
@@ -65081,7 +65081,7 @@
         <v>5</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q19">
         <v>-1</v>
@@ -65158,7 +65158,7 @@
         <v>7</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q20">
         <v>-1</v>
@@ -65176,7 +65176,7 @@
         <v>9</v>
       </c>
       <c r="V20">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W20">
         <v>9</v>
@@ -65235,7 +65235,7 @@
         <v>10</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q21">
         <v>-1</v>
@@ -65253,7 +65253,7 @@
         <v>10</v>
       </c>
       <c r="V21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W21">
         <v>8</v>
@@ -65312,7 +65312,7 @@
         <v>7</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q22">
         <v>-1</v>
@@ -65389,7 +65389,7 @@
         <v>7</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q23">
         <v>-1</v>
@@ -65466,7 +65466,7 @@
         <v>5</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q24">
         <v>-1</v>
@@ -65543,7 +65543,7 @@
         <v>10</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q25">
         <v>-1</v>
@@ -65620,7 +65620,7 @@
         <v>5</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q26">
         <v>-1</v>
@@ -65697,7 +65697,7 @@
         <v>5</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q27">
         <v>-1</v>
@@ -65774,7 +65774,7 @@
         <v>10</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q28">
         <v>-1</v>
@@ -65792,7 +65792,7 @@
         <v>10</v>
       </c>
       <c r="V28">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W28">
         <v>7</v>
@@ -65851,7 +65851,7 @@
         <v>10</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q29">
         <v>-1</v>
@@ -65928,7 +65928,7 @@
         <v>6</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q30">
         <v>-1</v>
@@ -65946,7 +65946,7 @@
         <v>9</v>
       </c>
       <c r="V30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W30">
         <v>8</v>
@@ -66005,7 +66005,7 @@
         <v>10</v>
       </c>
       <c r="P31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q31">
         <v>-1</v>
@@ -66082,7 +66082,7 @@
         <v>10</v>
       </c>
       <c r="P32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q32">
         <v>-1</v>
@@ -66159,7 +66159,7 @@
         <v>10</v>
       </c>
       <c r="P33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q33">
         <v>-1</v>
@@ -66177,7 +66177,7 @@
         <v>10</v>
       </c>
       <c r="V33">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W33">
         <v>10</v>
@@ -66236,7 +66236,7 @@
         <v>10</v>
       </c>
       <c r="P34">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q34">
         <v>-1</v>
@@ -66313,7 +66313,7 @@
         <v>10</v>
       </c>
       <c r="P35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q35">
         <v>-1</v>
@@ -66390,7 +66390,7 @@
         <v>10</v>
       </c>
       <c r="P36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q36">
         <v>-1</v>
@@ -66467,7 +66467,7 @@
         <v>5</v>
       </c>
       <c r="P37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q37">
         <v>-1</v>
@@ -66485,7 +66485,7 @@
         <v>8</v>
       </c>
       <c r="V37">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W37">
         <v>8</v>
@@ -66544,7 +66544,7 @@
         <v>10</v>
       </c>
       <c r="P38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q38">
         <v>-1</v>
@@ -66562,7 +66562,7 @@
         <v>10</v>
       </c>
       <c r="V38">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W38">
         <v>10</v>
@@ -66621,7 +66621,7 @@
         <v>10</v>
       </c>
       <c r="P39">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q39">
         <v>-1</v>
@@ -66698,7 +66698,7 @@
         <v>10</v>
       </c>
       <c r="P40">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q40">
         <v>-1</v>
@@ -66775,7 +66775,7 @@
         <v>10</v>
       </c>
       <c r="P41">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q41">
         <v>-1</v>
@@ -66793,7 +66793,7 @@
         <v>10</v>
       </c>
       <c r="V41">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W41">
         <v>10</v>
@@ -66852,7 +66852,7 @@
         <v>7</v>
       </c>
       <c r="P42">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q42">
         <v>-1</v>
@@ -66929,7 +66929,7 @@
         <v>10</v>
       </c>
       <c r="P43">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q43">
         <v>-1</v>
@@ -66947,7 +66947,7 @@
         <v>10</v>
       </c>
       <c r="V43">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W43">
         <v>9</v>
@@ -75339,7 +75339,7 @@
         <v>10</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q4">
         <v>-1</v>
@@ -75357,7 +75357,7 @@
         <v>10</v>
       </c>
       <c r="V4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W4">
         <v>9</v>
@@ -75416,7 +75416,7 @@
         <v>10</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q5">
         <v>-1</v>
@@ -75493,7 +75493,7 @@
         <v>10</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q6">
         <v>-1</v>
@@ -75570,7 +75570,7 @@
         <v>5</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q7">
         <v>-1</v>
@@ -75588,7 +75588,7 @@
         <v>6</v>
       </c>
       <c r="V7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W7">
         <v>8</v>
@@ -75647,7 +75647,7 @@
         <v>7</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q8">
         <v>-1</v>
@@ -75724,7 +75724,7 @@
         <v>10</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q9">
         <v>-1</v>
@@ -75801,7 +75801,7 @@
         <v>10</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q10">
         <v>-1</v>
@@ -75878,7 +75878,7 @@
         <v>10</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q11">
         <v>-1</v>
@@ -75896,7 +75896,7 @@
         <v>7</v>
       </c>
       <c r="V11">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W11">
         <v>5</v>
@@ -75955,7 +75955,7 @@
         <v>10</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q12">
         <v>-1</v>
@@ -75973,7 +75973,7 @@
         <v>10</v>
       </c>
       <c r="V12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W12">
         <v>10</v>
@@ -76032,7 +76032,7 @@
         <v>10</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q13">
         <v>-1</v>
@@ -76109,7 +76109,7 @@
         <v>10</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q14">
         <v>-1</v>
@@ -76186,7 +76186,7 @@
         <v>10</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q15">
         <v>-1</v>
@@ -76204,7 +76204,7 @@
         <v>10</v>
       </c>
       <c r="V15">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W15">
         <v>9</v>
@@ -76263,7 +76263,7 @@
         <v>10</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q16">
         <v>-1</v>
@@ -76340,7 +76340,7 @@
         <v>10</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q17">
         <v>-1</v>
@@ -76417,7 +76417,7 @@
         <v>7</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q18">
         <v>-1</v>
@@ -76494,7 +76494,7 @@
         <v>10</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q19">
         <v>-1</v>
@@ -76512,7 +76512,7 @@
         <v>8</v>
       </c>
       <c r="V19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W19">
         <v>7</v>
@@ -76571,7 +76571,7 @@
         <v>6</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q20">
         <v>-1</v>
@@ -76589,7 +76589,7 @@
         <v>7</v>
       </c>
       <c r="V20">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W20">
         <v>7</v>
@@ -76648,7 +76648,7 @@
         <v>10</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q21">
         <v>-1</v>
@@ -76725,7 +76725,7 @@
         <v>10</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q22">
         <v>-1</v>
@@ -76743,7 +76743,7 @@
         <v>10</v>
       </c>
       <c r="V22">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W22">
         <v>10</v>
@@ -76802,7 +76802,7 @@
         <v>7</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q23">
         <v>-1</v>
@@ -76879,7 +76879,7 @@
         <v>10</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q24">
         <v>-1</v>
@@ -76956,7 +76956,7 @@
         <v>10</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q25">
         <v>-1</v>
@@ -77033,7 +77033,7 @@
         <v>10</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q26">
         <v>-1</v>
@@ -77110,7 +77110,7 @@
         <v>10</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q27">
         <v>-1</v>
@@ -77187,7 +77187,7 @@
         <v>6</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q28">
         <v>-1</v>
@@ -77205,7 +77205,7 @@
         <v>7</v>
       </c>
       <c r="V28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W28">
         <v>6</v>
@@ -77264,7 +77264,7 @@
         <v>10</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q29">
         <v>-1</v>
@@ -77282,7 +77282,7 @@
         <v>10</v>
       </c>
       <c r="V29">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W29">
         <v>10</v>
@@ -77341,7 +77341,7 @@
         <v>10</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q30">
         <v>-1</v>
@@ -77359,7 +77359,7 @@
         <v>10</v>
       </c>
       <c r="V30">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W30">
         <v>10</v>
@@ -77418,7 +77418,7 @@
         <v>7</v>
       </c>
       <c r="P31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q31">
         <v>-1</v>
@@ -77495,7 +77495,7 @@
         <v>10</v>
       </c>
       <c r="P32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q32">
         <v>-1</v>
@@ -77572,7 +77572,7 @@
         <v>10</v>
       </c>
       <c r="P33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q33">
         <v>-1</v>
@@ -77590,7 +77590,7 @@
         <v>10</v>
       </c>
       <c r="V33">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W33">
         <v>10</v>
@@ -77649,7 +77649,7 @@
         <v>10</v>
       </c>
       <c r="P34">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q34">
         <v>-1</v>
@@ -77726,7 +77726,7 @@
         <v>10</v>
       </c>
       <c r="P35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q35">
         <v>-1</v>
@@ -77803,7 +77803,7 @@
         <v>10</v>
       </c>
       <c r="P36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q36">
         <v>-1</v>
@@ -77821,7 +77821,7 @@
         <v>9</v>
       </c>
       <c r="V36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W36">
         <v>8</v>
@@ -77880,7 +77880,7 @@
         <v>10</v>
       </c>
       <c r="P37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q37">
         <v>-1</v>
@@ -77957,7 +77957,7 @@
         <v>7</v>
       </c>
       <c r="P38">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q38">
         <v>-1</v>
@@ -78034,7 +78034,7 @@
         <v>10</v>
       </c>
       <c r="P39">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q39">
         <v>-1</v>
@@ -78111,7 +78111,7 @@
         <v>10</v>
       </c>
       <c r="P40">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q40">
         <v>-1</v>
@@ -78188,7 +78188,7 @@
         <v>9</v>
       </c>
       <c r="P41">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q41">
         <v>-1</v>
@@ -78206,7 +78206,7 @@
         <v>8</v>
       </c>
       <c r="V41">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W41">
         <v>8</v>
@@ -78265,7 +78265,7 @@
         <v>10</v>
       </c>
       <c r="P42">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q42">
         <v>-1</v>
@@ -78342,7 +78342,7 @@
         <v>10</v>
       </c>
       <c r="P43">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q43">
         <v>-1</v>
@@ -78360,7 +78360,7 @@
         <v>8</v>
       </c>
       <c r="V43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W43">
         <v>6</v>
@@ -78419,7 +78419,7 @@
         <v>7</v>
       </c>
       <c r="P44">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q44">
         <v>-1</v>
@@ -78437,7 +78437,7 @@
         <v>9</v>
       </c>
       <c r="V44">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W44">
         <v>8</v>
@@ -78496,7 +78496,7 @@
         <v>5</v>
       </c>
       <c r="P45">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q45">
         <v>-1</v>
@@ -78573,7 +78573,7 @@
         <v>10</v>
       </c>
       <c r="P46">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q46">
         <v>-1</v>
@@ -78650,7 +78650,7 @@
         <v>10</v>
       </c>
       <c r="P47">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q47">
         <v>-1</v>
@@ -78863,7 +78863,7 @@
         <v>5</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q4">
         <v>-1</v>
@@ -78881,7 +78881,7 @@
         <v>7</v>
       </c>
       <c r="V4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W4">
         <v>7</v>
@@ -78940,7 +78940,7 @@
         <v>5</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q5">
         <v>-1</v>
@@ -78958,7 +78958,7 @@
         <v>8</v>
       </c>
       <c r="V5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="W5">
         <v>8</v>
@@ -79017,7 +79017,7 @@
         <v>10</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q6">
         <v>-1</v>
@@ -79035,7 +79035,7 @@
         <v>9</v>
       </c>
       <c r="V6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>7</v>
@@ -79094,7 +79094,7 @@
         <v>6</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q7">
         <v>-1</v>
@@ -79112,7 +79112,7 @@
         <v>8</v>
       </c>
       <c r="V7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W7">
         <v>8</v>
@@ -79171,7 +79171,7 @@
         <v>6</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q8">
         <v>-1</v>
@@ -79248,7 +79248,7 @@
         <v>8</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q9">
         <v>-1</v>
@@ -79325,7 +79325,7 @@
         <v>10</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q10">
         <v>-1</v>
@@ -79402,7 +79402,7 @@
         <v>10</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q11">
         <v>-1</v>
@@ -79479,7 +79479,7 @@
         <v>5</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q12">
         <v>-1</v>
@@ -79556,7 +79556,7 @@
         <v>10</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q13">
         <v>-1</v>
@@ -79633,7 +79633,7 @@
         <v>9</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q14">
         <v>-1</v>
@@ -79651,7 +79651,7 @@
         <v>10</v>
       </c>
       <c r="V14">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W14">
         <v>8</v>
@@ -79710,7 +79710,7 @@
         <v>10</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q15">
         <v>-1</v>
@@ -79728,7 +79728,7 @@
         <v>10</v>
       </c>
       <c r="V15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W15">
         <v>7</v>
@@ -79787,7 +79787,7 @@
         <v>6</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q16">
         <v>-1</v>
@@ -79805,7 +79805,7 @@
         <v>7</v>
       </c>
       <c r="V16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W16">
         <v>6</v>
@@ -79864,7 +79864,7 @@
         <v>5</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q17">
         <v>-1</v>
@@ -79882,7 +79882,7 @@
         <v>8</v>
       </c>
       <c r="V17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W17">
         <v>10</v>
@@ -79941,7 +79941,7 @@
         <v>10</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q18">
         <v>-1</v>
@@ -80018,7 +80018,7 @@
         <v>10</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q19">
         <v>-1</v>
@@ -80095,7 +80095,7 @@
         <v>8</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q20">
         <v>-1</v>
@@ -80172,7 +80172,7 @@
         <v>6</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q21">
         <v>-1</v>
@@ -80190,7 +80190,7 @@
         <v>7</v>
       </c>
       <c r="V21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W21">
         <v>8</v>
@@ -80249,7 +80249,7 @@
         <v>10</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q22">
         <v>-1</v>
@@ -80326,7 +80326,7 @@
         <v>10</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q23">
         <v>-1</v>
@@ -80403,7 +80403,7 @@
         <v>10</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q24">
         <v>-1</v>
@@ -80480,7 +80480,7 @@
         <v>5</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q25">
         <v>-1</v>
@@ -80557,7 +80557,7 @@
         <v>10</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q26">
         <v>-1</v>
@@ -80575,7 +80575,7 @@
         <v>10</v>
       </c>
       <c r="V26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W26">
         <v>9</v>
@@ -80634,7 +80634,7 @@
         <v>10</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q27">
         <v>-1</v>
@@ -80711,7 +80711,7 @@
         <v>10</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q28">
         <v>-1</v>
@@ -80788,7 +80788,7 @@
         <v>7</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q29">
         <v>-1</v>
@@ -80865,7 +80865,7 @@
         <v>5</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q30">
         <v>-1</v>
@@ -80942,7 +80942,7 @@
         <v>5</v>
       </c>
       <c r="P31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q31">
         <v>-1</v>
@@ -81019,7 +81019,7 @@
         <v>10</v>
       </c>
       <c r="P32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q32">
         <v>-1</v>
@@ -81096,7 +81096,7 @@
         <v>5</v>
       </c>
       <c r="P33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q33">
         <v>-1</v>
@@ -81173,7 +81173,7 @@
         <v>8</v>
       </c>
       <c r="P34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q34">
         <v>-1</v>
@@ -81250,7 +81250,7 @@
         <v>7</v>
       </c>
       <c r="P35">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q35">
         <v>-1</v>
@@ -81327,7 +81327,7 @@
         <v>8</v>
       </c>
       <c r="P36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q36">
         <v>-1</v>
@@ -81345,7 +81345,7 @@
         <v>7</v>
       </c>
       <c r="V36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W36">
         <v>7</v>
@@ -81404,7 +81404,7 @@
         <v>5</v>
       </c>
       <c r="P37">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q37">
         <v>-1</v>
@@ -81422,7 +81422,7 @@
         <v>8</v>
       </c>
       <c r="V37">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W37">
         <v>8</v>
@@ -81481,7 +81481,7 @@
         <v>5</v>
       </c>
       <c r="P38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q38">
         <v>-1</v>
@@ -81558,7 +81558,7 @@
         <v>8</v>
       </c>
       <c r="P39">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q39">
         <v>-1</v>
@@ -81635,7 +81635,7 @@
         <v>10</v>
       </c>
       <c r="P40">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q40">
         <v>-1</v>
@@ -81653,7 +81653,7 @@
         <v>10</v>
       </c>
       <c r="V40">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W40">
         <v>7</v>
@@ -81712,7 +81712,7 @@
         <v>10</v>
       </c>
       <c r="P41">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q41">
         <v>-1</v>
@@ -81789,7 +81789,7 @@
         <v>5</v>
       </c>
       <c r="P42">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q42">
         <v>-1</v>
@@ -81866,7 +81866,7 @@
         <v>10</v>
       </c>
       <c r="P43">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q43">
         <v>-1</v>
@@ -81884,7 +81884,7 @@
         <v>10</v>
       </c>
       <c r="V43">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W43">
         <v>10</v>
@@ -81943,7 +81943,7 @@
         <v>9</v>
       </c>
       <c r="P44">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q44">
         <v>-1</v>
@@ -82020,7 +82020,7 @@
         <v>10</v>
       </c>
       <c r="P45">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q45">
         <v>-1</v>
@@ -82038,7 +82038,7 @@
         <v>10</v>
       </c>
       <c r="V45">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W45">
         <v>10</v>
@@ -82097,7 +82097,7 @@
         <v>10</v>
       </c>
       <c r="P46">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q46">
         <v>-1</v>
@@ -82115,7 +82115,7 @@
         <v>10</v>
       </c>
       <c r="V46">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W46">
         <v>7</v>
@@ -82310,7 +82310,7 @@
         <v>10</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q4">
         <v>-1</v>
@@ -82387,7 +82387,7 @@
         <v>5</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q5">
         <v>-1</v>
@@ -82464,7 +82464,7 @@
         <v>10</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q6">
         <v>-1</v>
@@ -82541,7 +82541,7 @@
         <v>7</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q7">
         <v>-1</v>
@@ -82618,7 +82618,7 @@
         <v>10</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q8">
         <v>-1</v>
@@ -82636,7 +82636,7 @@
         <v>10</v>
       </c>
       <c r="V8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W8">
         <v>9</v>
@@ -82695,7 +82695,7 @@
         <v>7</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q9">
         <v>-1</v>
@@ -82772,7 +82772,7 @@
         <v>10</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q10">
         <v>-1</v>
@@ -82849,7 +82849,7 @@
         <v>10</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q11">
         <v>-1</v>
@@ -82926,7 +82926,7 @@
         <v>6</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q12">
         <v>-1</v>
@@ -82944,7 +82944,7 @@
         <v>8</v>
       </c>
       <c r="V12">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W12">
         <v>6</v>
@@ -83003,7 +83003,7 @@
         <v>10</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q13">
         <v>-1</v>
@@ -83080,7 +83080,7 @@
         <v>5</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q14">
         <v>-1</v>
@@ -83157,7 +83157,7 @@
         <v>10</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q15">
         <v>-1</v>
@@ -83234,7 +83234,7 @@
         <v>6</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q16">
         <v>-1</v>
@@ -83311,7 +83311,7 @@
         <v>7</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q17">
         <v>-1</v>
@@ -83388,7 +83388,7 @@
         <v>5</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q18">
         <v>-1</v>
@@ -83465,7 +83465,7 @@
         <v>5</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q19">
         <v>-1</v>
@@ -83483,7 +83483,7 @@
         <v>6</v>
       </c>
       <c r="V19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W19">
         <v>7</v>
@@ -83542,7 +83542,7 @@
         <v>8</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q20">
         <v>-1</v>
@@ -83619,7 +83619,7 @@
         <v>10</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q21">
         <v>-1</v>
@@ -83696,7 +83696,7 @@
         <v>5</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q22">
         <v>-1</v>
@@ -83714,7 +83714,7 @@
         <v>6</v>
       </c>
       <c r="V22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W22">
         <v>5</v>
@@ -83773,7 +83773,7 @@
         <v>10</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q23">
         <v>-1</v>
@@ -83791,7 +83791,7 @@
         <v>9</v>
       </c>
       <c r="V23">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W23">
         <v>8</v>
@@ -83850,7 +83850,7 @@
         <v>10</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q24">
         <v>-1</v>
@@ -83927,7 +83927,7 @@
         <v>10</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q25">
         <v>-1</v>
@@ -84004,7 +84004,7 @@
         <v>10</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q26">
         <v>-1</v>
@@ -84022,7 +84022,7 @@
         <v>10</v>
       </c>
       <c r="V26">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W26">
         <v>9</v>
@@ -84081,7 +84081,7 @@
         <v>5</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q27">
         <v>-1</v>
@@ -84158,7 +84158,7 @@
         <v>5</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q28">
         <v>-1</v>
@@ -84235,7 +84235,7 @@
         <v>10</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q29">
         <v>-1</v>
@@ -84253,7 +84253,7 @@
         <v>10</v>
       </c>
       <c r="V29">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W29">
         <v>8</v>
@@ -84312,7 +84312,7 @@
         <v>10</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q30">
         <v>-1</v>
@@ -84389,7 +84389,7 @@
         <v>6</v>
       </c>
       <c r="P31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q31">
         <v>-1</v>
@@ -84466,7 +84466,7 @@
         <v>10</v>
       </c>
       <c r="P32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q32">
         <v>-1</v>
@@ -84543,7 +84543,7 @@
         <v>10</v>
       </c>
       <c r="P33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q33">
         <v>-1</v>
@@ -84620,7 +84620,7 @@
         <v>10</v>
       </c>
       <c r="P34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q34">
         <v>-1</v>
@@ -84697,7 +84697,7 @@
         <v>5</v>
       </c>
       <c r="P35">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q35">
         <v>-1</v>
@@ -84774,7 +84774,7 @@
         <v>6</v>
       </c>
       <c r="P36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q36">
         <v>-1</v>
@@ -84792,7 +84792,7 @@
         <v>8</v>
       </c>
       <c r="V36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W36">
         <v>7</v>
@@ -84851,7 +84851,7 @@
         <v>10</v>
       </c>
       <c r="P37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q37">
         <v>-1</v>
@@ -84869,7 +84869,7 @@
         <v>10</v>
       </c>
       <c r="V37">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W37">
         <v>9</v>
@@ -84928,7 +84928,7 @@
         <v>8</v>
       </c>
       <c r="P38">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q38">
         <v>-1</v>
@@ -85005,7 +85005,7 @@
         <v>7</v>
       </c>
       <c r="P39">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q39">
         <v>-1</v>
@@ -85082,7 +85082,7 @@
         <v>9</v>
       </c>
       <c r="P40">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q40">
         <v>-1</v>
@@ -85159,7 +85159,7 @@
         <v>10</v>
       </c>
       <c r="P41">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q41">
         <v>-1</v>
@@ -85236,7 +85236,7 @@
         <v>10</v>
       </c>
       <c r="P42">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q42">
         <v>-1</v>
@@ -85313,7 +85313,7 @@
         <v>7</v>
       </c>
       <c r="P43">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q43">
         <v>-1</v>
@@ -85331,7 +85331,7 @@
         <v>9</v>
       </c>
       <c r="V43">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W43">
         <v>8</v>
@@ -85390,7 +85390,7 @@
         <v>10</v>
       </c>
       <c r="P44">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q44">
         <v>-1</v>
@@ -85408,7 +85408,7 @@
         <v>10</v>
       </c>
       <c r="V44">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W44">
         <v>9</v>
@@ -85467,7 +85467,7 @@
         <v>10</v>
       </c>
       <c r="P45">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q45">
         <v>-1</v>
@@ -85485,7 +85485,7 @@
         <v>8</v>
       </c>
       <c r="V45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W45">
         <v>8</v>
@@ -85544,7 +85544,7 @@
         <v>10</v>
       </c>
       <c r="P46">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q46">
         <v>-1</v>
@@ -85562,7 +85562,7 @@
         <v>9</v>
       </c>
       <c r="V46">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W46">
         <v>5</v>
@@ -91582,7 +91582,7 @@
         <v>9</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T4">
         <v>8</v>
@@ -91600,7 +91600,7 @@
         <v>7</v>
       </c>
       <c r="Y4">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -91659,7 +91659,7 @@
         <v>9</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T5">
         <v>8</v>
@@ -91677,7 +91677,7 @@
         <v>10</v>
       </c>
       <c r="Y5">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -91736,7 +91736,7 @@
         <v>8</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T6">
         <v>6</v>
@@ -91754,7 +91754,7 @@
         <v>8</v>
       </c>
       <c r="Y6">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -91813,7 +91813,7 @@
         <v>6</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T7">
         <v>6</v>
@@ -91890,7 +91890,7 @@
         <v>8</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T8">
         <v>8</v>
@@ -91908,7 +91908,7 @@
         <v>9</v>
       </c>
       <c r="Y8">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -91967,7 +91967,7 @@
         <v>7</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T9">
         <v>8</v>
@@ -92044,7 +92044,7 @@
         <v>8</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T10">
         <v>9</v>
@@ -92121,7 +92121,7 @@
         <v>9</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T11">
         <v>8</v>
@@ -92139,7 +92139,7 @@
         <v>9</v>
       </c>
       <c r="Y11">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -92198,7 +92198,7 @@
         <v>8</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T12">
         <v>10</v>
@@ -92216,7 +92216,7 @@
         <v>9</v>
       </c>
       <c r="Y12">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -92275,7 +92275,7 @@
         <v>8</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T13">
         <v>9</v>
@@ -92352,7 +92352,7 @@
         <v>6</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T14">
         <v>8</v>
@@ -92370,7 +92370,7 @@
         <v>8</v>
       </c>
       <c r="Y14">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -92429,7 +92429,7 @@
         <v>6</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T15">
         <v>8</v>
@@ -92447,7 +92447,7 @@
         <v>8</v>
       </c>
       <c r="Y15">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:25">
@@ -92506,7 +92506,7 @@
         <v>8</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T16">
         <v>8</v>
@@ -92583,7 +92583,7 @@
         <v>9</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T17">
         <v>8</v>
@@ -92601,7 +92601,7 @@
         <v>10</v>
       </c>
       <c r="Y17">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:25">
@@ -92660,7 +92660,7 @@
         <v>9</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T18">
         <v>9</v>
@@ -92737,7 +92737,7 @@
         <v>9</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T19">
         <v>9</v>
@@ -92755,7 +92755,7 @@
         <v>9</v>
       </c>
       <c r="Y19">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:25">
@@ -92814,7 +92814,7 @@
         <v>6</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T20">
         <v>7</v>
@@ -92891,7 +92891,7 @@
         <v>6</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T21">
         <v>8</v>
@@ -92968,7 +92968,7 @@
         <v>9</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T22">
         <v>9</v>
@@ -93045,7 +93045,7 @@
         <v>6</v>
       </c>
       <c r="S23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T23">
         <v>8</v>
@@ -93122,7 +93122,7 @@
         <v>7</v>
       </c>
       <c r="S24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T24">
         <v>6</v>
@@ -93199,7 +93199,7 @@
         <v>9</v>
       </c>
       <c r="S25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T25">
         <v>9</v>
@@ -93276,7 +93276,7 @@
         <v>9</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T26">
         <v>10</v>
@@ -93353,7 +93353,7 @@
         <v>8</v>
       </c>
       <c r="S27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T27">
         <v>8</v>
@@ -93430,7 +93430,7 @@
         <v>9</v>
       </c>
       <c r="S28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T28">
         <v>10</v>
@@ -93448,7 +93448,7 @@
         <v>10</v>
       </c>
       <c r="Y28">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:25">
@@ -93507,7 +93507,7 @@
         <v>6</v>
       </c>
       <c r="S29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T29">
         <v>6</v>
@@ -93525,7 +93525,7 @@
         <v>7</v>
       </c>
       <c r="Y29">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:25">
@@ -93584,7 +93584,7 @@
         <v>8</v>
       </c>
       <c r="S30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T30">
         <v>10</v>

</xml_diff>

<commit_message>
Segundo Parcial 18 mayo
</commit_message>
<xml_diff>
--- a/Calificaciones.xlsx
+++ b/Calificaciones.xlsx
@@ -3870,7 +3870,7 @@
         <v>10</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J4">
         <v>10</v>
@@ -3947,7 +3947,7 @@
         <v>10</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J5">
         <v>10</v>
@@ -4024,7 +4024,7 @@
         <v>10</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J6">
         <v>7</v>
@@ -4060,7 +4060,7 @@
         <v>9</v>
       </c>
       <c r="U6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V6">
         <v>7</v>
@@ -4101,7 +4101,7 @@
         <v>10</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J7">
         <v>10</v>
@@ -4178,7 +4178,7 @@
         <v>9</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J8">
         <v>6</v>
@@ -4214,7 +4214,7 @@
         <v>10</v>
       </c>
       <c r="U8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V8">
         <v>6</v>
@@ -4255,7 +4255,7 @@
         <v>6</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J9">
         <v>5</v>
@@ -4332,7 +4332,7 @@
         <v>4</v>
       </c>
       <c r="I10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J10">
         <v>5</v>
@@ -4368,7 +4368,7 @@
         <v>5</v>
       </c>
       <c r="U10">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V10">
         <v>5</v>
@@ -4409,7 +4409,7 @@
         <v>9</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J11">
         <v>9</v>
@@ -4445,7 +4445,7 @@
         <v>10</v>
       </c>
       <c r="U11">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V11">
         <v>9</v>
@@ -4486,7 +4486,7 @@
         <v>6</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J12">
         <v>5</v>
@@ -4563,7 +4563,7 @@
         <v>3</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J13">
         <v>5</v>
@@ -4599,7 +4599,7 @@
         <v>5</v>
       </c>
       <c r="U13">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V13">
         <v>5</v>
@@ -4640,7 +4640,7 @@
         <v>10</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J14">
         <v>10</v>
@@ -4676,7 +4676,7 @@
         <v>10</v>
       </c>
       <c r="U14">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V14">
         <v>10</v>
@@ -4717,7 +4717,7 @@
         <v>7</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J15">
         <v>6</v>
@@ -4753,7 +4753,7 @@
         <v>8</v>
       </c>
       <c r="U15">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V15">
         <v>6</v>
@@ -4794,7 +4794,7 @@
         <v>10</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J16">
         <v>10</v>
@@ -4871,7 +4871,7 @@
         <v>7</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J17">
         <v>8</v>
@@ -4948,7 +4948,7 @@
         <v>10</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J18">
         <v>10</v>
@@ -4984,7 +4984,7 @@
         <v>10</v>
       </c>
       <c r="U18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V18">
         <v>10</v>
@@ -5025,7 +5025,7 @@
         <v>9</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J19">
         <v>9</v>
@@ -5061,7 +5061,7 @@
         <v>10</v>
       </c>
       <c r="U19">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V19">
         <v>10</v>
@@ -5102,7 +5102,7 @@
         <v>9</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J20">
         <v>9</v>
@@ -5179,7 +5179,7 @@
         <v>7</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J21">
         <v>10</v>
@@ -5215,7 +5215,7 @@
         <v>8</v>
       </c>
       <c r="U21">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V21">
         <v>8</v>
@@ -5256,7 +5256,7 @@
         <v>10</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J22">
         <v>9</v>
@@ -5333,7 +5333,7 @@
         <v>10</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J23">
         <v>10</v>
@@ -5410,7 +5410,7 @@
         <v>7</v>
       </c>
       <c r="I24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J24">
         <v>6</v>
@@ -5446,7 +5446,7 @@
         <v>8</v>
       </c>
       <c r="U24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V24">
         <v>7</v>
@@ -5487,7 +5487,7 @@
         <v>3</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J25">
         <v>6</v>
@@ -5523,7 +5523,7 @@
         <v>5</v>
       </c>
       <c r="U25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V25">
         <v>6</v>
@@ -5564,7 +5564,7 @@
         <v>6</v>
       </c>
       <c r="I26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J26">
         <v>6</v>
@@ -5600,7 +5600,7 @@
         <v>8</v>
       </c>
       <c r="U26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V26">
         <v>6</v>
@@ -5641,7 +5641,7 @@
         <v>10</v>
       </c>
       <c r="I27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J27">
         <v>7</v>
@@ -5718,7 +5718,7 @@
         <v>10</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J28">
         <v>8</v>
@@ -5795,7 +5795,7 @@
         <v>10</v>
       </c>
       <c r="I29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J29">
         <v>9</v>
@@ -5831,7 +5831,7 @@
         <v>10</v>
       </c>
       <c r="U29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V29">
         <v>9</v>
@@ -5872,7 +5872,7 @@
         <v>10</v>
       </c>
       <c r="I30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J30">
         <v>10</v>
@@ -5949,7 +5949,7 @@
         <v>10</v>
       </c>
       <c r="I31">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J31">
         <v>9</v>
@@ -5985,7 +5985,7 @@
         <v>10</v>
       </c>
       <c r="U31">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V31">
         <v>9</v>
@@ -6026,7 +6026,7 @@
         <v>10</v>
       </c>
       <c r="I32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J32">
         <v>8</v>
@@ -6062,7 +6062,7 @@
         <v>10</v>
       </c>
       <c r="U32">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V32">
         <v>9</v>
@@ -6103,7 +6103,7 @@
         <v>8</v>
       </c>
       <c r="I33">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J33">
         <v>8</v>
@@ -6139,7 +6139,7 @@
         <v>9</v>
       </c>
       <c r="U33">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V33">
         <v>9</v>
@@ -6180,7 +6180,7 @@
         <v>10</v>
       </c>
       <c r="I34">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J34">
         <v>10</v>
@@ -6216,7 +6216,7 @@
         <v>10</v>
       </c>
       <c r="U34">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V34">
         <v>10</v>
@@ -6257,7 +6257,7 @@
         <v>10</v>
       </c>
       <c r="I35">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J35">
         <v>10</v>
@@ -6293,7 +6293,7 @@
         <v>10</v>
       </c>
       <c r="U35">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V35">
         <v>10</v>
@@ -6334,7 +6334,7 @@
         <v>4</v>
       </c>
       <c r="I36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J36">
         <v>6</v>
@@ -6411,7 +6411,7 @@
         <v>9</v>
       </c>
       <c r="I37">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J37">
         <v>8</v>
@@ -6447,7 +6447,7 @@
         <v>9</v>
       </c>
       <c r="U37">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V37">
         <v>8</v>
@@ -7622,7 +7622,7 @@
         <v>6</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I17">
         <v>7</v>
@@ -7658,7 +7658,7 @@
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U17">
         <v>7</v>
@@ -23048,7 +23048,7 @@
         <v>9</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J4">
         <v>10</v>
@@ -23125,7 +23125,7 @@
         <v>10</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J5">
         <v>9</v>
@@ -23202,7 +23202,7 @@
         <v>9</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J6">
         <v>9</v>
@@ -23238,7 +23238,7 @@
         <v>9</v>
       </c>
       <c r="U6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V6">
         <v>9</v>
@@ -23279,7 +23279,7 @@
         <v>10</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J7">
         <v>9</v>
@@ -23356,7 +23356,7 @@
         <v>10</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J8">
         <v>9</v>
@@ -23433,7 +23433,7 @@
         <v>10</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J9">
         <v>9</v>
@@ -23510,7 +23510,7 @@
         <v>9</v>
       </c>
       <c r="I10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J10">
         <v>10</v>
@@ -23587,7 +23587,7 @@
         <v>9</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J11">
         <v>10</v>
@@ -23623,7 +23623,7 @@
         <v>9</v>
       </c>
       <c r="U11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V11">
         <v>10</v>
@@ -23664,7 +23664,7 @@
         <v>10</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J12">
         <v>10</v>
@@ -23741,7 +23741,7 @@
         <v>7</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J13">
         <v>9</v>
@@ -23818,7 +23818,7 @@
         <v>10</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J14">
         <v>10</v>
@@ -23854,7 +23854,7 @@
         <v>10</v>
       </c>
       <c r="U14">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="V14">
         <v>10</v>
@@ -23895,7 +23895,7 @@
         <v>7</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J15">
         <v>10</v>
@@ -23931,7 +23931,7 @@
         <v>8</v>
       </c>
       <c r="U15">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V15">
         <v>10</v>
@@ -23972,7 +23972,7 @@
         <v>10</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J16">
         <v>10</v>
@@ -24049,7 +24049,7 @@
         <v>8</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J17">
         <v>10</v>
@@ -24126,7 +24126,7 @@
         <v>9</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J18">
         <v>9</v>
@@ -24203,7 +24203,7 @@
         <v>10</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J19">
         <v>10</v>
@@ -24280,7 +24280,7 @@
         <v>9</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J20">
         <v>10</v>
@@ -24357,7 +24357,7 @@
         <v>8</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J21">
         <v>9</v>
@@ -24434,7 +24434,7 @@
         <v>8</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J22">
         <v>10</v>
@@ -24511,7 +24511,7 @@
         <v>5</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J23">
         <v>10</v>
@@ -24547,7 +24547,7 @@
         <v>8</v>
       </c>
       <c r="U23">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V23">
         <v>10</v>
@@ -24588,7 +24588,7 @@
         <v>8</v>
       </c>
       <c r="I24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J24">
         <v>9</v>
@@ -24665,7 +24665,7 @@
         <v>10</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J25">
         <v>10</v>
@@ -24742,7 +24742,7 @@
         <v>5</v>
       </c>
       <c r="I26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J26">
         <v>10</v>
@@ -24778,7 +24778,7 @@
         <v>8</v>
       </c>
       <c r="U26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V26">
         <v>10</v>
@@ -24819,7 +24819,7 @@
         <v>8</v>
       </c>
       <c r="I27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J27">
         <v>10</v>
@@ -24855,7 +24855,7 @@
         <v>8</v>
       </c>
       <c r="U27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V27">
         <v>10</v>
@@ -24896,7 +24896,7 @@
         <v>6</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J28">
         <v>9</v>
@@ -24973,7 +24973,7 @@
         <v>10</v>
       </c>
       <c r="I29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J29">
         <v>9</v>
@@ -25050,7 +25050,7 @@
         <v>9</v>
       </c>
       <c r="I30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J30">
         <v>10</v>
@@ -25127,7 +25127,7 @@
         <v>10</v>
       </c>
       <c r="I31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J31">
         <v>9</v>
@@ -25204,7 +25204,7 @@
         <v>10</v>
       </c>
       <c r="I32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J32">
         <v>10</v>
@@ -25281,7 +25281,7 @@
         <v>9</v>
       </c>
       <c r="I33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J33">
         <v>10</v>
@@ -25358,7 +25358,7 @@
         <v>9</v>
       </c>
       <c r="I34">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J34">
         <v>10</v>
@@ -25435,7 +25435,7 @@
         <v>7</v>
       </c>
       <c r="I35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J35">
         <v>9</v>
@@ -25512,7 +25512,7 @@
         <v>10</v>
       </c>
       <c r="I36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J36">
         <v>10</v>
@@ -25589,7 +25589,7 @@
         <v>9</v>
       </c>
       <c r="I37">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J37">
         <v>10</v>
@@ -25666,7 +25666,7 @@
         <v>10</v>
       </c>
       <c r="I38">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J38">
         <v>9</v>
@@ -25743,7 +25743,7 @@
         <v>9</v>
       </c>
       <c r="I39">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J39">
         <v>10</v>
@@ -33414,7 +33414,7 @@
         <v>9</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I4">
         <v>10</v>
@@ -33450,7 +33450,7 @@
         <v>-1</v>
       </c>
       <c r="T4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U4">
         <v>10</v>
@@ -33491,7 +33491,7 @@
         <v>9</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I5">
         <v>10</v>
@@ -33527,7 +33527,7 @@
         <v>-1</v>
       </c>
       <c r="T5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U5">
         <v>10</v>
@@ -33568,7 +33568,7 @@
         <v>5</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I6">
         <v>9</v>
@@ -33604,7 +33604,7 @@
         <v>-1</v>
       </c>
       <c r="T6">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U6">
         <v>10</v>
@@ -33645,7 +33645,7 @@
         <v>3</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I7">
         <v>5</v>
@@ -33722,7 +33722,7 @@
         <v>8</v>
       </c>
       <c r="H8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I8">
         <v>7</v>
@@ -33758,7 +33758,7 @@
         <v>-1</v>
       </c>
       <c r="T8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U8">
         <v>7</v>
@@ -33799,7 +33799,7 @@
         <v>8</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I9">
         <v>6</v>
@@ -33835,7 +33835,7 @@
         <v>-1</v>
       </c>
       <c r="T9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U9">
         <v>8</v>
@@ -33876,7 +33876,7 @@
         <v>10</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I10">
         <v>10</v>
@@ -33912,7 +33912,7 @@
         <v>-1</v>
       </c>
       <c r="T10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U10">
         <v>10</v>
@@ -33953,7 +33953,7 @@
         <v>9</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I11">
         <v>10</v>
@@ -33989,7 +33989,7 @@
         <v>-1</v>
       </c>
       <c r="T11">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U11">
         <v>10</v>
@@ -34030,7 +34030,7 @@
         <v>9</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I12">
         <v>9</v>
@@ -34066,7 +34066,7 @@
         <v>-1</v>
       </c>
       <c r="T12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U12">
         <v>10</v>
@@ -34107,7 +34107,7 @@
         <v>9</v>
       </c>
       <c r="H13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I13">
         <v>9</v>
@@ -34143,7 +34143,7 @@
         <v>-1</v>
       </c>
       <c r="T13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U13">
         <v>10</v>
@@ -34184,7 +34184,7 @@
         <v>8</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I14">
         <v>10</v>
@@ -34220,7 +34220,7 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U14">
         <v>10</v>
@@ -34261,7 +34261,7 @@
         <v>9</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I15">
         <v>8</v>
@@ -34297,7 +34297,7 @@
         <v>-1</v>
       </c>
       <c r="T15">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U15">
         <v>8</v>
@@ -34338,7 +34338,7 @@
         <v>8</v>
       </c>
       <c r="H16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I16">
         <v>9</v>
@@ -34415,7 +34415,7 @@
         <v>10</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I17">
         <v>10</v>
@@ -34451,7 +34451,7 @@
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U17">
         <v>10</v>
@@ -34492,7 +34492,7 @@
         <v>5</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I18">
         <v>10</v>
@@ -34569,7 +34569,7 @@
         <v>6</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I19">
         <v>9</v>
@@ -34646,7 +34646,7 @@
         <v>8</v>
       </c>
       <c r="H20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I20">
         <v>6</v>
@@ -34723,7 +34723,7 @@
         <v>6</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I21">
         <v>6</v>
@@ -34800,7 +34800,7 @@
         <v>6</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I22">
         <v>9</v>
@@ -34877,7 +34877,7 @@
         <v>5</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I23">
         <v>6</v>
@@ -34954,7 +34954,7 @@
         <v>6</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I24">
         <v>10</v>
@@ -34990,7 +34990,7 @@
         <v>-1</v>
       </c>
       <c r="T24">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U24">
         <v>10</v>
@@ -35031,7 +35031,7 @@
         <v>10</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I25">
         <v>10</v>
@@ -35108,7 +35108,7 @@
         <v>8</v>
       </c>
       <c r="H26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I26">
         <v>9</v>
@@ -35144,7 +35144,7 @@
         <v>-1</v>
       </c>
       <c r="T26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U26">
         <v>9</v>
@@ -35185,7 +35185,7 @@
         <v>10</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I27">
         <v>10</v>
@@ -35262,7 +35262,7 @@
         <v>7</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I28">
         <v>5</v>
@@ -35339,7 +35339,7 @@
         <v>9</v>
       </c>
       <c r="H29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I29">
         <v>10</v>
@@ -35416,7 +35416,7 @@
         <v>7</v>
       </c>
       <c r="H30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I30">
         <v>8</v>
@@ -35452,7 +35452,7 @@
         <v>-1</v>
       </c>
       <c r="T30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U30">
         <v>9</v>
@@ -35493,7 +35493,7 @@
         <v>9</v>
       </c>
       <c r="H31">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I31">
         <v>8</v>
@@ -35570,7 +35570,7 @@
         <v>10</v>
       </c>
       <c r="H32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I32">
         <v>10</v>
@@ -35606,7 +35606,7 @@
         <v>-1</v>
       </c>
       <c r="T32">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U32">
         <v>10</v>
@@ -35647,7 +35647,7 @@
         <v>10</v>
       </c>
       <c r="H33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I33">
         <v>9</v>
@@ -35683,7 +35683,7 @@
         <v>-1</v>
       </c>
       <c r="T33">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U33">
         <v>10</v>
@@ -35724,7 +35724,7 @@
         <v>10</v>
       </c>
       <c r="H34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I34">
         <v>8</v>
@@ -35760,7 +35760,7 @@
         <v>-1</v>
       </c>
       <c r="T34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U34">
         <v>9</v>
@@ -35801,7 +35801,7 @@
         <v>8</v>
       </c>
       <c r="H35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I35">
         <v>10</v>
@@ -35878,7 +35878,7 @@
         <v>4</v>
       </c>
       <c r="H36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I36">
         <v>6</v>
@@ -35914,7 +35914,7 @@
         <v>-1</v>
       </c>
       <c r="T36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U36">
         <v>7</v>
@@ -35955,7 +35955,7 @@
         <v>10</v>
       </c>
       <c r="H37">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I37">
         <v>10</v>
@@ -35991,7 +35991,7 @@
         <v>-1</v>
       </c>
       <c r="T37">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U37">
         <v>10</v>
@@ -36032,7 +36032,7 @@
         <v>3</v>
       </c>
       <c r="H38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I38">
         <v>5</v>
@@ -36109,7 +36109,7 @@
         <v>10</v>
       </c>
       <c r="H39">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I39">
         <v>10</v>
@@ -36186,7 +36186,7 @@
         <v>10</v>
       </c>
       <c r="H40">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I40">
         <v>9</v>
@@ -36222,7 +36222,7 @@
         <v>-1</v>
       </c>
       <c r="T40">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U40">
         <v>10</v>
@@ -36263,7 +36263,7 @@
         <v>9</v>
       </c>
       <c r="H41">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I41">
         <v>6</v>
@@ -36299,7 +36299,7 @@
         <v>-1</v>
       </c>
       <c r="T41">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U41">
         <v>6</v>
@@ -36340,7 +36340,7 @@
         <v>10</v>
       </c>
       <c r="H42">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I42">
         <v>10</v>
@@ -36417,7 +36417,7 @@
         <v>9</v>
       </c>
       <c r="H43">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I43">
         <v>8</v>
@@ -36453,7 +36453,7 @@
         <v>-1</v>
       </c>
       <c r="T43">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U43">
         <v>8</v>
@@ -36494,7 +36494,7 @@
         <v>8</v>
       </c>
       <c r="H44">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I44">
         <v>6</v>
@@ -36530,7 +36530,7 @@
         <v>-1</v>
       </c>
       <c r="T44">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U44">
         <v>8</v>
@@ -36571,7 +36571,7 @@
         <v>9</v>
       </c>
       <c r="H45">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I45">
         <v>8</v>
@@ -36607,7 +36607,7 @@
         <v>-1</v>
       </c>
       <c r="T45">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U45">
         <v>9</v>
@@ -36648,7 +36648,7 @@
         <v>10</v>
       </c>
       <c r="H46">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I46">
         <v>10</v>
@@ -48407,7 +48407,7 @@
         <v>5</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J4">
         <v>5</v>
@@ -48422,7 +48422,7 @@
         <v>5</v>
       </c>
       <c r="N4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O4">
         <v>5</v>
@@ -48496,7 +48496,7 @@
         <v>5</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J5">
         <v>8</v>
@@ -48511,7 +48511,7 @@
         <v>6</v>
       </c>
       <c r="N5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O5">
         <v>6</v>
@@ -48553,7 +48553,7 @@
         <v>5</v>
       </c>
       <c r="AB5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC5">
         <v>5</v>
@@ -48585,7 +48585,7 @@
         <v>6</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J6">
         <v>5</v>
@@ -48600,7 +48600,7 @@
         <v>5</v>
       </c>
       <c r="N6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O6">
         <v>5</v>
@@ -48674,7 +48674,7 @@
         <v>5</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J7">
         <v>5</v>
@@ -48689,7 +48689,7 @@
         <v>4</v>
       </c>
       <c r="N7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O7">
         <v>6</v>
@@ -48763,7 +48763,7 @@
         <v>8</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J8">
         <v>9</v>
@@ -48778,7 +48778,7 @@
         <v>9</v>
       </c>
       <c r="N8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O8">
         <v>8</v>
@@ -48805,7 +48805,7 @@
         <v>-1</v>
       </c>
       <c r="W8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X8">
         <v>9</v>
@@ -48852,7 +48852,7 @@
         <v>5</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J9">
         <v>10</v>
@@ -48867,7 +48867,7 @@
         <v>8</v>
       </c>
       <c r="N9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O9">
         <v>6</v>
@@ -48894,7 +48894,7 @@
         <v>-1</v>
       </c>
       <c r="W9">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X9">
         <v>9</v>
@@ -48941,7 +48941,7 @@
         <v>8</v>
       </c>
       <c r="I10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J10">
         <v>8</v>
@@ -48956,7 +48956,7 @@
         <v>6</v>
       </c>
       <c r="N10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O10">
         <v>8</v>
@@ -48998,7 +48998,7 @@
         <v>8</v>
       </c>
       <c r="AB10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AC10">
         <v>8</v>
@@ -49030,7 +49030,7 @@
         <v>7</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J11">
         <v>7</v>
@@ -49045,7 +49045,7 @@
         <v>9</v>
       </c>
       <c r="N11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O11">
         <v>8</v>
@@ -49072,7 +49072,7 @@
         <v>-1</v>
       </c>
       <c r="W11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X11">
         <v>7</v>
@@ -49087,7 +49087,7 @@
         <v>9</v>
       </c>
       <c r="AB11">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AC11">
         <v>8</v>
@@ -49119,7 +49119,7 @@
         <v>5</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J12">
         <v>5</v>
@@ -49134,7 +49134,7 @@
         <v>5</v>
       </c>
       <c r="N12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O12">
         <v>6</v>
@@ -49208,7 +49208,7 @@
         <v>7</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J13">
         <v>10</v>
@@ -49223,7 +49223,7 @@
         <v>9</v>
       </c>
       <c r="N13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O13">
         <v>8</v>
@@ -49265,7 +49265,7 @@
         <v>10</v>
       </c>
       <c r="AB13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AC13">
         <v>8</v>
@@ -49297,7 +49297,7 @@
         <v>7</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J14">
         <v>6</v>
@@ -49312,7 +49312,7 @@
         <v>9</v>
       </c>
       <c r="N14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O14">
         <v>5</v>
@@ -49339,7 +49339,7 @@
         <v>-1</v>
       </c>
       <c r="W14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X14">
         <v>6</v>
@@ -49386,7 +49386,7 @@
         <v>6</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J15">
         <v>5</v>
@@ -49401,7 +49401,7 @@
         <v>7</v>
       </c>
       <c r="N15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O15">
         <v>5</v>
@@ -49475,7 +49475,7 @@
         <v>7</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J16">
         <v>8</v>
@@ -49490,7 +49490,7 @@
         <v>9</v>
       </c>
       <c r="N16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O16">
         <v>6</v>
@@ -49517,7 +49517,7 @@
         <v>-1</v>
       </c>
       <c r="W16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X16">
         <v>7</v>
@@ -49564,7 +49564,7 @@
         <v>6</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J17">
         <v>7</v>
@@ -49579,7 +49579,7 @@
         <v>9</v>
       </c>
       <c r="N17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O17">
         <v>5</v>
@@ -49653,7 +49653,7 @@
         <v>5</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J18">
         <v>5</v>
@@ -49668,7 +49668,7 @@
         <v>4</v>
       </c>
       <c r="N18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -49742,7 +49742,7 @@
         <v>9</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J19">
         <v>10</v>
@@ -49757,7 +49757,7 @@
         <v>10</v>
       </c>
       <c r="N19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="O19">
         <v>8</v>
@@ -49831,7 +49831,7 @@
         <v>7</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J20">
         <v>7</v>
@@ -49846,7 +49846,7 @@
         <v>5</v>
       </c>
       <c r="N20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O20">
         <v>8</v>
@@ -49920,7 +49920,7 @@
         <v>5</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J21">
         <v>5</v>
@@ -49935,7 +49935,7 @@
         <v>0</v>
       </c>
       <c r="N21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O21">
         <v>5</v>
@@ -50009,7 +50009,7 @@
         <v>8</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J22">
         <v>10</v>
@@ -50024,7 +50024,7 @@
         <v>10</v>
       </c>
       <c r="N22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O22">
         <v>8</v>
@@ -50066,7 +50066,7 @@
         <v>10</v>
       </c>
       <c r="AB22">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AC22">
         <v>8</v>
@@ -50098,7 +50098,7 @@
         <v>5</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J23">
         <v>10</v>
@@ -50113,7 +50113,7 @@
         <v>10</v>
       </c>
       <c r="N23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="O23">
         <v>9</v>
@@ -50140,7 +50140,7 @@
         <v>-1</v>
       </c>
       <c r="W23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="X23">
         <v>9</v>
@@ -50155,7 +50155,7 @@
         <v>10</v>
       </c>
       <c r="AB23">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AC23">
         <v>7</v>
@@ -50184,7 +50184,7 @@
         <v>4</v>
       </c>
       <c r="N24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O24">
         <v>5</v>
@@ -50240,7 +50240,7 @@
         <v>6</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J25">
         <v>6</v>
@@ -50255,7 +50255,7 @@
         <v>9</v>
       </c>
       <c r="N25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O25">
         <v>9</v>
@@ -50297,7 +50297,7 @@
         <v>8</v>
       </c>
       <c r="AB25">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AC25">
         <v>8</v>
@@ -50326,7 +50326,7 @@
         <v>5</v>
       </c>
       <c r="I26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J26">
         <v>8</v>
@@ -50338,7 +50338,7 @@
         <v>9</v>
       </c>
       <c r="N26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O26">
         <v>6</v>
@@ -50403,7 +50403,7 @@
         <v>8</v>
       </c>
       <c r="I27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J27">
         <v>7</v>
@@ -50415,7 +50415,7 @@
         <v>5</v>
       </c>
       <c r="N27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O27">
         <v>6</v>
@@ -50483,7 +50483,7 @@
         <v>7</v>
       </c>
       <c r="I28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J28">
         <v>7</v>
@@ -50498,7 +50498,7 @@
         <v>7</v>
       </c>
       <c r="N28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O28">
         <v>8</v>
@@ -50525,7 +50525,7 @@
         <v>-1</v>
       </c>
       <c r="W28">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X28">
         <v>7</v>
@@ -50540,7 +50540,7 @@
         <v>9</v>
       </c>
       <c r="AB28">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AC28">
         <v>8</v>
@@ -50572,7 +50572,7 @@
         <v>8</v>
       </c>
       <c r="I29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J29">
         <v>10</v>
@@ -50587,7 +50587,7 @@
         <v>10</v>
       </c>
       <c r="N29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O29">
         <v>6</v>
@@ -50614,7 +50614,7 @@
         <v>-1</v>
       </c>
       <c r="W29">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X29">
         <v>9</v>
@@ -50661,7 +50661,7 @@
         <v>8</v>
       </c>
       <c r="I30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J30">
         <v>8</v>
@@ -50676,7 +50676,7 @@
         <v>10</v>
       </c>
       <c r="N30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O30">
         <v>7</v>
@@ -50750,7 +50750,7 @@
         <v>6</v>
       </c>
       <c r="I31">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J31">
         <v>7</v>
@@ -50765,7 +50765,7 @@
         <v>8</v>
       </c>
       <c r="N31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O31">
         <v>8</v>
@@ -50839,7 +50839,7 @@
         <v>7</v>
       </c>
       <c r="I32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J32">
         <v>7</v>
@@ -50854,7 +50854,7 @@
         <v>8</v>
       </c>
       <c r="N32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O32">
         <v>5</v>
@@ -50928,7 +50928,7 @@
         <v>9</v>
       </c>
       <c r="I33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J33">
         <v>9</v>
@@ -50943,7 +50943,7 @@
         <v>10</v>
       </c>
       <c r="N33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="O33">
         <v>8</v>
@@ -50970,7 +50970,7 @@
         <v>-1</v>
       </c>
       <c r="W33">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="X33">
         <v>8</v>
@@ -51017,7 +51017,7 @@
         <v>7</v>
       </c>
       <c r="I34">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J34">
         <v>7</v>
@@ -51032,7 +51032,7 @@
         <v>7</v>
       </c>
       <c r="N34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O34">
         <v>6</v>
@@ -51059,7 +51059,7 @@
         <v>-1</v>
       </c>
       <c r="W34">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X34">
         <v>7</v>
@@ -51106,7 +51106,7 @@
         <v>9</v>
       </c>
       <c r="I35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J35">
         <v>10</v>
@@ -51121,7 +51121,7 @@
         <v>10</v>
       </c>
       <c r="N35">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="O35">
         <v>9</v>
@@ -51148,7 +51148,7 @@
         <v>-1</v>
       </c>
       <c r="W35">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X35">
         <v>10</v>
@@ -51163,7 +51163,7 @@
         <v>10</v>
       </c>
       <c r="AB35">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AC35">
         <v>9</v>
@@ -51195,7 +51195,7 @@
         <v>6</v>
       </c>
       <c r="I36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J36">
         <v>5</v>
@@ -51210,7 +51210,7 @@
         <v>4</v>
       </c>
       <c r="N36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O36">
         <v>6</v>
@@ -53820,7 +53820,7 @@
         <v>6</v>
       </c>
       <c r="E32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="F32">
         <v>10</v>
@@ -53841,7 +53841,7 @@
         <v>5</v>
       </c>
       <c r="L32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M32">
         <v>10</v>
@@ -53883,7 +53883,7 @@
         <v>5</v>
       </c>
       <c r="Z32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="AA32">
         <v>10</v>
@@ -54803,7 +54803,7 @@
         <v>5</v>
       </c>
       <c r="O5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P5">
         <v>-1</v>
@@ -54892,7 +54892,7 @@
         <v>5</v>
       </c>
       <c r="O6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P6">
         <v>-1</v>
@@ -54981,7 +54981,7 @@
         <v>7</v>
       </c>
       <c r="O7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P7">
         <v>-1</v>
@@ -55023,7 +55023,7 @@
         <v>7</v>
       </c>
       <c r="AC7">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:29">
@@ -55248,7 +55248,7 @@
         <v>7</v>
       </c>
       <c r="O10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P10">
         <v>-1</v>
@@ -55290,7 +55290,7 @@
         <v>6</v>
       </c>
       <c r="AC10">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:29">
@@ -55426,7 +55426,7 @@
         <v>5</v>
       </c>
       <c r="O12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P12">
         <v>-1</v>
@@ -55468,7 +55468,7 @@
         <v>7</v>
       </c>
       <c r="AC12">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:29">
@@ -55782,7 +55782,7 @@
         <v>5</v>
       </c>
       <c r="O16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P16">
         <v>-1</v>
@@ -55871,7 +55871,7 @@
         <v>5</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P17">
         <v>-1</v>
@@ -55954,7 +55954,7 @@
         <v>0</v>
       </c>
       <c r="O18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P18">
         <v>-1</v>
@@ -56126,7 +56126,7 @@
         <v>5</v>
       </c>
       <c r="O20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P20">
         <v>-1</v>
@@ -56215,7 +56215,7 @@
         <v>6</v>
       </c>
       <c r="O21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P21">
         <v>-1</v>
@@ -56304,7 +56304,7 @@
         <v>6</v>
       </c>
       <c r="O22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P22">
         <v>-1</v>
@@ -56393,7 +56393,7 @@
         <v>7</v>
       </c>
       <c r="O23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P23">
         <v>-1</v>
@@ -56838,7 +56838,7 @@
         <v>5</v>
       </c>
       <c r="O28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P28">
         <v>-1</v>
@@ -56880,7 +56880,7 @@
         <v>5</v>
       </c>
       <c r="AC28">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -58259,7 +58259,7 @@
         <v>6</v>
       </c>
       <c r="G20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="H20">
         <v>5</v>
@@ -58277,7 +58277,7 @@
         <v>5</v>
       </c>
       <c r="M20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="N20">
         <v>-1</v>
@@ -58313,7 +58313,7 @@
         <v>5</v>
       </c>
       <c r="Y20">
-        <v>-1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:25">
@@ -69680,7 +69680,7 @@
         <v>9</v>
       </c>
       <c r="K4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L4">
         <v>9</v>
@@ -69757,7 +69757,7 @@
         <v>9</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L5">
         <v>9</v>
@@ -69834,7 +69834,7 @@
         <v>9</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L6">
         <v>9</v>
@@ -69911,7 +69911,7 @@
         <v>10</v>
       </c>
       <c r="K7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L7">
         <v>10</v>
@@ -69988,7 +69988,7 @@
         <v>9</v>
       </c>
       <c r="K8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L8">
         <v>9</v>
@@ -70024,7 +70024,7 @@
         <v>9</v>
       </c>
       <c r="W8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X8">
         <v>9</v>
@@ -70065,7 +70065,7 @@
         <v>10</v>
       </c>
       <c r="K9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L9">
         <v>10</v>
@@ -70101,7 +70101,7 @@
         <v>9</v>
       </c>
       <c r="W9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X9">
         <v>9</v>
@@ -70142,7 +70142,7 @@
         <v>9</v>
       </c>
       <c r="K10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L10">
         <v>9</v>
@@ -70178,7 +70178,7 @@
         <v>9</v>
       </c>
       <c r="W10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X10">
         <v>9</v>
@@ -70219,7 +70219,7 @@
         <v>9</v>
       </c>
       <c r="K11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L11">
         <v>9</v>
@@ -70296,7 +70296,7 @@
         <v>9</v>
       </c>
       <c r="K12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L12">
         <v>9</v>
@@ -70332,7 +70332,7 @@
         <v>9</v>
       </c>
       <c r="W12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X12">
         <v>9</v>
@@ -70373,7 +70373,7 @@
         <v>8</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L13">
         <v>8</v>
@@ -70409,7 +70409,7 @@
         <v>8</v>
       </c>
       <c r="W13">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X13">
         <v>8</v>
@@ -70450,7 +70450,7 @@
         <v>9</v>
       </c>
       <c r="K14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L14">
         <v>9</v>
@@ -70486,7 +70486,7 @@
         <v>9</v>
       </c>
       <c r="W14">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="X14">
         <v>9</v>
@@ -70527,7 +70527,7 @@
         <v>9</v>
       </c>
       <c r="K15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L15">
         <v>9</v>
@@ -70563,7 +70563,7 @@
         <v>9</v>
       </c>
       <c r="W15">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X15">
         <v>9</v>
@@ -70604,7 +70604,7 @@
         <v>8</v>
       </c>
       <c r="K16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L16">
         <v>8</v>
@@ -70640,7 +70640,7 @@
         <v>8</v>
       </c>
       <c r="W16">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X16">
         <v>8</v>
@@ -70681,7 +70681,7 @@
         <v>9</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L17">
         <v>9</v>
@@ -70717,7 +70717,7 @@
         <v>9</v>
       </c>
       <c r="W17">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X17">
         <v>9</v>
@@ -70758,7 +70758,7 @@
         <v>7</v>
       </c>
       <c r="K18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="L18">
         <v>7</v>
@@ -70835,7 +70835,7 @@
         <v>9</v>
       </c>
       <c r="K19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L19">
         <v>9</v>
@@ -70871,7 +70871,7 @@
         <v>9</v>
       </c>
       <c r="W19">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X19">
         <v>9</v>
@@ -70912,7 +70912,7 @@
         <v>9</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L20">
         <v>9</v>
@@ -70948,7 +70948,7 @@
         <v>9</v>
       </c>
       <c r="W20">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="X20">
         <v>9</v>
@@ -70989,7 +70989,7 @@
         <v>9</v>
       </c>
       <c r="K21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L21">
         <v>9</v>
@@ -71066,7 +71066,7 @@
         <v>10</v>
       </c>
       <c r="K22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L22">
         <v>10</v>
@@ -71143,7 +71143,7 @@
         <v>9</v>
       </c>
       <c r="K23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L23">
         <v>9</v>
@@ -71220,7 +71220,7 @@
         <v>9</v>
       </c>
       <c r="K24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L24">
         <v>9</v>
@@ -71297,7 +71297,7 @@
         <v>10</v>
       </c>
       <c r="K25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L25">
         <v>10</v>
@@ -71374,7 +71374,7 @@
         <v>10</v>
       </c>
       <c r="K26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L26">
         <v>10</v>
@@ -71451,7 +71451,7 @@
         <v>9</v>
       </c>
       <c r="K27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L27">
         <v>9</v>
@@ -71528,7 +71528,7 @@
         <v>9</v>
       </c>
       <c r="K28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L28">
         <v>9</v>
@@ -71564,7 +71564,7 @@
         <v>9</v>
       </c>
       <c r="W28">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X28">
         <v>9</v>
@@ -71605,7 +71605,7 @@
         <v>9</v>
       </c>
       <c r="K29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L29">
         <v>9</v>
@@ -71641,7 +71641,7 @@
         <v>9</v>
       </c>
       <c r="W29">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X29">
         <v>9</v>
@@ -71682,7 +71682,7 @@
         <v>9</v>
       </c>
       <c r="K30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L30">
         <v>9</v>
@@ -71718,7 +71718,7 @@
         <v>9</v>
       </c>
       <c r="W30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X30">
         <v>9</v>
@@ -71759,7 +71759,7 @@
         <v>10</v>
       </c>
       <c r="K31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L31">
         <v>10</v>
@@ -71836,7 +71836,7 @@
         <v>6</v>
       </c>
       <c r="K32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L32">
         <v>6</v>
@@ -71872,7 +71872,7 @@
         <v>6</v>
       </c>
       <c r="W32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X32">
         <v>6</v>
@@ -71913,7 +71913,7 @@
         <v>9</v>
       </c>
       <c r="K33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L33">
         <v>9</v>
@@ -71981,7 +71981,7 @@
         <v>6</v>
       </c>
       <c r="K34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M34">
         <v>6</v>
@@ -73775,7 +73775,7 @@
         <v>8</v>
       </c>
       <c r="J4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K4">
         <v>7</v>
@@ -73852,7 +73852,7 @@
         <v>8</v>
       </c>
       <c r="J5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>5</v>
@@ -73929,7 +73929,7 @@
         <v>9</v>
       </c>
       <c r="J6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K6">
         <v>6</v>
@@ -73965,7 +73965,7 @@
         <v>8</v>
       </c>
       <c r="V6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>6</v>
@@ -74006,7 +74006,7 @@
         <v>8</v>
       </c>
       <c r="J7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K7">
         <v>6</v>
@@ -74042,7 +74042,7 @@
         <v>8</v>
       </c>
       <c r="V7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W7">
         <v>6</v>
@@ -74083,7 +74083,7 @@
         <v>8</v>
       </c>
       <c r="J8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K8">
         <v>10</v>
@@ -74160,7 +74160,7 @@
         <v>9</v>
       </c>
       <c r="J9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K9">
         <v>8</v>
@@ -74196,7 +74196,7 @@
         <v>9</v>
       </c>
       <c r="V9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W9">
         <v>9</v>
@@ -74237,7 +74237,7 @@
         <v>8</v>
       </c>
       <c r="J10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K10">
         <v>10</v>
@@ -74314,7 +74314,7 @@
         <v>9</v>
       </c>
       <c r="J11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K11">
         <v>8</v>
@@ -74350,7 +74350,7 @@
         <v>10</v>
       </c>
       <c r="V11">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W11">
         <v>8</v>
@@ -74391,7 +74391,7 @@
         <v>8</v>
       </c>
       <c r="J12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K12">
         <v>6</v>
@@ -74468,7 +74468,7 @@
         <v>9</v>
       </c>
       <c r="J13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K13">
         <v>10</v>
@@ -74504,7 +74504,7 @@
         <v>10</v>
       </c>
       <c r="V13">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="W13">
         <v>10</v>
@@ -74545,7 +74545,7 @@
         <v>8</v>
       </c>
       <c r="J14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K14">
         <v>6</v>
@@ -74581,7 +74581,7 @@
         <v>8</v>
       </c>
       <c r="V14">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W14">
         <v>6</v>
@@ -74622,7 +74622,7 @@
         <v>8</v>
       </c>
       <c r="J15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K15">
         <v>9</v>
@@ -74658,7 +74658,7 @@
         <v>8</v>
       </c>
       <c r="V15">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W15">
         <v>9</v>
@@ -74699,7 +74699,7 @@
         <v>9</v>
       </c>
       <c r="J16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K16">
         <v>10</v>
@@ -74776,7 +74776,7 @@
         <v>9</v>
       </c>
       <c r="J17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K17">
         <v>7</v>
@@ -74853,7 +74853,7 @@
         <v>8</v>
       </c>
       <c r="J18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K18">
         <v>6</v>
@@ -74889,7 +74889,7 @@
         <v>8</v>
       </c>
       <c r="V18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W18">
         <v>7</v>
@@ -74930,7 +74930,7 @@
         <v>5</v>
       </c>
       <c r="J19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K19">
         <v>5</v>
@@ -75007,7 +75007,7 @@
         <v>9</v>
       </c>
       <c r="J20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K20">
         <v>9</v>
@@ -75084,7 +75084,7 @@
         <v>9</v>
       </c>
       <c r="J21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K21">
         <v>6</v>
@@ -75120,7 +75120,7 @@
         <v>9</v>
       </c>
       <c r="V21">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W21">
         <v>7</v>
@@ -75161,7 +75161,7 @@
         <v>8</v>
       </c>
       <c r="J22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K22">
         <v>6</v>
@@ -75197,7 +75197,7 @@
         <v>9</v>
       </c>
       <c r="V22">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W22">
         <v>6</v>
@@ -75238,7 +75238,7 @@
         <v>9</v>
       </c>
       <c r="J23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K23">
         <v>10</v>
@@ -75315,7 +75315,7 @@
         <v>10</v>
       </c>
       <c r="J24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K24">
         <v>7</v>
@@ -75392,7 +75392,7 @@
         <v>6</v>
       </c>
       <c r="J25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K25">
         <v>6</v>
@@ -75428,7 +75428,7 @@
         <v>7</v>
       </c>
       <c r="V25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W25">
         <v>6</v>
@@ -75469,7 +75469,7 @@
         <v>8</v>
       </c>
       <c r="J26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K26">
         <v>9</v>
@@ -75505,7 +75505,7 @@
         <v>8</v>
       </c>
       <c r="V26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W26">
         <v>10</v>
@@ -75546,7 +75546,7 @@
         <v>8</v>
       </c>
       <c r="J27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K27">
         <v>6</v>
@@ -75582,7 +75582,7 @@
         <v>8</v>
       </c>
       <c r="V27">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W27">
         <v>7</v>
@@ -75623,7 +75623,7 @@
         <v>5</v>
       </c>
       <c r="J28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K28">
         <v>5</v>
@@ -75700,7 +75700,7 @@
         <v>8</v>
       </c>
       <c r="J29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K29">
         <v>8</v>
@@ -75736,7 +75736,7 @@
         <v>9</v>
       </c>
       <c r="V29">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W29">
         <v>7</v>
@@ -75777,7 +75777,7 @@
         <v>8</v>
       </c>
       <c r="J30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K30">
         <v>6</v>
@@ -75813,7 +75813,7 @@
         <v>8</v>
       </c>
       <c r="V30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W30">
         <v>7</v>
@@ -75854,7 +75854,7 @@
         <v>6</v>
       </c>
       <c r="J31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K31">
         <v>6</v>
@@ -75890,7 +75890,7 @@
         <v>7</v>
       </c>
       <c r="V31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W31">
         <v>8</v>
@@ -75931,7 +75931,7 @@
         <v>5</v>
       </c>
       <c r="J32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K32">
         <v>5</v>
@@ -76008,7 +76008,7 @@
         <v>9</v>
       </c>
       <c r="J33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K33">
         <v>10</v>
@@ -76044,7 +76044,7 @@
         <v>10</v>
       </c>
       <c r="V33">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W33">
         <v>10</v>
@@ -76085,7 +76085,7 @@
         <v>9</v>
       </c>
       <c r="J34">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K34">
         <v>10</v>
@@ -76162,7 +76162,7 @@
         <v>8</v>
       </c>
       <c r="J35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K35">
         <v>8</v>
@@ -76198,7 +76198,7 @@
         <v>8</v>
       </c>
       <c r="V35">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W35">
         <v>8</v>
@@ -76239,7 +76239,7 @@
         <v>10</v>
       </c>
       <c r="J36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K36">
         <v>10</v>
@@ -76316,7 +76316,7 @@
         <v>10</v>
       </c>
       <c r="J37">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="K37">
         <v>10</v>
@@ -76393,7 +76393,7 @@
         <v>8</v>
       </c>
       <c r="J38">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K38">
         <v>7</v>
@@ -76429,7 +76429,7 @@
         <v>8</v>
       </c>
       <c r="V38">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W38">
         <v>7</v>
@@ -76470,7 +76470,7 @@
         <v>9</v>
       </c>
       <c r="J39">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="K39">
         <v>10</v>
@@ -76547,7 +76547,7 @@
         <v>9</v>
       </c>
       <c r="J40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K40">
         <v>9</v>
@@ -76583,7 +76583,7 @@
         <v>9</v>
       </c>
       <c r="V40">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W40">
         <v>9</v>
@@ -76624,7 +76624,7 @@
         <v>9</v>
       </c>
       <c r="J41">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K41">
         <v>9</v>
@@ -76660,7 +76660,7 @@
         <v>9</v>
       </c>
       <c r="V41">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W41">
         <v>9</v>
@@ -76701,7 +76701,7 @@
         <v>9</v>
       </c>
       <c r="J42">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K42">
         <v>8</v>
@@ -76778,7 +76778,7 @@
         <v>7</v>
       </c>
       <c r="J43">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K43">
         <v>5</v>
@@ -76814,7 +76814,7 @@
         <v>8</v>
       </c>
       <c r="V43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W43">
         <v>5</v>
@@ -79970,7 +79970,7 @@
         <v>8</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I4">
         <v>10</v>
@@ -80006,7 +80006,7 @@
         <v>-1</v>
       </c>
       <c r="T4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U4">
         <v>10</v>
@@ -80047,7 +80047,7 @@
         <v>7</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I5">
         <v>8</v>
@@ -80124,7 +80124,7 @@
         <v>3</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I6">
         <v>5</v>
@@ -80201,7 +80201,7 @@
         <v>8</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I7">
         <v>9</v>
@@ -80278,7 +80278,7 @@
         <v>8</v>
       </c>
       <c r="H8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I8">
         <v>8</v>
@@ -80355,7 +80355,7 @@
         <v>6</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I9">
         <v>6</v>
@@ -80432,7 +80432,7 @@
         <v>3</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I10">
         <v>5</v>
@@ -80509,7 +80509,7 @@
         <v>8</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I11">
         <v>10</v>
@@ -80586,7 +80586,7 @@
         <v>10</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I12">
         <v>10</v>
@@ -80663,7 +80663,7 @@
         <v>6</v>
       </c>
       <c r="H13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I13">
         <v>7</v>
@@ -80699,7 +80699,7 @@
         <v>-1</v>
       </c>
       <c r="T13">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U13">
         <v>8</v>
@@ -80740,7 +80740,7 @@
         <v>7</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I14">
         <v>9</v>
@@ -80817,7 +80817,7 @@
         <v>6</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I15">
         <v>5</v>
@@ -80894,7 +80894,7 @@
         <v>6</v>
       </c>
       <c r="H16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I16">
         <v>8</v>
@@ -80930,7 +80930,7 @@
         <v>-1</v>
       </c>
       <c r="T16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U16">
         <v>9</v>
@@ -80971,7 +80971,7 @@
         <v>3</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I17">
         <v>5</v>
@@ -81007,7 +81007,7 @@
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U17">
         <v>5</v>
@@ -81048,7 +81048,7 @@
         <v>6</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I18">
         <v>8</v>
@@ -81084,7 +81084,7 @@
         <v>-1</v>
       </c>
       <c r="T18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U18">
         <v>9</v>
@@ -81125,7 +81125,7 @@
         <v>10</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I19">
         <v>10</v>
@@ -81202,7 +81202,7 @@
         <v>8</v>
       </c>
       <c r="H20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I20">
         <v>10</v>
@@ -81279,7 +81279,7 @@
         <v>3</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I21">
         <v>5</v>
@@ -81356,7 +81356,7 @@
         <v>5</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I22">
         <v>6</v>
@@ -81392,7 +81392,7 @@
         <v>-1</v>
       </c>
       <c r="T22">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U22">
         <v>6</v>
@@ -81433,7 +81433,7 @@
         <v>5</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I23">
         <v>6</v>
@@ -81510,7 +81510,7 @@
         <v>8</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I24">
         <v>8</v>
@@ -81546,7 +81546,7 @@
         <v>-1</v>
       </c>
       <c r="T24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="U24">
         <v>9</v>
@@ -81587,7 +81587,7 @@
         <v>10</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I25">
         <v>10</v>
@@ -81741,7 +81741,7 @@
         <v>8</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I27">
         <v>9</v>
@@ -81818,7 +81818,7 @@
         <v>6</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I28">
         <v>10</v>
@@ -81854,7 +81854,7 @@
         <v>-1</v>
       </c>
       <c r="T28">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U28">
         <v>10</v>
@@ -81895,7 +81895,7 @@
         <v>7</v>
       </c>
       <c r="H29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I29">
         <v>10</v>
@@ -81931,7 +81931,7 @@
         <v>-1</v>
       </c>
       <c r="T29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U29">
         <v>10</v>
@@ -81972,7 +81972,7 @@
         <v>6</v>
       </c>
       <c r="H30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I30">
         <v>7</v>
@@ -82008,7 +82008,7 @@
         <v>-1</v>
       </c>
       <c r="T30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U30">
         <v>7</v>
@@ -82049,7 +82049,7 @@
         <v>7</v>
       </c>
       <c r="H31">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I31">
         <v>8</v>
@@ -82085,7 +82085,7 @@
         <v>-1</v>
       </c>
       <c r="T31">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U31">
         <v>8</v>
@@ -82126,7 +82126,7 @@
         <v>6</v>
       </c>
       <c r="H32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I32">
         <v>6</v>
@@ -82203,7 +82203,7 @@
         <v>8</v>
       </c>
       <c r="H33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I33">
         <v>9</v>
@@ -82280,7 +82280,7 @@
         <v>7</v>
       </c>
       <c r="H34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I34">
         <v>9</v>
@@ -82316,7 +82316,7 @@
         <v>-1</v>
       </c>
       <c r="T34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U34">
         <v>10</v>
@@ -82357,7 +82357,7 @@
         <v>8</v>
       </c>
       <c r="H35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I35">
         <v>10</v>
@@ -82434,7 +82434,7 @@
         <v>5</v>
       </c>
       <c r="H36">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I36">
         <v>6</v>
@@ -82511,7 +82511,7 @@
         <v>5</v>
       </c>
       <c r="H37">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I37">
         <v>10</v>
@@ -82547,7 +82547,7 @@
         <v>-1</v>
       </c>
       <c r="T37">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U37">
         <v>9</v>
@@ -82588,7 +82588,7 @@
         <v>7</v>
       </c>
       <c r="H38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I38">
         <v>6</v>
@@ -82624,7 +82624,7 @@
         <v>-1</v>
       </c>
       <c r="T38">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U38">
         <v>6</v>
@@ -82665,7 +82665,7 @@
         <v>5</v>
       </c>
       <c r="H39">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I39">
         <v>9</v>
@@ -82701,7 +82701,7 @@
         <v>-1</v>
       </c>
       <c r="T39">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U39">
         <v>10</v>
@@ -82742,7 +82742,7 @@
         <v>3</v>
       </c>
       <c r="H40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I40">
         <v>6</v>
@@ -82778,7 +82778,7 @@
         <v>-1</v>
       </c>
       <c r="T40">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U40">
         <v>6</v>
@@ -82819,7 +82819,7 @@
         <v>2</v>
       </c>
       <c r="H41">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I41">
         <v>6</v>
@@ -82896,7 +82896,7 @@
         <v>7</v>
       </c>
       <c r="H42">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I42">
         <v>9</v>
@@ -82973,7 +82973,7 @@
         <v>8</v>
       </c>
       <c r="H43">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I43">
         <v>8</v>
@@ -83050,7 +83050,7 @@
         <v>8</v>
       </c>
       <c r="H44">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I44">
         <v>10</v>
@@ -83086,7 +83086,7 @@
         <v>-1</v>
       </c>
       <c r="T44">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U44">
         <v>10</v>
@@ -83127,7 +83127,7 @@
         <v>7</v>
       </c>
       <c r="H45">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I45">
         <v>9</v>
@@ -84089,7 +84089,7 @@
         <v>7</v>
       </c>
       <c r="O12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P12">
         <v>-1</v>
@@ -84131,7 +84131,7 @@
         <v>8</v>
       </c>
       <c r="AC12">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:29">
@@ -84534,7 +84534,7 @@
         <v>5</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P17">
         <v>-1</v>
@@ -84576,7 +84576,7 @@
         <v>6</v>
       </c>
       <c r="AC17">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:29">
@@ -84623,7 +84623,7 @@
         <v>5</v>
       </c>
       <c r="O18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P18">
         <v>-1</v>
@@ -84665,7 +84665,7 @@
         <v>6</v>
       </c>
       <c r="AC18">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" spans="1:29">
@@ -84712,7 +84712,7 @@
         <v>5</v>
       </c>
       <c r="O19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P19">
         <v>-1</v>
@@ -84754,7 +84754,7 @@
         <v>6</v>
       </c>
       <c r="AC19">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:29">
@@ -84979,7 +84979,7 @@
         <v>5</v>
       </c>
       <c r="O22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P22">
         <v>-1</v>

</xml_diff>